<commit_message>
Aktualizácia ponúk – 2026-09-18 09:57 UTC
</commit_message>
<xml_diff>
--- a/public/ponuky.xlsx
+++ b/public/ponuky.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Prehľad" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ponuky'!$A$1:$D$350</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ponuky'!$A$1:$D$346</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D350"/>
+  <dimension ref="A1:D346"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -883,22 +883,22 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Tomas Jendek</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3547,17 +3547,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Senec, okres Senec</t>
+          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Alena Rydzikova</t>
+          <t>Tomáš Doubek</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -3569,17 +3569,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Cyprichova, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Tomáš Doubek</t>
+          <t>Anton K</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -3591,17 +3591,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Cyprichova, Bratislava-Rača, okres Bratislava III</t>
+          <t>Dvojkrížna, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Anton K</t>
+          <t>Ladislav Sipos</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
@@ -3613,17 +3613,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Dvojkrížna, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Na varte, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Ladislav Sipos</t>
+          <t>Alexander Milly</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -3635,17 +3635,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Na varte, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Budatínska 3718, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Alexander Milly</t>
+          <t>Eva Grochalová</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -3657,17 +3657,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Budatínska 3718, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Eva Grochalová</t>
+          <t>Matúš Sedlák</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -3679,12 +3679,12 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Jungmannova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Matúš Sedlák</t>
+          <t>Jana B</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -3701,17 +3701,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Jungmannova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Nezábudková 24, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Jana B</t>
+          <t>Martin Palla</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D148" s="2" t="inlineStr">
@@ -3723,17 +3723,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Nezábudková 24, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Malé Leváre, okres Malacky</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Martin Palla</t>
+          <t>Victoria Ivanová</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -3745,17 +3745,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Malé Leváre, okres Malacky</t>
+          <t>Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Victoria Ivanová</t>
+          <t>Vaše Bývanie</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -3767,17 +3767,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Nejedlého 20, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Vaše Bývanie</t>
+          <t>Mojmír Gaško</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -3789,17 +3789,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Nejedlého 20, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Rumančeková, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Mojmír Gaško</t>
+          <t>Ella Vitková</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D152" s="2" t="inlineStr">
@@ -3811,17 +3811,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Rumančeková, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Miletičova 5A, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Ella Vitková</t>
+          <t>Kristián Németh</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
@@ -3833,7 +3833,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Miletičova 5A, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Grösslingova 23, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -3843,7 +3843,7 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -3855,17 +3855,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Grösslingova 23, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Veltlínska, Svätý Jur, okres Pezinok</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Kristián Németh</t>
+          <t>Jaroslav Š</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -3877,17 +3877,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Veltlínska, Svätý Jur, okres Pezinok</t>
+          <t>Miletičova 34, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Jaroslav Š</t>
+          <t>Samuel Kostka</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -3899,17 +3899,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Miletičova 34, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Riazanská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Samuel Kostka</t>
+          <t>Ivan Beňo</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -3921,17 +3921,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Riazanská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Školská, Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Ivan Beňo</t>
+          <t>Terezia Kostolanska</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D158" s="2" t="inlineStr">
@@ -3943,17 +3943,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Školská, Chorvátsky Grob, okres Senec</t>
+          <t>Dopravná, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Terezia Kostolanska</t>
+          <t>Dagmar Semrisová</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -3965,12 +3965,12 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Dopravná, Bratislava-Rača, okres Bratislava III</t>
+          <t>Račianske mýto, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Dagmar Semrisová</t>
+          <t>Viera Lacika</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -3987,17 +3987,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Račianske mýto, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Tomášikova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Viera Lacika</t>
+          <t>Peter Dorday</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -4009,17 +4009,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Tomášikova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Peter Dorday</t>
+          <t>Robert B</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
@@ -4031,17 +4031,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Dunajská Lužná, okres Senec</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Robert B</t>
+          <t>Kristína Gatyášová</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
@@ -4053,17 +4053,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Dunajská Lužná, okres Senec</t>
+          <t>Bajkalská 45C, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Kristína Gatyášová</t>
+          <t>Eva Valáriková</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
@@ -4075,17 +4075,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Bajkalská 45C, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Eva Valáriková</t>
+          <t>Štefan Pántik</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
@@ -4097,17 +4097,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Karasová 68, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Štefan Pántik</t>
+          <t>Juraj Várady</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
@@ -4119,17 +4119,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Karasová 68, Senec, okres Senec</t>
+          <t>A. Gwerkovej 15, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Juraj Várady</t>
+          <t>Michal Weismann</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
@@ -4151,7 +4151,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -4163,17 +4163,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>A. Gwerkovej 15, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Oblačná 7155, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Michal Weismann</t>
+          <t>Roman R</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
@@ -4185,17 +4185,17 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Oblačná 7155, Bratislava-Rača, okres Bratislava III</t>
+          <t>Novohorská, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Roman R</t>
+          <t>Martin Klaučo</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D170" s="2" t="inlineStr">
@@ -4207,17 +4207,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Novohorská, Bratislava-Rača, okres Bratislava III</t>
+          <t>Zuzany Chalupovej 3981, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Martin Klaučo</t>
+          <t>Karol Jurčik</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -4229,17 +4229,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej 3981, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Karol Jurčik</t>
+          <t xml:space="preserve">Anton Englart </t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Vinica / chmeľnica</t>
         </is>
       </c>
       <c r="D172" s="2" t="inlineStr">
@@ -4251,17 +4251,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Pezinok, okres Pezinok</t>
+          <t>Senec, okres Senec</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t xml:space="preserve">Anton Englart </t>
+          <t>denisa vds</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Vinica / chmeľnica</t>
+          <t>Other object for housing</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
@@ -4273,17 +4273,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Senec, okres Senec</t>
+          <t>Nobelova, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>denisa vds</t>
+          <t>Ondrej R</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Other object for housing</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -4295,17 +4295,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Nobelova, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Kukučínova, Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Ondrej R</t>
+          <t>Jaro Hanzel</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
@@ -4317,17 +4317,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Kukučínova, Ivanka pri Dunaji, okres Senec</t>
+          <t>Račianska 69B, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Jaro Hanzel</t>
+          <t>Nadia Hofierkova</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
@@ -4339,12 +4339,12 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Račianska 69B, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Račianska 31, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Nadia Hofierkova</t>
+          <t>Peter Šimonka</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -4361,17 +4361,17 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Račianska 31, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Peter Šimonka</t>
+          <t>jana Lieskovska</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D178" s="2" t="inlineStr">
@@ -4383,17 +4383,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Pri vinohradoch 6179, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>jana Lieskovska</t>
+          <t>Tibor Tokár</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
@@ -4405,17 +4405,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Pri vinohradoch 6179, Bratislava-Rača, okres Bratislava III</t>
+          <t>Trebišovská, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Tibor Tokár</t>
+          <t>Stana Paulik</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
@@ -4427,12 +4427,12 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Trebišovská, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Rusovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Stana Paulik</t>
+          <t>petra svetik</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -4449,17 +4449,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Bratislava-Rusovce, okres Bratislava V</t>
+          <t>Mikulášska 1B, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>petra svetik</t>
+          <t>Martin Mančík</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
@@ -4471,17 +4471,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Mikulášska 1B, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bélu Bartóka 9, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Martin Mančík</t>
+          <t>Igor Gottgeisl</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
@@ -4493,12 +4493,12 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Bélu Bartóka 9, Senec, okres Senec</t>
+          <t>Pribinova, Bernolákovo, okres Senec</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Igor Gottgeisl</t>
+          <t>Juraj Adamčík</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -4515,17 +4515,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Pribinova, Bernolákovo, okres Senec</t>
+          <t>Bernolákovo, okres Senec</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Juraj Adamčík</t>
+          <t>Lucia Tacovska</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Záhrada</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
@@ -4537,17 +4537,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Bernolákovo, okres Senec</t>
+          <t>Bezručova 5, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Lucia Tacovska</t>
+          <t>Peter Moravcik</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>Záhrada</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
@@ -4559,17 +4559,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Bezručova 5, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Peter Moravcik</t>
+          <t>Lineta Uhrinová</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
@@ -4581,17 +4581,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Šancová, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Lineta Uhrinová</t>
+          <t>Miroslava Vojtekova</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -4603,17 +4603,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Šancová, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Doľany, okres Pezinok</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Miroslava Vojtekova</t>
+          <t>Gabriela Wenhardt</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
@@ -4625,17 +4625,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Doľany, okres Pezinok</t>
+          <t>Svetlá 3, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Gabriela Wenhardt</t>
+          <t>Adrian Cintula</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
@@ -4647,17 +4647,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Svetlá 3, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Adrian Cintula</t>
+          <t>Tomáš Kotlaba</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
@@ -4669,17 +4669,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Na pasekách, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Tomáš Kotlaba</t>
+          <t>Jaroslav Babik</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
@@ -4691,12 +4691,12 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Hornádska, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Západný rad, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Miro Kralovic</t>
+          <t>Iveta Kopecká</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -4713,17 +4713,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Na pasekách, Bratislava-Rača, okres Bratislava III</t>
+          <t>Dlhá 8/D, Stupava, okres Malacky</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Jaroslav Babik</t>
+          <t>Jaroslav Timko</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
@@ -4735,17 +4735,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Západný rad, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Ožvoldíkova, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Iveta Kopecká</t>
+          <t>Marek Riesz</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
@@ -4757,17 +4757,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Dlhá 8/D, Stupava, okres Malacky</t>
+          <t>Miloslavov, okres Senec</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Jaroslav Timko</t>
+          <t>Roman Pavelka</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
@@ -4779,12 +4779,12 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Ožvoldíkova, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Rovniankova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Marek Riesz</t>
+          <t>Katerina Koroleva</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -4801,12 +4801,12 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Miloslavov, okres Senec</t>
+          <t>Jablonec, okres Pezinok</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Roman Pavelka</t>
+          <t>Martin Chudoba</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -4823,17 +4823,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Rovniankova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Borská, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Katerina Koroleva</t>
+          <t>Jan Kuna</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
@@ -4845,17 +4845,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Jablonec, okres Pezinok</t>
+          <t>Ožvoldíkova, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Martin Chudoba</t>
+          <t>Samuel Kovalčík</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
@@ -4867,17 +4867,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Borská, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Žabí majer, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Jan Kuna</t>
+          <t>Marcel Buttko</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Mobilný dom</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
@@ -4889,17 +4889,17 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Ožvoldíkova, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Tomášikova 50C, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Samuel Kovalčík</t>
+          <t>Z C</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
@@ -4911,17 +4911,17 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Žabí majer, Bratislava-Rača, okres Bratislava III</t>
+          <t>Ulica Sauberg, Svätý Jur, okres Pezinok</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Marcel Buttko</t>
+          <t>Boris Haviar</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Mobilný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
@@ -4933,17 +4933,17 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Tomášikova 50C, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Z C</t>
+          <t>Patricia P</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D204" s="2" t="inlineStr">
@@ -4955,17 +4955,17 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Ulica Sauberg, Svätý Jur, okres Pezinok</t>
+          <t>Frankovská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Boris Haviar</t>
+          <t>Michal Klempai</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
@@ -4977,17 +4977,17 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Žilinská 1, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Patricia P</t>
+          <t>Mat Nav</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Obchodné priestory</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -4999,12 +4999,12 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Frankovská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Limbach, okres Pezinok</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Michal Klempai</t>
+          <t>Zuzana Farbulová</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -5021,7 +5021,7 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Žilinská 1, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bajkalská 9A, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -5031,7 +5031,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>Obchodné priestory</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -5043,17 +5043,17 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Limbach, okres Pezinok</t>
+          <t>Dúhová, Slovenský Grob, okres Pezinok</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Zuzana Farbulová</t>
+          <t>Peter Albert</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
@@ -5065,17 +5065,17 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Bajkalská 9A, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Kuklovská, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Mat Nav</t>
+          <t>Ra Fa</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -5087,12 +5087,12 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Dúhová, Slovenský Grob, okres Pezinok</t>
+          <t>Podhradie 68, Svätý Jur, okres Pezinok</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Peter Albert</t>
+          <t>Dávid Boháč</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -5109,17 +5109,17 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Kuklovská, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Schengenská, Bratislava-Čunovo, okres Bratislava V</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Ra Fa</t>
+          <t>Ľudovít Braniš</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rekreačný pozemok</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
@@ -5131,17 +5131,17 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Podhradie 68, Svätý Jur, okres Pezinok</t>
+          <t>Železničná 43, Bernolákovo, okres Senec</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Dávid Boháč</t>
+          <t>Tomáš Tenczer</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
@@ -5153,17 +5153,17 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Schengenská, Bratislava-Čunovo, okres Bratislava V</t>
+          <t>Antolská 6, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Ľudovít Braniš</t>
+          <t>Rudolf Lachkovic</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Rekreačný pozemok</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -5175,17 +5175,17 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Železničná 43, Bernolákovo, okres Senec</t>
+          <t>Lovinského 35, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Tomáš Tenczer</t>
+          <t xml:space="preserve">Pavol Kupec </t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Administratívna budova</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -5197,17 +5197,17 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Antolská 6, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Drieňová 16940, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Rudolf Lachkovic</t>
+          <t>Mat Nav</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Obchodné priestory</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -5219,17 +5219,17 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>Lovinského 35, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Fedinova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pavol Kupec </t>
+          <t>Tomáš  Vizina</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>Administratívna budova</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D217" s="2" t="inlineStr">
@@ -5241,17 +5241,17 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Drieňová 16940, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Hlavná 244, Záhorská Ves, okres Malacky</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Mat Nav</t>
+          <t>Alexander Horvath</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>Obchodné priestory</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D218" s="2" t="inlineStr">
@@ -5263,12 +5263,12 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Fedinova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Jána Jonáša, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Tomáš  Vizina</t>
+          <t>Katarína Kachmanová</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -5285,12 +5285,12 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>Hlavná 244, Záhorská Ves, okres Malacky</t>
+          <t>Pri vinohradoch 142, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Alexander Horvath</t>
+          <t>Ľuboš Čmelko</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -5307,17 +5307,17 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>Jána Jonáša, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
+          <t>Ulica Svornosti, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Katarína Kachmanová</t>
+          <t>Matuš  Žemlička</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Zmiešaná zóna</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -5329,17 +5329,17 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>Pri vinohradoch 142, Bratislava-Rača, okres Bratislava III</t>
+          <t>Košická 10, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Ľuboš Čmelko</t>
+          <t>David A</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -5351,17 +5351,17 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>Ulica Svornosti, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Nejedlého, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Matuš  Žemlička</t>
+          <t>Stanislava B</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Zmiešaná zóna</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D223" s="2" t="inlineStr">
@@ -5373,17 +5373,17 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>Košická 10, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Zlatý Karas, Nová Dedinka, okres Senec</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>David A</t>
+          <t>Vincent Durbak</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -5395,17 +5395,17 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Nejedlého, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Stanislava B</t>
+          <t>Edmund Edmund</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -5417,17 +5417,17 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>Zlatý Karas, Nová Dedinka, okres Senec</t>
+          <t>Jedľová ulica, Zohor, okres Malacky</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Vincent Durbak</t>
+          <t>Andrea Bencová</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -5439,17 +5439,17 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Plavecký Štvrtok, okres Malacky</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Edmund Edmund</t>
+          <t>Sisi Belo</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -5461,17 +5461,17 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>Jedľová ulica, Zohor, okres Malacky</t>
+          <t>Baltská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Andrea Bencová</t>
+          <t>L M</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -5483,17 +5483,17 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Plavecký Štvrtok, okres Malacky</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Sisi Belo</t>
+          <t>radovan reis</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -5505,12 +5505,12 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>Baltská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Trnavská cesta, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>L M</t>
+          <t>LEX vision</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -5527,17 +5527,17 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Male Pole 111, Vištuk, okres Pezinok</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>radovan reis</t>
+          <t>Frantisek Krasnansky</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -5549,17 +5549,17 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Trnavská cesta, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Uránová, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>LEX vision</t>
+          <t>Erik Varchol</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
@@ -5571,17 +5571,17 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Male Pole 111, Vištuk, okres Pezinok</t>
+          <t>Andreja Mráza 3160, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Frantisek Krasnansky</t>
+          <t>Michal Ruš</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
@@ -5593,12 +5593,12 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Uránová, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Hlavná 10E, Nová Dedinka, okres Senec</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Erik Varchol</t>
+          <t>Miroslava Magulova</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
@@ -5615,17 +5615,17 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Andreja Mráza 3160, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Ľ. Podjavorinskej, Most pri Bratislave, okres Senec</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Michal Ruš</t>
+          <t>Ľudovít Tomaškovič</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -5637,17 +5637,17 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Hlavná 10E, Nová Dedinka, okres Senec</t>
+          <t>Veľké Leváre, okres Malacky</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Miroslava Magulova</t>
+          <t>Denis  Klempa</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -5659,12 +5659,12 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Ľ. Podjavorinskej, Most pri Bratislave, okres Senec</t>
+          <t>Plavecký Štvrtok, okres Malacky</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Ľudovít Tomaškovič</t>
+          <t>Peter J</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
@@ -5681,17 +5681,17 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Veľké Leváre, okres Malacky</t>
+          <t>Cementárenská, Stupava, okres Malacky</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Denis  Klempa</t>
+          <t>Peter Haco</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Polyfunkčná budova</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -5703,12 +5703,12 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Plavecký Štvrtok, okres Malacky</t>
+          <t>Sama Chalúpku, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Peter J</t>
+          <t>Boris Cambalik</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
@@ -5725,17 +5725,17 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Cementárenská, Stupava, okres Malacky</t>
+          <t>Cyprichova 2, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Peter Haco</t>
+          <t>Anna Boríková</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>Polyfunkčná budova</t>
+          <t>Reštauračné priestory</t>
         </is>
       </c>
       <c r="D240" s="2" t="inlineStr">
@@ -5747,17 +5747,17 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Sama Chalúpku, Malacky, okres Malacky</t>
+          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Boris Cambalik</t>
+          <t>Lucia Danišová</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D241" s="2" t="inlineStr">
@@ -5769,17 +5769,17 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Cyprichova 2, Bratislava-Rača, okres Bratislava III</t>
+          <t>Karloveské rameno, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Anna Boríková</t>
+          <t>Pavol Bak</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Reštauračné priestory</t>
+          <t>Pozemok pre bytovú výstavbu</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
@@ -5791,17 +5791,17 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Karloveské rameno, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Lucia Danišová</t>
+          <t>Pavol Bak</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Bytový dom</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -5813,17 +5813,17 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Karloveské rameno, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Stromová, Slovenský Grob, okres Pezinok</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Pavol Bak</t>
+          <t>Barbora Slovíková</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Pozemok pre bytovú výstavbu</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
@@ -5835,17 +5835,17 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>Karloveské rameno, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Pavol Bak</t>
+          <t>Miroslav  Pinka</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Bytový dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -5857,12 +5857,12 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Stromová, Slovenský Grob, okres Pezinok</t>
+          <t>Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Barbora Slovíková</t>
+          <t>Nova Rekonštrukcia</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -5879,17 +5879,17 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Miroslav  Pinka</t>
+          <t>Lukáš Jurkovič</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -5901,17 +5901,17 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Studená, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Nova Rekonštrukcia</t>
+          <t>Byt Studena</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -5923,17 +5923,17 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>Malacky, okres Malacky</t>
+          <t>Ulica Závodu Matador, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Lukáš Jurkovič</t>
+          <t>Robert Antal</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
@@ -5945,17 +5945,17 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>Studená, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Krížna 1, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Byt Studena</t>
+          <t>martina busova</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -5967,17 +5967,17 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Ulica Závodu Matador, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Kresánkova, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Robert Antal</t>
+          <t>Igor Lorincik</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -5989,17 +5989,17 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>Krížna 1, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Hany Meličkovej, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>martina busova</t>
+          <t>Viera Peterkova</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -6011,12 +6011,12 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>Kresánkova, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Haburská, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Igor Lorincik</t>
+          <t>M Žitňanská</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
@@ -6033,17 +6033,17 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>Hany Meličkovej, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Bratislava-Lamač, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Viera Peterkova</t>
+          <t>E S</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
@@ -6055,17 +6055,17 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>Haburská, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Senec, okres Senec</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>M Žitňanská</t>
+          <t>Jana Muhlova</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
@@ -6077,17 +6077,17 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>Bratislava-Lamač, okres Bratislava IV</t>
+          <t>Košická, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>E S</t>
+          <t>Timea Henry</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -6099,17 +6099,17 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Senec, okres Senec</t>
+          <t>Košická, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Jana Muhlova</t>
+          <t>Timea Henry</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
@@ -6121,17 +6121,17 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>Košická, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Jantárová, Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Timea Henry</t>
+          <t>Monika Szocsova</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -6143,12 +6143,12 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Košická, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Západný rad, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Timea Henry</t>
+          <t>Iveta Kopecká</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
@@ -6165,17 +6165,17 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Jantárová, Bratislava-Jarovce, okres Bratislava V</t>
+          <t>Gaštanová 9, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Monika Szocsova</t>
+          <t>Iveta Kopecká</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -6187,17 +6187,17 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>Západný rad, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Jána L.Bellu (Lužianky), Senec, okres Senec</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Iveta Kopecká</t>
+          <t>Marian Mičko</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
@@ -6209,17 +6209,17 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>Gaštanová 9, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Iveta Kopecká</t>
+          <t>Jozef súkromná osoba</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Hotel / penzión</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
@@ -6231,17 +6231,17 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>Jána L.Bellu (Lužianky), Senec, okres Senec</t>
+          <t>Most pri Bratislave, okres Senec</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Marian Mičko</t>
+          <t>Matúš Štúber</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
@@ -6253,17 +6253,17 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Modra, okres Pezinok</t>
+          <t>Dunajská, Most pri Bratislave, okres Senec</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Jozef súkromná osoba</t>
+          <t>Ľuboš Štvrtecký</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Hotel / penzión</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
@@ -6275,17 +6275,17 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Most pri Bratislave, okres Senec</t>
+          <t>Pionierska, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Matúš Štúber</t>
+          <t>Peter Nagy</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
@@ -6297,17 +6297,17 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Dunajská, Most pri Bratislave, okres Senec</t>
+          <t>Koniarková, Bratislava-Vajnory, okres Bratislava III</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Ľuboš Štvrtecký</t>
+          <t>Daniela Kiniková</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
@@ -6319,17 +6319,17 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Pionierska, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Opálová, Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Peter Nagy</t>
+          <t>Jana Malisova</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D267" s="2" t="inlineStr">
@@ -6341,12 +6341,12 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>Koniarková, Bratislava-Vajnory, okres Bratislava III</t>
+          <t>Hydinárska 9617, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Daniela Kiniková</t>
+          <t>Alex Medek</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
@@ -6363,17 +6363,17 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Opálová, Bratislava-Jarovce, okres Bratislava V</t>
+          <t>Slnečné jazerá, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Jana Malisova</t>
+          <t>Filip Lečko</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
@@ -6385,17 +6385,17 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Hydinárska 9617, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Pod Vtáčnikom, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Alex Medek</t>
+          <t>Ivan Sanislo</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
@@ -6407,12 +6407,12 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Slnečné jazerá, Senec, okres Senec</t>
+          <t>Pekná 1061, Veľké Leváre, okres Malacky</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Filip Lečko</t>
+          <t>Valéria Micháleková</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
@@ -6429,17 +6429,17 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Pod Vtáčnikom, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Banšelova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Ivan Sanislo</t>
+          <t>Ivan Beňo</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
@@ -6451,12 +6451,12 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>Pekná 1061, Veľké Leváre, okres Malacky</t>
+          <t>Avanárska, Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Valéria Micháleková</t>
+          <t>Julius Bohunsky</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
@@ -6473,12 +6473,12 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>Banšelova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Dlhé diely, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Ivan Beňo</t>
+          <t>Matusk Tomas</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
@@ -6495,17 +6495,17 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Platanová ulica, Miloslavov, okres Senec</t>
+          <t>Jozefa Kubinu, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Richard Löffler</t>
+          <t>Martina Hlubocká</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
@@ -6517,17 +6517,17 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Avanárska, Rohožník, okres Malacky</t>
+          <t>Markova 7, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Julius Bohunsky</t>
+          <t>Martin Číž</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D276" s="2" t="inlineStr">
@@ -6539,17 +6539,17 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Dlhé diely, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Matusk Tomas</t>
+          <t>Peter Kovár</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -6561,17 +6561,17 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Jozefa Kubinu, Malacky, okres Malacky</t>
+          <t>Steinov dvor, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Martina Hlubocká</t>
+          <t>Ing Šalátová Zuzana</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
@@ -6583,17 +6583,17 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Markova 7, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Svätý Martin, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Martin Číž</t>
+          <t>Stanislav Sakac</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -6605,17 +6605,17 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Šancová, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Peter Kovár</t>
+          <t>Eva Tarasovič</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -6627,12 +6627,12 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Steinov dvor, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Žižkova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Ing Šalátová Zuzana</t>
+          <t>Denisa Slančová</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -6649,17 +6649,17 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Svätý Martin, Senec, okres Senec</t>
+          <t>Strmý vŕšok 164, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Stanislav Sakac</t>
+          <t>Tereza Adámyová</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -6671,17 +6671,17 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Šancová, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Lackova, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Eva Tarasovič</t>
+          <t>Predaj Bytu</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -6693,17 +6693,17 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Žižkova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Denisa Slančová</t>
+          <t>Tatiana B</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -6715,17 +6715,17 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Strmý vŕšok 164, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
+          <t>Vlastenecké námestie, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Tereza Adámyová</t>
+          <t>Luboš Wenzl</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
@@ -6737,12 +6737,12 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Lackova, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Nevädzová 6, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Predaj Bytu</t>
+          <t>Daniel l</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -6759,17 +6759,17 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Rohožník, okres Malacky</t>
+          <t>Makovického, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Tatiana B</t>
+          <t>Predaj Nehnutelosti</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -6781,17 +6781,17 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Vlastenecké námestie, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Čsl. parašutistov, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Luboš Wenzl</t>
+          <t>Tomáš Tóth</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -6803,17 +6803,17 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>Nevädzová 6, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Holíčska 9, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Daniel l</t>
+          <t>Zuzana Pišteková</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
@@ -6825,17 +6825,17 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>Makovického, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Talihov dvor, Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Predaj Nehnutelosti</t>
+          <t>Marian Virgovič</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Záhrada</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
@@ -6847,17 +6847,17 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>Čsl. parašutistov, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Račianska 64, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Tomáš Tóth</t>
+          <t>Roman Miškulynets</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D291" s="2" t="inlineStr">
@@ -6869,17 +6869,17 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>Holíčska 9, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Kukučínova, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Zuzana Pišteková</t>
+          <t>Eva Tarasovič</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
@@ -6891,17 +6891,17 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>Talihov dvor, Pezinok, okres Pezinok</t>
+          <t>Suchý vrch, Limbach, okres Pezinok</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Marian Virgovič</t>
+          <t>Miloslav Moravec</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Záhrada</t>
+          <t>Zrub / chalupa</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -6913,17 +6913,17 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>Račianska 64, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Ružová dolina 16, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Roman Miškulynets</t>
+          <t>Ľuboš Ľahký</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
@@ -6935,17 +6935,17 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Kukučínova, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Na vrátkach, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Eva Tarasovič</t>
+          <t>Roland Samek</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -6957,17 +6957,17 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Suchý vrch, Limbach, okres Pezinok</t>
+          <t>Námestie 1. mája 3866, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Miloslav Moravec</t>
+          <t>Oleksiy Namestie</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Zrub / chalupa</t>
+          <t>Polyfunkčná budova</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
@@ -6979,17 +6979,17 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>Ružová dolina 16, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Limbašská cesta, Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Ľuboš Ľahký</t>
+          <t>Ganna Naichuk</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -7001,17 +7001,17 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>Na vrátkach, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Solivarská, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Roland Samek</t>
+          <t>Michal Olšiak</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
@@ -7023,17 +7023,17 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>Námestie 1. mája 3866, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Jungmannova 2, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Oleksiy Namestie</t>
+          <t>Laco Vanko</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>Polyfunkčná budova</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
@@ -7045,17 +7045,17 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>Limbašská cesta, Pezinok, okres Pezinok</t>
+          <t>Kristy Bendovej, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Ganna Naichuk</t>
+          <t>Jana Gottstein</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
@@ -7067,12 +7067,12 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>Solivarská, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Sklenárova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Michal Olšiak</t>
+          <t>Dagmar Ivanová</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
@@ -7089,17 +7089,17 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>Jungmannova 2, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Pod vŕškom, Stupava, okres Malacky</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Laco Vanko</t>
+          <t>Lenka Višňovská</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr">
@@ -7111,17 +7111,17 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>Kristy Bendovej, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Galbavého 1, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Jana Gottstein</t>
+          <t>Denisa Lukačovičová</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Obchodné priestory</t>
         </is>
       </c>
       <c r="D303" s="2" t="inlineStr">
@@ -7133,17 +7133,17 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Sklenárova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Vážska, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Dagmar Ivanová</t>
+          <t>Kristína Erazmusová</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
@@ -7155,17 +7155,17 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Pod vŕškom, Stupava, okres Malacky</t>
+          <t>Stromová 25, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Lenka Višňovská</t>
+          <t>Michal Rusek</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D305" s="2" t="inlineStr">
@@ -7177,17 +7177,17 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Galbavého 1, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Chatová rekreačná oblasť, Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Denisa Lukačovičová</t>
+          <t>M J</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Obchodné priestory</t>
+          <t>Zrub / chalupa</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
@@ -7199,17 +7199,17 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Vážska, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Hagarova, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Kristína Erazmusová</t>
+          <t>Pavol Kusenda</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
@@ -7221,17 +7221,17 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>Stromová 25, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Michal Rusek</t>
+          <t>L G</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
@@ -7243,17 +7243,17 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>Chatová rekreačná oblasť, Rohožník, okres Malacky</t>
+          <t>Námestie Hraničiarov, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>M J</t>
+          <t>predaj nehnutelnosti</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>Zrub / chalupa</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D309" s="2" t="inlineStr">
@@ -7265,17 +7265,17 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>Hagarova, Bratislava-Rača, okres Bratislava III</t>
+          <t>Chotárna, Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Pavol Kusenda</t>
+          <t>Tomáš Stolárik</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D310" s="2" t="inlineStr">
@@ -7287,17 +7287,17 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Vavrinecká, Limbach, okres Pezinok</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>L G</t>
+          <t>Peter Petrina</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
@@ -7309,17 +7309,17 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>Námestie Hraničiarov, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Máchova, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>predaj nehnutelnosti</t>
+          <t xml:space="preserve">Andrea  Majchráková </t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D312" s="2" t="inlineStr">
@@ -7329,22 +7329,22 @@
       </c>
     </row>
     <row r="313">
-      <c r="A313" t="inlineStr">
-        <is>
-          <t>Chotárna, Bratislava-Jarovce, okres Bratislava V</t>
-        </is>
-      </c>
-      <c r="B313" t="inlineStr">
-        <is>
-          <t>Tomáš Stolárik</t>
-        </is>
-      </c>
-      <c r="C313" t="inlineStr">
-        <is>
-          <t>Rodinný dom</t>
-        </is>
-      </c>
-      <c r="D313" s="2" t="inlineStr">
+      <c r="A313" s="3" t="inlineStr">
+        <is>
+          <t>Komenského 2, Modra, okres Pezinok</t>
+        </is>
+      </c>
+      <c r="B313" s="3" t="inlineStr">
+        <is>
+          <t>Andrej B</t>
+        </is>
+      </c>
+      <c r="C313" s="3" t="inlineStr">
+        <is>
+          <t>Garsónka</t>
+        </is>
+      </c>
+      <c r="D313" s="4" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7353,12 +7353,12 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>Vavrinecká, Limbach, okres Pezinok</t>
+          <t>Knižkova dolina, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Peter Petrina</t>
+          <t>Daniel Presul</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -7375,12 +7375,12 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Máchova, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t xml:space="preserve">Andrea  Majchráková </t>
+          <t>Soňa Slobodníková</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -7397,17 +7397,17 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Knižkova dolina, Bratislava-Rača, okres Bratislava III</t>
+          <t>Na Revíne 19, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Daniel Presul</t>
+          <t>Dušan Cintula</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D316" s="2" t="inlineStr">
@@ -7419,17 +7419,17 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Bratislava-Jarovce, okres Bratislava V</t>
+          <t>Plzenská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Soňa Slobodníková</t>
+          <t>Martin H</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D317" s="2" t="inlineStr">
@@ -7441,12 +7441,12 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Na Revíne 19, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Hrušková 44H, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Dušan Cintula</t>
+          <t>Jasna Rumanková</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -7463,17 +7463,17 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>Plzenská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Konventná 5, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Martin H</t>
+          <t>Vladimir Taraba</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D319" s="2" t="inlineStr">
@@ -7485,17 +7485,17 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>Hrušková 44H, Bratislava-Rača, okres Bratislava III</t>
+          <t>Landererova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Jasna Rumanková</t>
+          <t>Jan Kovac</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D320" s="2" t="inlineStr">
@@ -7507,17 +7507,17 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>Obuvnícka, Stupava, okres Malacky</t>
+          <t>Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Viera Nováková</t>
+          <t>Tomáš Machciník</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D321" s="2" t="inlineStr">
@@ -7529,17 +7529,17 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>Konventná 5, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Malokarpatská 1, Svätý Jur, okres Pezinok</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Vladimir Taraba</t>
+          <t>Jana Zárecká</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D322" s="2" t="inlineStr">
@@ -7551,12 +7551,12 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>Landererova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Koceľova, Slovenský Grob, okres Pezinok</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Jan Kovac</t>
+          <t>Ján Hudec</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -7573,17 +7573,17 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>Pezinok, okres Pezinok</t>
+          <t>Panónska cesta, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Tomáš Machciník</t>
+          <t>Oliver Práznovský</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D324" s="2" t="inlineStr">
@@ -7595,17 +7595,17 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>Malokarpatská 1, Svätý Jur, okres Pezinok</t>
+          <t>Mariánska cesta, Svätý Jur, okres Pezinok</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Jana Zárecká</t>
+          <t>Marian Machalek</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Rekreačný pozemok</t>
         </is>
       </c>
       <c r="D325" s="2" t="inlineStr">
@@ -7617,17 +7617,17 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>Koceľova, Slovenský Grob, okres Pezinok</t>
+          <t>Homolova, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Ján Hudec</t>
+          <t>Jaroslav Janco</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D326" s="2" t="inlineStr">
@@ -7639,17 +7639,17 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>Panónska cesta, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Potočná, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Oliver Práznovský</t>
+          <t>Pavol Beblavy</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D327" s="2" t="inlineStr">
@@ -7661,17 +7661,17 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>Mariánska cesta, Svätý Jur, okres Pezinok</t>
+          <t>Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Marian Machalek</t>
+          <t>Peter Urban</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Rekreačný pozemok</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D328" s="2" t="inlineStr">
@@ -7683,17 +7683,17 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>Homolova, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Miletičova 60, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Jaroslav Janco</t>
+          <t>Michael Kollár</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D329" s="2" t="inlineStr">
@@ -7705,17 +7705,17 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>Potočná, Bratislava-Rača, okres Bratislava III</t>
+          <t>Svätovavrinecká, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Pavol Beblavy</t>
+          <t>Katarína Rusňáková</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>5+ izbový byt</t>
         </is>
       </c>
       <c r="D330" s="2" t="inlineStr">
@@ -7727,17 +7727,17 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>Pezinok, okres Pezinok</t>
+          <t>Hraničiarska, Vysoká pri Morave, okres Malacky</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Peter Urban</t>
+          <t>Andrea Bencová</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D331" s="2" t="inlineStr">
@@ -7749,17 +7749,17 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>Miletičova 60, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Ľanová ulica, Rovinka, okres Senec</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Michael Kollár</t>
+          <t>Alena Alena</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D332" s="2" t="inlineStr">
@@ -7771,17 +7771,17 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>Svätovavrinecká, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Bajkalská, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Katarína Rusňáková</t>
+          <t>Jakub Osuský</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>5+ izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D333" s="2" t="inlineStr">
@@ -7793,17 +7793,17 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>Hraničiarska, Vysoká pri Morave, okres Malacky</t>
+          <t>Devínska cesta, Bratislava-Devín, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Andrea Bencová</t>
+          <t>ales malina</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Záhradná chatka</t>
         </is>
       </c>
       <c r="D334" s="2" t="inlineStr">
@@ -7815,12 +7815,12 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>Ľanová ulica, Rovinka, okres Senec</t>
+          <t>Svätovavrinecká, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Alena Alena</t>
+          <t>Katarína Rusňáková</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -7837,17 +7837,17 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>Bajkalská, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Maďarská, Bratislava-Rusovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Jakub Osuský</t>
+          <t>Vlastníčka nehnuteľnosti</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D336" s="2" t="inlineStr">
@@ -7859,17 +7859,17 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>Devínska cesta, Bratislava-Devín, okres Bratislava IV</t>
+          <t>Jakubov, okres Malacky</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>ales malina</t>
+          <t>Tomas M</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Záhradná chatka</t>
+          <t>Zrub / chalupa</t>
         </is>
       </c>
       <c r="D337" s="2" t="inlineStr">
@@ -7881,12 +7881,12 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>Svätovavrinecká, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Konvalinková ulica, Miloslavov, okres Senec</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Katarína Rusňáková</t>
+          <t>Ing Robert Stanek</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -7903,12 +7903,12 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>Maďarská, Bratislava-Rusovce, okres Bratislava V</t>
+          <t>Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Vlastníčka nehnuteľnosti</t>
+          <t>Samo Mravec</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -7925,17 +7925,17 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>Jakubov, okres Malacky</t>
+          <t>Elektrárenská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Tomas M</t>
+          <t>Petr Jašák</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Zrub / chalupa</t>
+          <t>Manufacturing facility</t>
         </is>
       </c>
       <c r="D340" s="2" t="inlineStr">
@@ -7947,17 +7947,17 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>Konvalinková ulica, Miloslavov, okres Senec</t>
+          <t>Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Ing Robert Stanek</t>
+          <t>Vlastník bytu</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D341" s="2" t="inlineStr">
@@ -7969,12 +7969,12 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>Bratislava-Jarovce, okres Bratislava V</t>
+          <t>Ferdinanda Píseckého, Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Samo Mravec</t>
+          <t>Martin K</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -7991,17 +7991,17 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>Elektrárenská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Ivanská cesta, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Petr Jašák</t>
+          <t>Ľuboš Ľuboš</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>Manufacturing facility</t>
+          <t>Zmiešaná zóna</t>
         </is>
       </c>
       <c r="D343" s="2" t="inlineStr">
@@ -8013,17 +8013,17 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Koreničova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Vlastník bytu</t>
+          <t>Barbara Hodásová</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D344" s="2" t="inlineStr">
@@ -8035,17 +8035,17 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>Ferdinanda Píseckého, Modra, okres Pezinok</t>
+          <t>Na barine, Bratislava-Lamač, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Martin K</t>
+          <t>Peter Durica</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D345" s="2" t="inlineStr">
@@ -8057,17 +8057,17 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>Ivanská cesta, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Cementárenská, Stupava, okres Malacky</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Ľuboš Ľuboš</t>
+          <t>Jevgenija Bilousko</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>Zmiešaná zóna</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D346" s="2" t="inlineStr">
@@ -8076,96 +8076,8 @@
         </is>
       </c>
     </row>
-    <row r="347">
-      <c r="A347" t="inlineStr">
-        <is>
-          <t>Koreničova, Bratislava-Staré Mesto, okres Bratislava I</t>
-        </is>
-      </c>
-      <c r="B347" t="inlineStr">
-        <is>
-          <t>Barbara Hodásová</t>
-        </is>
-      </c>
-      <c r="C347" t="inlineStr">
-        <is>
-          <t>1-izbový byt</t>
-        </is>
-      </c>
-      <c r="D347" s="2" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
-    <row r="348">
-      <c r="A348" t="inlineStr">
-        <is>
-          <t>Na barine, Bratislava-Lamač, okres Bratislava IV</t>
-        </is>
-      </c>
-      <c r="B348" t="inlineStr">
-        <is>
-          <t>Peter Durica</t>
-        </is>
-      </c>
-      <c r="C348" t="inlineStr">
-        <is>
-          <t>3-izbový byt</t>
-        </is>
-      </c>
-      <c r="D348" s="2" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
-    <row r="349">
-      <c r="A349" t="inlineStr">
-        <is>
-          <t>Cementárenská, Stupava, okres Malacky</t>
-        </is>
-      </c>
-      <c r="B349" t="inlineStr">
-        <is>
-          <t>Jevgenija Bilousko</t>
-        </is>
-      </c>
-      <c r="C349" t="inlineStr">
-        <is>
-          <t>4-izbový byt</t>
-        </is>
-      </c>
-      <c r="D349" s="2" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
-    <row r="350">
-      <c r="A350" t="inlineStr">
-        <is>
-          <t>Martinčekova, Bratislava-Ružinov, okres Bratislava II</t>
-        </is>
-      </c>
-      <c r="B350" t="inlineStr">
-        <is>
-          <t>R Bujna</t>
-        </is>
-      </c>
-      <c r="C350" t="inlineStr">
-        <is>
-          <t>2-izbový byt</t>
-        </is>
-      </c>
-      <c r="D350" s="2" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D350"/>
+  <autoFilter ref="A1:D346"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -8512,10 +8424,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D344" r:id="rId343"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D345" r:id="rId344"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D346" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D347" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D348" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D349" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D350" r:id="rId349"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8548,7 +8456,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>349</v>
+        <v>345</v>
       </c>
     </row>
     <row r="4">
@@ -8559,7 +8467,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>17.09.2026 20:28</t>
+          <t>18.09.2026 09:57</t>
         </is>
       </c>
     </row>
@@ -8599,7 +8507,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10">
@@ -8629,7 +8537,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>44</v>
+        <v>42</v>
       </c>
     </row>
     <row r="13">
@@ -8649,7 +8557,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15">
@@ -8659,7 +8567,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17">
@@ -8688,7 +8596,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="20">
@@ -8698,7 +8606,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21">
@@ -8708,7 +8616,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="22">
@@ -8748,7 +8656,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="26">

</xml_diff>

<commit_message>
Aktualizácia ponúk – 2026-09-25 20:42 UTC
</commit_message>
<xml_diff>
--- a/public/ponuky.xlsx
+++ b/public/ponuky.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Prehľad" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ponuky'!$A$1:$D$351</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ponuky'!$A$1:$D$349</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D351"/>
+  <dimension ref="A1:D349"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -489,42 +489,42 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Okružná 47, Senec, okres Senec</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Roman Gazdik</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Rodinný dom</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>otvoriť ponuku</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>Slovenský Grob, okres Pezinok</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Igor Šramka</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Kozia, Bratislava-Staré Mesto, okres Bratislava I</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Ľubor Mendel</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>4-izbový byt</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -533,17 +533,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Dopravná 23, Bratislava-Rača, okres Bratislava III</t>
+          <t>Kozia, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Peter Pipiš</t>
+          <t>Ľubor Mendel</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -555,17 +555,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Šalviová, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Dopravná 23, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Juraj Valašťan</t>
+          <t>Peter Pipiš</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -577,12 +577,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Agátová, Ivanka pri Dunaji, okres Senec</t>
+          <t>Šalviová, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Viktória Krupová</t>
+          <t>Juraj Valašťan</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -599,17 +599,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Kaplinská 7, Bratislava-Rača, okres Bratislava III</t>
+          <t>Agátová, Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Eva Žíhlavníková</t>
+          <t>Viktória Krupová</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -621,17 +621,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Repašského 1, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Kaplinská 7, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Michal Weismann</t>
+          <t>Eva Žíhlavníková</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -665,17 +665,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Repašského 1, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Alexander Kernaševič</t>
+          <t>Michal Weismann</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Mobile cells and stands</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -687,17 +687,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>167, Borinka, okres Malacky</t>
+          <t>Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Kamil Semeš</t>
+          <t>Alexander Kernaševič</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>Mobile cells and stands</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -709,17 +709,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Gregorovej, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>167, Borinka, okres Malacky</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Andrej Miko</t>
+          <t>Kamil Semeš</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -731,17 +731,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Jablonec, okres Pezinok</t>
+          <t>Gregorovej, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Andrea Valentová</t>
+          <t>Andrej Miko</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -753,17 +753,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Ivanka pri Dunaji, okres Senec</t>
+          <t>Jablonec, okres Pezinok</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Andrea Bášková</t>
+          <t>Andrea Valentová</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -775,12 +775,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Katarína Rusňáková</t>
+          <t>Andrea Bášková</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -797,12 +797,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Ulica 8. mája 22A, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Vladimír Mitrík</t>
+          <t>Katarína Rusňáková</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -819,17 +819,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Partizánska 1081, Malacky, okres Malacky</t>
+          <t>Ulica 8. mája 22A, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Peter Ondrovič</t>
+          <t>Vladimír Mitrík</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -841,12 +841,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Čulenova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Partizánska 1081, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>M I</t>
+          <t>Peter Ondrovič</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -863,17 +863,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Lachova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Čulenova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Zuzana V</t>
+          <t>M I</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -885,17 +885,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Drobného, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Lachova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Peter Chovanec</t>
+          <t>Zuzana V</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -907,17 +907,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Vysoká pri Morave, okres Malacky</t>
+          <t>Drobného, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Miroslav Vojkovic</t>
+          <t>Peter Chovanec</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -929,12 +929,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Vinárska, Modra, okres Pezinok</t>
+          <t>Vysoká pri Morave, okres Malacky</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>marek rozic</t>
+          <t>Miroslav Vojkovic</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -951,17 +951,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Vinárska, Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Anton K</t>
+          <t>marek rozic</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -973,17 +973,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Tupolevova 18, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Ivan Hargas</t>
+          <t>Anton K</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -995,12 +995,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Stavbárska 4, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Tupolevova 18, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Jaroslav Valus</t>
+          <t>Ivan Hargas</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1017,17 +1017,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Bratislava-Vajnory, okres Bratislava III</t>
+          <t>Stavbárska 4, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Juraj Varacka</t>
+          <t>Jaroslav Valus</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1039,17 +1039,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Vajnory, okres Bratislava III</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Juraj Litomerický</t>
+          <t>Juraj Varacka</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1061,17 +1061,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Vyšehradská 16, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Juraj Kovašich</t>
+          <t>Juraj Litomerický</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -1083,17 +1083,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Grösslingova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Vyšehradská 16, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Viktor Riegel</t>
+          <t>Juraj Kovašich</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1105,17 +1105,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Sekurisova, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Grösslingova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Matej Kohucik</t>
+          <t>Viktor Riegel</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -1127,17 +1127,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Ipeľská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Sekurisova, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>David Ivanov</t>
+          <t>Matej Kohucik</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1149,17 +1149,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Karloveské rameno, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Ipeľská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Boris Emrich</t>
+          <t>David Ivanov</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -1171,17 +1171,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Landauova, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Karloveské rameno, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>peter klvac</t>
+          <t>Boris Emrich</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -1193,42 +1193,42 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>Landauova, Bratislava-Dúbravka, okres Bratislava IV</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>peter klvac</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>1-izbový byt</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>otvoriť ponuku</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t>Tomášikova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>BaTom P</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>Garsónka</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="2" t="inlineStr">
-        <is>
-          <t>Krížna, Bratislava-Staré Mesto, okres Bratislava I</t>
-        </is>
-      </c>
-      <c r="B35" s="2" t="inlineStr">
-        <is>
-          <t>Peter Valenta</t>
-        </is>
-      </c>
-      <c r="C35" s="2" t="inlineStr">
-        <is>
-          <t>Kancelárie</t>
-        </is>
-      </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D35" s="4" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1237,17 +1237,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Námestie Slobody, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Krížna, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Martin Gažo</t>
+          <t>Peter Valenta</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Kancelárie</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -1259,17 +1259,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Bratislava-Rusovce, okres Bratislava V</t>
+          <t>Námestie Slobody, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Milan Dzilsky</t>
+          <t>Martin Gažo</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -1281,17 +1281,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Rovniankova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Bratislava-Rusovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Roman N</t>
+          <t>Milan Dzilsky</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -1303,17 +1303,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Rovniankova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Martin Chamko</t>
+          <t>Roman N</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -1325,17 +1325,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Jaskový rad 47, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Angela Brinzova</t>
+          <t>Martin Chamko</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -1347,17 +1347,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Podjavorinskej 13, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Jaskový rad 47, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Tomáš Čitbaj</t>
+          <t>Angela Brinzova</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -1369,17 +1369,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Krušpánová, Bratislava-Čunovo, okres Bratislava V</t>
+          <t>Podjavorinskej 13, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Alena Horváthová</t>
+          <t>Tomáš Čitbaj</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -1391,17 +1391,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Rovniankova 20, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Krušpánová, Bratislava-Čunovo, okres Bratislava V</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Michal Weismann</t>
+          <t>Alena Horváthová</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -1435,17 +1435,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Šancová 37, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Rovniankova 20, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Frantisek Manduch</t>
+          <t>Michal Weismann</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -1457,17 +1457,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Miloslavov, okres Senec</t>
+          <t>Šancová 37, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Jakub Hronec</t>
+          <t>Frantisek Manduch</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -1479,17 +1479,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Malé Leváre, okres Malacky</t>
+          <t>Miloslavov, okres Senec</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Michal Fajták</t>
+          <t>Jakub Hronec</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -1501,17 +1501,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Komenského, Modra, okres Pezinok</t>
+          <t>Malé Leváre, okres Malacky</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Richard Baranovic</t>
+          <t>Michal Fajták</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -1523,17 +1523,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Markova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Komenského, Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Peter Novotný</t>
+          <t>Richard Baranovic</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -1545,12 +1545,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Hornádska 28, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Markova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Miro Kralovic</t>
+          <t>Peter Novotný</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1567,12 +1567,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Plzenská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Hornádska 28, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Peter Kubica</t>
+          <t>Miro Kralovic</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1589,17 +1589,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Plzenská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Lukáš K</t>
+          <t>Peter Kubica</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -1611,17 +1611,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Hattalova, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Šťastný  Vlastník</t>
+          <t>Lukáš K</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -1633,17 +1633,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Slovenský Grob, okres Pezinok</t>
+          <t>Hattalova, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Jozef Brom</t>
+          <t>Šťastný  Vlastník</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -1655,17 +1655,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Slovenský Grob, okres Pezinok</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>MM victory</t>
+          <t>Jozef Brom</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -1677,12 +1677,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Ružinov Štrkovec</t>
+          <t>MM victory</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1699,17 +1699,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Bernolákova, Nová Dedinka, okres Senec</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Karina Szutyányiová</t>
+          <t>Ružinov Štrkovec</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -1721,17 +1721,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Senec, okres Senec</t>
+          <t>Bernolákova, Nová Dedinka, okres Senec</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>RD RD</t>
+          <t>Karina Szutyányiová</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -1743,12 +1743,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Školská, Rovinka, okres Senec</t>
+          <t>Senec, okres Senec</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Alena Alena</t>
+          <t>RD RD</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1765,17 +1765,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Školská, Rovinka, okres Senec</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lukas Novosiadly </t>
+          <t>Alena Alena</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -1787,17 +1787,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Hany Zelinovej, Senec, okres Senec</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Peter Veselsky</t>
+          <t xml:space="preserve">Lukas Novosiadly </t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -1809,17 +1809,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Dunajská, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Hany Zelinovej, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Tatiana B</t>
+          <t>Peter Veselsky</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>5+ izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -1831,17 +1831,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Malacky, okres Malacky</t>
+          <t>Dunajská, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Martin Jendek</t>
+          <t>Tatiana B</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>5+ izbový byt</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -1853,12 +1853,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Antolská, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Peter K</t>
+          <t>Martin Jendek</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1875,17 +1875,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Zidiny 11, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Antolská, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Vratislav Jurica</t>
+          <t>Peter K</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -1897,17 +1897,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Čulenova 5, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Zidiny 11, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Martin Martin</t>
+          <t>Vratislav Jurica</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -1919,17 +1919,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Betliarska, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Čulenova 5, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Hana Habartova</t>
+          <t>Martin Martin</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Zmiešaná zóna</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -1941,17 +1941,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Sliačska 13903, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Betliarska, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Jan Syč</t>
+          <t>Hana Habartova</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Zmiešaná zóna</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -1963,17 +1963,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Sliačska 13903, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Denisa Slančová</t>
+          <t>Jan Syč</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -1985,17 +1985,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Dúbravčická, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Jakub Brondoš</t>
+          <t>Denisa Slančová</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Rekreačný pozemok</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -2007,17 +2007,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Miletičova 16, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Dúbravčická, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Kristián Németh</t>
+          <t>Jakub Brondoš</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rekreačný pozemok</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -2029,12 +2029,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Vrabčia, Senec, okres Senec</t>
+          <t>Miletičova 16, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Katarína Lattová</t>
+          <t>Kristián Németh</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2051,17 +2051,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Lipová ulica, Hrubá Borša, okres Senec</t>
+          <t>Vrabčia, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Štefan Hencel</t>
+          <t>Katarína Lattová</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -2073,12 +2073,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Šenkvice, okres Pezinok</t>
+          <t>Lipová ulica, Hrubá Borša, okres Senec</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Jaro Jaro</t>
+          <t>Štefan Hencel</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2095,17 +2095,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Ota Holúska, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
+          <t>Šenkvice, okres Pezinok</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Nikola Mináčová</t>
+          <t>Jaro Jaro</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -2117,17 +2117,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Plachého, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Ota Holúska, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Alojz Hančin</t>
+          <t>Nikola Mináčová</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Other object for housing</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -2139,17 +2139,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Bebravská, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Plachého, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARZE MARZE </t>
+          <t>Alojz Hančin</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Other object for housing</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -2161,17 +2161,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Banskobystrická, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bebravská, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Jozef Novák</t>
+          <t xml:space="preserve">MARZE MARZE </t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -2183,17 +2183,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Banskobystrická, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>RD RD</t>
+          <t>Jozef Novák</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -2205,17 +2205,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Peter Szell</t>
+          <t>RD RD</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Iný priestor</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -2227,17 +2227,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Albrechtova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARZE MARZE </t>
+          <t>Peter Szell</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Iný priestor</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -2249,17 +2249,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Geologická, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Albrechtova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Elena Raucinova</t>
+          <t xml:space="preserve">MARZE MARZE </t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -2271,12 +2271,12 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Ružová dolina, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Geologická, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Michal Sadloň</t>
+          <t>Elena Raucinova</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2293,17 +2293,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Okružná ulica, Tomášov, okres Senec</t>
+          <t>Ružová dolina, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>D P</t>
+          <t>Michal Sadloň</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -2315,12 +2315,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Bratislava-Vajnory, okres Bratislava III</t>
+          <t>Okružná ulica, Tomášov, okres Senec</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Radoslav Totkovic</t>
+          <t>D P</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2337,17 +2337,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Rudroffova, Bratislava-Rača, okres Bratislava III</t>
+          <t>Bratislava-Vajnory, okres Bratislava III</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Ján Vlk</t>
+          <t>Radoslav Totkovic</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -2359,17 +2359,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Krížna 1, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Rudroffova, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Hadi Beheshti</t>
+          <t>Ján Vlk</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -2381,17 +2381,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Dostojevského rad, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Krížna 1, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Lara Ondrejková</t>
+          <t>Hadi Beheshti</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -2403,17 +2403,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Vysoká pri Morave, okres Malacky</t>
+          <t>Dostojevského rad, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Dalibor Švihla</t>
+          <t>Lara Ondrejková</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Mobilný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -2425,17 +2425,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Bernolákovská, Ivanka pri Dunaji, okres Senec</t>
+          <t>Vysoká pri Morave, okres Malacky</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Oľga Šimáková</t>
+          <t>Dalibor Švihla</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Mobilný dom</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -2447,17 +2447,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Miletičova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bernolákovská, Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Lubo Stransky</t>
+          <t>Oľga Šimáková</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -2469,17 +2469,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Segnerova, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Miletičova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Samuel Kovalčík</t>
+          <t>Lubo Stransky</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -2491,17 +2491,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Jánošíkova, Malacky, okres Malacky</t>
+          <t>Segnerova, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Viliam Pavelka</t>
+          <t>Samuel Kovalčík</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -2513,17 +2513,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Bartoškova, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Jánošíkova, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Tibor S</t>
+          <t>Viliam Pavelka</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -2535,17 +2535,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>D. Skuteckého 1650, Malacky, okres Malacky</t>
+          <t>Bartoškova, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Mario Kral</t>
+          <t>Tibor S</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Double studio apartment</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
@@ -2557,17 +2557,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Dukelská, Modra, okres Pezinok</t>
+          <t>D. Skuteckého 1650, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Maroš Németh</t>
+          <t>Mario Kral</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Double studio apartment</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
@@ -2579,12 +2579,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Tajovského, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Dukelská, Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Martin Gažo</t>
+          <t>Maroš Németh</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2601,17 +2601,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Tajovského, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Tomas Riegel</t>
+          <t>Martin Gažo</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
@@ -2623,17 +2623,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Bratislavská 49, Senec, okres Senec</t>
+          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Vlado Svorec</t>
+          <t>Tomas Riegel</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Obchodné priestory</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -2645,17 +2645,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Kpt. Jána Rašu, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Bratislavská 49, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Monika Manova</t>
+          <t>Vlado Svorec</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Obchodné priestory</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
@@ -2667,17 +2667,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Chorvátsky Grob, okres Senec</t>
+          <t>Kpt. Jána Rašu, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Viliam Červenka</t>
+          <t>Monika Manova</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -2689,17 +2689,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Budatínska 22, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Martin Hraboš</t>
+          <t>Viliam Červenka</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
@@ -2711,12 +2711,12 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Studenohorská, Bratislava-Lamač, okres Bratislava IV</t>
+          <t>Budatínska 22, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Richard Remeník</t>
+          <t>Martin Hraboš</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2733,17 +2733,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Žltá 2A, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Studenohorská, Bratislava-Lamač, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Peter Slánský</t>
+          <t>Richard Remeník</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
@@ -2755,17 +2755,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Banšelova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Žltá 2A, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Miroslava Mihalikova</t>
+          <t>Peter Slánský</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
@@ -2777,17 +2777,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Máchova 11, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Banšelova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Marian Varga</t>
+          <t>Miroslava Mihalikova</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
@@ -2799,12 +2799,12 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Bratislava-Rusovce, okres Bratislava V</t>
+          <t>Máchova 11, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Milan Dzilsky</t>
+          <t>Marian Varga</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -2821,17 +2821,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Rozvodná, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Bratislava-Rusovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Daniela Súkromná osoba</t>
+          <t>Milan Dzilsky</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
@@ -2843,17 +2843,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
+          <t>Rozvodná, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Michal POLÁČEK</t>
+          <t>Daniela Súkromná osoba</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
@@ -2865,17 +2865,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Častá, okres Pezinok</t>
+          <t>Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Monika Zatkalíková</t>
+          <t>Michal POLÁČEK</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Záhradná chatka</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
@@ -2887,17 +2887,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Arménska, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Častá, okres Pezinok</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARZE MARZE </t>
+          <t>Monika Zatkalíková</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Záhradná chatka</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
@@ -2909,17 +2909,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Športová, Limbach, okres Pezinok</t>
+          <t>Arménska, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Michal Mravec</t>
+          <t xml:space="preserve">MARZE MARZE </t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
@@ -2931,17 +2931,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Železničiarska, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Športová, Limbach, okres Pezinok</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Dávid Uličný</t>
+          <t>Michal Mravec</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
@@ -2953,17 +2953,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Balkánska 67, Bratislava-Rusovce, okres Bratislava V</t>
+          <t>Železničiarska, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Peter Kalas</t>
+          <t>Dávid Uličný</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
@@ -2975,12 +2975,12 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Malacky, okres Malacky</t>
+          <t>Balkánska 67, Bratislava-Rusovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>pán Budkovský</t>
+          <t>Peter Kalas</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -2997,17 +2997,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Jána Jonáša, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
+          <t>Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Jana Švecová</t>
+          <t>pán Budkovský</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
@@ -3019,17 +3019,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Horská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Jána Jonáša, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Michaela Weberova</t>
+          <t>Jana Švecová</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Mezonet</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
@@ -3051,7 +3051,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Mezonet</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
@@ -3063,17 +3063,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Tallerova 4, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Horská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Daniela Ondriašová</t>
+          <t>Michaela Weberova</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
@@ -3085,17 +3085,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Bernolákova ulica, Miloslavov, okres Senec</t>
+          <t>Tallerova 4, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Erik Mihok</t>
+          <t>Daniela Ondriašová</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
@@ -3107,17 +3107,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Východná, Bratislava-Rača, okres Bratislava III</t>
+          <t>Bernolákova ulica, Miloslavov, okres Senec</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Marek Vodička</t>
+          <t>Erik Mihok</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
@@ -3129,17 +3129,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Bratislava-Rusovce, okres Bratislava V</t>
+          <t>Východná, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Alexandra Belašičová</t>
+          <t>Marek Vodička</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D122" s="4" t="inlineStr">
@@ -3151,17 +3151,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Letná 392, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Bratislava-Rusovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Magdaléna Jakubíková</t>
+          <t>Alexandra Belašičová</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D123" s="4" t="inlineStr">
@@ -3173,12 +3173,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>L. Novomeského, Pezinok, okres Pezinok</t>
+          <t>Letná 392, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Stefan PASTVA</t>
+          <t>Magdaléna Jakubíková</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -3195,17 +3195,17 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Pri Pálenici, Ivanka pri Dunaji, okres Senec</t>
+          <t>L. Novomeského, Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Dominika Ševčíková</t>
+          <t>Stefan PASTVA</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
@@ -3217,17 +3217,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Vyšehradská, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Pri Pálenici, Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Anna Zábrelová</t>
+          <t>Dominika Ševčíková</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D126" s="4" t="inlineStr">
@@ -3239,17 +3239,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Vígľašská, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Vyšehradská, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Kristína Gatyášová</t>
+          <t>Anna Zábrelová</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
@@ -3261,17 +3261,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>M. Schneidra - Trnavského, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Vígľašská, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Miroslav Potančok</t>
+          <t>Kristína Gatyášová</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D128" s="4" t="inlineStr">
@@ -3283,17 +3283,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Zidiny, Bratislava-Lamač, okres Bratislava IV</t>
+          <t>M. Schneidra - Trnavského, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Vratislav Jurica</t>
+          <t>Miroslav Potančok</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
@@ -3305,17 +3305,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Hrušovská 1, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Zidiny, Bratislava-Lamač, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Juraj Vigláš</t>
+          <t>Vratislav Jurica</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Záhrada</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
@@ -6473,17 +6473,17 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>Kresánkova, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Fedákova, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Igor Lorincik</t>
+          <t>Magdaléna Helísek</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D274" s="4" t="inlineStr">
@@ -6495,17 +6495,17 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Fedákova, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Hany Meličkovej, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Magdaléna Helísek</t>
+          <t>Viera Peterkova</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D275" s="4" t="inlineStr">
@@ -6517,12 +6517,12 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Hany Meličkovej, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Haburská, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Viera Peterkova</t>
+          <t>M Žitňanská</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -6539,17 +6539,17 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Haburská, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Lamač, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>M Žitňanská</t>
+          <t>E S</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D277" s="4" t="inlineStr">
@@ -6561,17 +6561,17 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Bratislava-Lamač, okres Bratislava IV</t>
+          <t>Hamuliakovo, okres Senec</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>E S</t>
+          <t>Sebastian Bognár</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D278" s="4" t="inlineStr">
@@ -6583,12 +6583,12 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Hamuliakovo, okres Senec</t>
+          <t>Senec, okres Senec</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Sebastian Bognár</t>
+          <t>Jana Muhlova</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -6605,17 +6605,17 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Senec, okres Senec</t>
+          <t>Košická, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Jana Muhlova</t>
+          <t>Timea Henry</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D280" s="4" t="inlineStr">
@@ -6637,7 +6637,7 @@
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D281" s="4" t="inlineStr">
@@ -6649,17 +6649,17 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Košická, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Jantárová, Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Timea Henry</t>
+          <t>Monika Szocsova</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D282" s="4" t="inlineStr">
@@ -6671,17 +6671,17 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Jantárová, Bratislava-Jarovce, okres Bratislava V</t>
+          <t>Západný rad, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Monika Szocsova</t>
+          <t>Iveta Kopecká</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D283" s="4" t="inlineStr">
@@ -6693,7 +6693,7 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Západný rad, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Gaštanová 9, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
@@ -6703,7 +6703,7 @@
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D284" s="4" t="inlineStr">
@@ -6715,17 +6715,17 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Gaštanová 9, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Jána L.Bellu (Lužianky), Senec, okres Senec</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Iveta Kopecká</t>
+          <t>Marian Mičko</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D285" s="4" t="inlineStr">
@@ -6737,17 +6737,17 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Jána L.Bellu (Lužianky), Senec, okres Senec</t>
+          <t>Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>Marian Mičko</t>
+          <t>Jozef súkromná osoba</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Hotel / penzión</t>
         </is>
       </c>
       <c r="D286" s="4" t="inlineStr">
@@ -6759,17 +6759,17 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Modra, okres Pezinok</t>
+          <t>Dunajská, Most pri Bratislave, okres Senec</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Jozef súkromná osoba</t>
+          <t>Ľuboš Štvrtecký</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Hotel / penzión</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D287" s="4" t="inlineStr">
@@ -6781,17 +6781,17 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Dunajská, Most pri Bratislave, okres Senec</t>
+          <t>Pionierska, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Ľuboš Štvrtecký</t>
+          <t>Peter Nagy</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D288" s="4" t="inlineStr">
@@ -6803,17 +6803,17 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>Pionierska, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Koniarková, Bratislava-Vajnory, okres Bratislava III</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Peter Nagy</t>
+          <t>Daniela Kiniková</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D289" s="4" t="inlineStr">
@@ -6825,17 +6825,17 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>Koniarková, Bratislava-Vajnory, okres Bratislava III</t>
+          <t>Opálová, Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Daniela Kiniková</t>
+          <t>Jana Malisova</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D290" s="4" t="inlineStr">
@@ -6847,17 +6847,17 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>Opálová, Bratislava-Jarovce, okres Bratislava V</t>
+          <t>Hydinárska 9617, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Jana Malisova</t>
+          <t>Alex Medek</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D291" s="4" t="inlineStr">
@@ -6869,12 +6869,12 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>Hydinárska 9617, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Slnečné jazerá, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Alex Medek</t>
+          <t>Filip Lečko</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
@@ -6891,17 +6891,17 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>Slnečné jazerá, Senec, okres Senec</t>
+          <t>Pod Vtáčnikom, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
         <is>
-          <t>Filip Lečko</t>
+          <t>Ivan Sanislo</t>
         </is>
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D293" s="4" t="inlineStr">
@@ -6913,17 +6913,17 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>Pod Vtáčnikom, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Pekná 1061, Veľké Leváre, okres Malacky</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Ivan Sanislo</t>
+          <t>Valéria Micháleková</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D294" s="4" t="inlineStr">
@@ -6935,12 +6935,12 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Pekná 1061, Veľké Leváre, okres Malacky</t>
+          <t>Avanárska, Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Valéria Micháleková</t>
+          <t>Julius Bohunsky</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
@@ -6957,17 +6957,17 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Avanárska, Rohožník, okres Malacky</t>
+          <t>Dlhé diely, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Julius Bohunsky</t>
+          <t>Matusk Tomas</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D296" s="4" t="inlineStr">
@@ -6979,17 +6979,17 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>Dlhé diely, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Jozefa Kubinu, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Matusk Tomas</t>
+          <t>Martina Hlubocká</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D297" s="4" t="inlineStr">
@@ -7001,17 +7001,17 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>Jozefa Kubinu, Malacky, okres Malacky</t>
+          <t>Markova 7, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Martina Hlubocká</t>
+          <t>Martin Číž</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D298" s="4" t="inlineStr">
@@ -7023,17 +7023,17 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>Markova 7, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Martin Číž</t>
+          <t>Peter Kovár</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D299" s="4" t="inlineStr">
@@ -7045,17 +7045,17 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Steinov dvor, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Peter Kovár</t>
+          <t>Ing Šalátová Zuzana</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D300" s="4" t="inlineStr">
@@ -7067,17 +7067,17 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>Steinov dvor, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Svätý Martin, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Ing Šalátová Zuzana</t>
+          <t>Stanislav Sakac</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D301" s="4" t="inlineStr">
@@ -7089,17 +7089,17 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>Svätý Martin, Senec, okres Senec</t>
+          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Stanislav Sakac</t>
+          <t>Sandra zahradnikova</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D302" s="4" t="inlineStr">
@@ -7111,17 +7111,17 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Žižkova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Sandra zahradnikova</t>
+          <t>Denisa Slančová</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
@@ -7133,17 +7133,17 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Žižkova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Strmý vŕšok 164, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Denisa Slančová</t>
+          <t>Tereza Adámyová</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D304" s="4" t="inlineStr">
@@ -7155,17 +7155,17 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Strmý vŕšok 164, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
+          <t>Lackova, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Tereza Adámyová</t>
+          <t>Predaj Bytu</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D305" s="4" t="inlineStr">
@@ -7177,17 +7177,17 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Lackova, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Predaj Bytu</t>
+          <t>Tatiana B</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D306" s="4" t="inlineStr">
@@ -7199,17 +7199,17 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Rohožník, okres Malacky</t>
+          <t>Vlastenecké námestie, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Tatiana B</t>
+          <t>Luboš Wenzl</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
@@ -7221,12 +7221,12 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>Vlastenecké námestie, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Nevädzová 6, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Luboš Wenzl</t>
+          <t>Daniel l</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
@@ -7243,12 +7243,12 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>Nevädzová 6, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Makovického, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Daniel l</t>
+          <t>Predaj Nehnutelosti</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
@@ -7265,17 +7265,17 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>Makovického, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Čsl. parašutistov, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Predaj Nehnutelosti</t>
+          <t>Tomáš Tóth</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D310" s="4" t="inlineStr">
@@ -7287,12 +7287,12 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>Čsl. parašutistov, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Holíčska 9, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Tomáš Tóth</t>
+          <t>Zuzana Pišteková</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
@@ -7309,17 +7309,17 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>Holíčska 9, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Talihov dvor, Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Zuzana Pišteková</t>
+          <t>Marian Virgovič</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Záhrada</t>
         </is>
       </c>
       <c r="D312" s="4" t="inlineStr">
@@ -7331,17 +7331,17 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>Talihov dvor, Pezinok, okres Pezinok</t>
+          <t>Račianska 64, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Marian Virgovič</t>
+          <t>Roman Miškulynets</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>Záhrada</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr">
@@ -7353,17 +7353,17 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>Račianska 64, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Suchý vrch, Limbach, okres Pezinok</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Roman Miškulynets</t>
+          <t>Miloslav Moravec</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Zrub / chalupa</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
@@ -7375,17 +7375,17 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Suchý vrch, Limbach, okres Pezinok</t>
+          <t>Ružová dolina 16, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Miloslav Moravec</t>
+          <t>Ľuboš Ľahký</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>Zrub / chalupa</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D315" s="4" t="inlineStr">
@@ -7397,17 +7397,17 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Ružová dolina 16, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Na vrátkach, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Ľuboš Ľahký</t>
+          <t>Roland Samek</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D316" s="4" t="inlineStr">
@@ -7419,17 +7419,17 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Na vrátkach, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Námestie 1. mája 3866, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Roland Samek</t>
+          <t>Oleksiy Namestie</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Polyfunkčná budova</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
@@ -7441,17 +7441,17 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Námestie 1. mája 3866, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Nejedlého 3394, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Oleksiy Namestie</t>
+          <t>Vladimír Žiga</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>Polyfunkčná budova</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
@@ -7463,12 +7463,12 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>Nejedlého 3394, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Limbašská cesta, Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Vladimír Žiga</t>
+          <t>Ganna Naichuk</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -7485,17 +7485,17 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>Limbašská cesta, Pezinok, okres Pezinok</t>
+          <t>Kristy Bendovej, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Ganna Naichuk</t>
+          <t>Jana Gottstein</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr">
@@ -7507,17 +7507,17 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>Kristy Bendovej, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Sklenárova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Jana Gottstein</t>
+          <t>Dagmar Ivanová</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr">
@@ -7529,17 +7529,17 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>Sklenárova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Pod vŕškom, Stupava, okres Malacky</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Dagmar Ivanová</t>
+          <t>Lenka Višňovská</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D322" s="4" t="inlineStr">
@@ -7551,17 +7551,17 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>Pod vŕškom, Stupava, okres Malacky</t>
+          <t>Galbavého 1, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Lenka Višňovská</t>
+          <t>Denisa Lukačovičová</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Obchodné priestory</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
@@ -7573,17 +7573,17 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>Galbavého 1, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Vážska, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Denisa Lukačovičová</t>
+          <t>Kristína Erazmusová</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>Obchodné priestory</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
@@ -7595,17 +7595,17 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>Vážska, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Stromová 25, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Kristína Erazmusová</t>
+          <t>Michal Rusek</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D325" s="4" t="inlineStr">
@@ -7617,17 +7617,17 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>Stromová 25, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Chatová rekreačná oblasť, Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Michal Rusek</t>
+          <t>M J</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Zrub / chalupa</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr">
@@ -7639,17 +7639,17 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>Chatová rekreačná oblasť, Rohožník, okres Malacky</t>
+          <t>Hagarova, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>M J</t>
+          <t>Pavol Kusenda</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>Zrub / chalupa</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr">
@@ -7661,17 +7661,17 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>Hagarova, Bratislava-Rača, okres Bratislava III</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Pavol Kusenda</t>
+          <t>L G</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
@@ -7683,17 +7683,17 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Námestie Hraničiarov, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>L G</t>
+          <t>predaj nehnutelnosti</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D329" s="4" t="inlineStr">
@@ -7705,17 +7705,17 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>Námestie Hraničiarov, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Chotárna, Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>predaj nehnutelnosti</t>
+          <t>Tomáš Stolárik</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr">
@@ -7727,17 +7727,17 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>Chotárna, Bratislava-Jarovce, okres Bratislava V</t>
+          <t>Vavrinecká, Limbach, okres Pezinok</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Tomáš Stolárik</t>
+          <t>Peter Petrina</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D331" s="4" t="inlineStr">
@@ -7749,17 +7749,17 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>Vavrinecká, Limbach, okres Pezinok</t>
+          <t>Komenského 2, Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Peter Petrina</t>
+          <t>Andrej B</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
@@ -7771,17 +7771,17 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>Komenského 2, Modra, okres Pezinok</t>
+          <t>Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>Andrej B</t>
+          <t>Soňa Slobodníková</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D333" s="4" t="inlineStr">
@@ -7793,17 +7793,17 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>Bratislava-Jarovce, okres Bratislava V</t>
+          <t>Na Revíne 19, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Soňa Slobodníková</t>
+          <t>Dušan Cintula</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D334" s="4" t="inlineStr">
@@ -7815,12 +7815,12 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>Na Revíne 19, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Hrušková 44H, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>Dušan Cintula</t>
+          <t>Jasna Rumanková</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -7837,17 +7837,17 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>Hrušková 44H, Bratislava-Rača, okres Bratislava III</t>
+          <t>Martina Granca, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Jasna Rumanková</t>
+          <t>Michal Michal</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D336" s="4" t="inlineStr">
@@ -7859,17 +7859,17 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>Martina Granca, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Konventná 5, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>Michal Michal</t>
+          <t>Vladimir Taraba</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D337" s="4" t="inlineStr">
@@ -7881,12 +7881,12 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>Konventná 5, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Landererova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Vladimir Taraba</t>
+          <t>Jan Kovac</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -7903,17 +7903,17 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>Landererova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Jan Kovac</t>
+          <t>Tomáš Machciník</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D339" s="4" t="inlineStr">
@@ -7925,12 +7925,12 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>Pezinok, okres Pezinok</t>
+          <t>Malokarpatská 1, Svätý Jur, okres Pezinok</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Tomáš Machciník</t>
+          <t>Jana Zárecká</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -7947,17 +7947,17 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>Malokarpatská 1, Svätý Jur, okres Pezinok</t>
+          <t>Panónska cesta, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Jana Zárecká</t>
+          <t>Oliver Práznovský</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D341" s="4" t="inlineStr">
@@ -7969,17 +7969,17 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>Panónska cesta, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Mariánska cesta, Svätý Jur, okres Pezinok</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Oliver Práznovský</t>
+          <t>Marian Machalek</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rekreačný pozemok</t>
         </is>
       </c>
       <c r="D342" s="4" t="inlineStr">
@@ -7991,17 +7991,17 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>Mariánska cesta, Svätý Jur, okres Pezinok</t>
+          <t>Homolova, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Marian Machalek</t>
+          <t>Jaroslav Janco</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>Rekreačný pozemok</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D343" s="4" t="inlineStr">
@@ -8013,17 +8013,17 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>Homolova, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Potočná, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Jaroslav Janco</t>
+          <t>Pavol Beblavy</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D344" s="4" t="inlineStr">
@@ -8035,12 +8035,12 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>Potočná, Bratislava-Rača, okres Bratislava III</t>
+          <t>Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Pavol Beblavy</t>
+          <t>Peter Urban</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -8057,17 +8057,17 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>Pezinok, okres Pezinok</t>
+          <t>Miletičova 60, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Peter Urban</t>
+          <t>Michael Kollár</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D346" s="4" t="inlineStr">
@@ -8079,17 +8079,17 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>Miletičova 60, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Svätovavrinecká, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Michael Kollár</t>
+          <t>Katarína Rusňáková</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>5+ izbový byt</t>
         </is>
       </c>
       <c r="D347" s="4" t="inlineStr">
@@ -8101,17 +8101,17 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>Svätovavrinecká, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Hraničiarska, Vysoká pri Morave, okres Malacky</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Katarína Rusňáková</t>
+          <t>Andrea Bencová</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>5+ izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D348" s="4" t="inlineStr">
@@ -8123,17 +8123,17 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>Hraničiarska, Vysoká pri Morave, okres Malacky</t>
+          <t>Bajkalská, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Andrea Bencová</t>
+          <t>Jakub Osuský</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D349" s="4" t="inlineStr">
@@ -8142,52 +8142,8 @@
         </is>
       </c>
     </row>
-    <row r="350">
-      <c r="A350" t="inlineStr">
-        <is>
-          <t>Bajkalská, Bratislava-Ružinov, okres Bratislava II</t>
-        </is>
-      </c>
-      <c r="B350" t="inlineStr">
-        <is>
-          <t>Jakub Osuský</t>
-        </is>
-      </c>
-      <c r="C350" t="inlineStr">
-        <is>
-          <t>3-izbový byt</t>
-        </is>
-      </c>
-      <c r="D350" s="4" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
-    <row r="351">
-      <c r="A351" t="inlineStr">
-        <is>
-          <t>Devínska cesta, Bratislava-Devín, okres Bratislava IV</t>
-        </is>
-      </c>
-      <c r="B351" t="inlineStr">
-        <is>
-          <t>ales malina</t>
-        </is>
-      </c>
-      <c r="C351" t="inlineStr">
-        <is>
-          <t>Záhradná chatka</t>
-        </is>
-      </c>
-      <c r="D351" s="4" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D351"/>
+  <autoFilter ref="A1:D349"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -8537,8 +8493,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D347" r:id="rId346"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D348" r:id="rId347"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D349" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D350" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D351" r:id="rId350"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8571,7 +8525,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>350</v>
+        <v>348</v>
       </c>
     </row>
     <row r="4">
@@ -8582,7 +8536,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>25.09.2026 16:04</t>
+          <t>25.09.2026 20:42</t>
         </is>
       </c>
     </row>
@@ -8622,7 +8576,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>54</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10">
@@ -8642,7 +8596,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12">
@@ -8652,7 +8606,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="13">
@@ -8711,7 +8665,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="20">
@@ -8721,7 +8675,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
     </row>
     <row r="21">
@@ -8807,17 +8761,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Záhrada</t>
+          <t>Rekreačný pozemok</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Rekreačný pozemok</t>
+          <t>Mobilný dom</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -8827,7 +8781,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Mobilný dom</t>
+          <t>Záhrada</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -8837,17 +8791,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Záhradná chatka</t>
+          <t>5+ izbový byt</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>5+ izbový byt</t>
+          <t>Zmiešaná zóna</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -8857,7 +8811,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Zmiešaná zóna</t>
+          <t>Iný priestor</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -8867,7 +8821,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Iný priestor</t>
+          <t>Záhradná chatka</t>
         </is>
       </c>
       <c r="B35" t="n">

</xml_diff>

<commit_message>
Aktualizácia ponúk – 2026-09-28 22:43 UTC
</commit_message>
<xml_diff>
--- a/public/ponuky.xlsx
+++ b/public/ponuky.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Prehľad" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ponuky'!$A$1:$D$355</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ponuky'!$A$1:$D$357</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D355"/>
+  <dimension ref="A1:D357"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -489,17 +489,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Heyrovského, Bratislava-Lamač, okres Bratislava IV</t>
+          <t>Družstevná, Bernolákovo, okres Senec</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Maros Palik</t>
+          <t>Michaela Jancek</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
@@ -511,12 +511,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Oravská 2, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Planét, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Zdena Bartošová</t>
+          <t>Július Július</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -533,17 +533,17 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Jarabinková 2, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Skalná, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Michael Kollár</t>
+          <t>katarina sekerka</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -555,12 +555,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Miletičova 60, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Heyrovského, Bratislava-Lamač, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Michael Kollár</t>
+          <t>Maros Palik</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -577,17 +577,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Bernolákova 2, Senec, okres Senec</t>
+          <t>Oravská 2, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Šimon Klúčik</t>
+          <t>Zdena Bartošová</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -599,17 +599,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rovinka, okres Senec</t>
+          <t>Jarabinková 2, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Petra Sárkány</t>
+          <t>Michael Kollár</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -621,17 +621,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>J. Holčeka, Budmerice, okres Pezinok</t>
+          <t>Miletičova 60, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Ondrej Kolciter</t>
+          <t>Michael Kollár</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -643,17 +643,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>J. Holčeka, Budmerice, okres Pezinok</t>
+          <t>Bernolákova 2, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Ondrej Kolciter</t>
+          <t>Šimon Klúčik</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -665,12 +665,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Chorvátsky Grob, okres Senec</t>
+          <t>Rovinka, okres Senec</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Dada Garajova</t>
+          <t>Petra Sárkány</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -687,17 +687,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bajkalská 45C, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>J. Holčeka, Budmerice, okres Pezinok</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Eva Valáriková</t>
+          <t>Ondrej Kolciter</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -709,17 +709,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Trebišovská, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>J. Holčeka, Budmerice, okres Pezinok</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Ružinov Štrkovec</t>
+          <t>Ondrej Kolciter</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -731,17 +731,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Rohožník, okres Malacky</t>
+          <t>Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Sukromna Osoba</t>
+          <t>Dada Garajova</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -753,17 +753,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Senec, okres Senec</t>
+          <t>Bajkalská 45C, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Jakub Králik</t>
+          <t>Eva Valáriková</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -775,17 +775,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Tomášikova 50A, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Trebišovská, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Daria Denisova</t>
+          <t>Ružinov Štrkovec</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -797,12 +797,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Malacky, okres Malacky</t>
+          <t>Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Elena Straznicka</t>
+          <t>Sukromna Osoba</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -819,17 +819,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Holubia, Senec, okres Senec</t>
+          <t>Senec, okres Senec</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Marko Klúčik</t>
+          <t>Jakub Králik</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -841,17 +841,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>1mája, Pezinok, okres Pezinok</t>
+          <t>Tomášikova 50A, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Ladislav Ružek</t>
+          <t>Daria Denisova</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -863,12 +863,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Lukas Durinak</t>
+          <t>Elena Straznicka</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -885,17 +885,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Okružná 47, Senec, okres Senec</t>
+          <t>Holubia, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Roman Gazdik</t>
+          <t>Marko Klúčik</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -907,17 +907,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Slovenský Grob, okres Pezinok</t>
+          <t>1mája, Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Igor Šramka</t>
+          <t>Ladislav Ružek</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -929,17 +929,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Kozia, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Ľubor Mendel</t>
+          <t>Lukas Durinak</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -951,17 +951,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Dopravná 23, Bratislava-Rača, okres Bratislava III</t>
+          <t>Okružná 47, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Peter Pipiš</t>
+          <t>Roman Gazdik</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -973,17 +973,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Šalviová, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Slovenský Grob, okres Pezinok</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Juraj Valašťan</t>
+          <t>Igor Šramka</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -995,17 +995,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Agátová, Ivanka pri Dunaji, okres Senec</t>
+          <t>Kozia, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Viktória Krupová</t>
+          <t>Ľubor Mendel</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1017,17 +1017,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Kaplinská 7, Bratislava-Rača, okres Bratislava III</t>
+          <t>Dopravná 23, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Eva Žíhlavníková</t>
+          <t>Peter Pipiš</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1039,17 +1039,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Repašského 1, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Šalviová, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Michal Weismann</t>
+          <t>Juraj Valašťan</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1061,17 +1061,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Repašského 1, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Agátová, Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Michal Weismann</t>
+          <t>Viktória Krupová</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -1083,17 +1083,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Kaplinská 7, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Alexander Kernaševič</t>
+          <t>Eva Žíhlavníková</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Mobile cells and stands</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1105,17 +1105,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Landererova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Repašského 1, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Simona Kourdi</t>
+          <t>Michal Weismann</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -1127,17 +1127,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>167, Borinka, okres Malacky</t>
+          <t>Repašského 1, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Kamil Semeš</t>
+          <t>Michal Weismann</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1149,17 +1149,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Gregorovej, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Andrej Miko</t>
+          <t>Alexander Kernaševič</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Mobile cells and stands</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -1171,17 +1171,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Jablonec, okres Pezinok</t>
+          <t>Landererova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Andrea Valentová</t>
+          <t>Simona Kourdi</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -1193,17 +1193,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Ivanka pri Dunaji, okres Senec</t>
+          <t>167, Borinka, okres Malacky</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Andrea Bášková</t>
+          <t>Kamil Semeš</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -1215,17 +1215,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Gregorovej, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Katarína Rusňáková</t>
+          <t>Andrej Miko</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -1237,17 +1237,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Ulica 8. mája 22A, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Jablonec, okres Pezinok</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Vladimír Mitrík</t>
+          <t>Andrea Valentová</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -1259,17 +1259,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Partizánska 1081, Malacky, okres Malacky</t>
+          <t>Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Peter Ondrovič</t>
+          <t>Andrea Bášková</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -1281,17 +1281,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Čulenova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>M I</t>
+          <t>Katarína Rusňáková</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -1303,17 +1303,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Lachova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Ulica 8. mája 22A, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Zuzana V</t>
+          <t>Vladimír Mitrík</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -1325,17 +1325,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Drobného, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Partizánska 1081, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Peter Chovanec</t>
+          <t>Peter Ondrovič</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -1347,17 +1347,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Vysoká pri Morave, okres Malacky</t>
+          <t>Čulenova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Miroslav Vojkovic</t>
+          <t>M I</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -1369,17 +1369,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Vinárska, Modra, okres Pezinok</t>
+          <t>Lachova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>marek rozic</t>
+          <t>Zuzana V</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -1391,12 +1391,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Drobného, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Anton K</t>
+          <t>Peter Chovanec</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1413,17 +1413,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Tupolevova 18, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Vysoká pri Morave, okres Malacky</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Ivan Hargas</t>
+          <t>Miroslav Vojkovic</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -1435,17 +1435,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Stavbárska 4, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Vinárska, Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Jaroslav Valus</t>
+          <t>marek rozic</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -1457,17 +1457,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Bratislava-Vajnory, okres Bratislava III</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Juraj Varacka</t>
+          <t>Anton K</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -1479,12 +1479,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Tupolevova 18, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Juraj Litomerický</t>
+          <t>Ivan Hargas</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1501,17 +1501,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Vyšehradská 16, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Stavbárska 4, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Juraj Kovašich</t>
+          <t>Jaroslav Valus</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -1523,17 +1523,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Grösslingova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bratislava-Vajnory, okres Bratislava III</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Viktor Riegel</t>
+          <t>Juraj Varacka</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -1545,17 +1545,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Sekurisova, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Matej Kohucik</t>
+          <t>Juraj Litomerický</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -1567,17 +1567,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Ipeľská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Vyšehradská 16, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>David Ivanov</t>
+          <t>Juraj Kovašich</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -1589,17 +1589,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Karloveské rameno, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Grösslingova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Boris Emrich</t>
+          <t>Viktor Riegel</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -1611,12 +1611,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Landauova, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Sekurisova, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>peter klvac</t>
+          <t>Matej Kohucik</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1633,17 +1633,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Malokrasňanská 8, Bratislava-Rača, okres Bratislava III</t>
+          <t>Ipeľská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Paula Baranová</t>
+          <t>David Ivanov</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -1655,17 +1655,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Tomášikova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Karloveské rameno, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>BaTom P</t>
+          <t>Boris Emrich</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -1677,17 +1677,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Krížna, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Landauova, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Peter Valenta</t>
+          <t>peter klvac</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Kancelárie</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -1699,17 +1699,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Námestie Slobody, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Malokrasňanská 8, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Martin Gažo</t>
+          <t>Paula Baranová</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -1721,17 +1721,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Bratislava-Rusovce, okres Bratislava V</t>
+          <t>Tomášikova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Milan Dzilsky</t>
+          <t>BaTom P</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -1743,17 +1743,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Rovniankova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Krížna, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Roman N</t>
+          <t>Peter Valenta</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Kancelárie</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -1765,12 +1765,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Námestie Slobody, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Martin Chamko</t>
+          <t>Martin Gažo</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1787,17 +1787,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Jaskový rad 47, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Bratislava-Rusovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Angela Brinzova</t>
+          <t>Milan Dzilsky</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -1809,17 +1809,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Podjavorinskej 13, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Rovniankova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Tomáš Čitbaj</t>
+          <t>Roman N</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -1831,17 +1831,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Krušpánová, Bratislava-Čunovo, okres Bratislava V</t>
+          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Alena Horváthová</t>
+          <t>Martin Chamko</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -1853,17 +1853,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Rovniankova 20, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Jaskový rad 47, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Michal Weismann</t>
+          <t>Angela Brinzova</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -1875,17 +1875,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Rovniankova 20, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Podjavorinskej 13, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Michal Weismann</t>
+          <t>Tomáš Čitbaj</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -1897,17 +1897,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Šancová 37, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Krušpánová, Bratislava-Čunovo, okres Bratislava V</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Frantisek Manduch</t>
+          <t>Alena Horváthová</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -1919,17 +1919,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Miloslavov, okres Senec</t>
+          <t>Šancová 37, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Jakub Hronec</t>
+          <t>Frantisek Manduch</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -1941,17 +1941,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Malé Leváre, okres Malacky</t>
+          <t>Miloslavov, okres Senec</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Michal Fajták</t>
+          <t>Jakub Hronec</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -1963,17 +1963,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Komenského, Modra, okres Pezinok</t>
+          <t>Malé Leváre, okres Malacky</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Richard Baranovic</t>
+          <t>Michal Fajták</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -1985,17 +1985,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Markova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Komenského, Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Peter Novotný</t>
+          <t>Richard Baranovic</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -2007,12 +2007,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Hornádska 28, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Markova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Miro Kralovic</t>
+          <t>Peter Novotný</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -2029,12 +2029,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Plzenská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Hornádska 28, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Peter Kubica</t>
+          <t>Miro Kralovic</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2051,17 +2051,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Plzenská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Lukáš K</t>
+          <t>Peter Kubica</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -2073,17 +2073,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Hattalova, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Šťastný  Vlastník</t>
+          <t>Lukáš K</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
@@ -2095,17 +2095,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Slovenský Grob, okres Pezinok</t>
+          <t>Hattalova, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Jozef Brom</t>
+          <t>Šťastný  Vlastník</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -2117,17 +2117,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Slovenský Grob, okres Pezinok</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>MM victory</t>
+          <t>Jozef Brom</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -2139,12 +2139,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Ružinov Štrkovec</t>
+          <t>MM victory</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2161,17 +2161,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Bernolákova, Nová Dedinka, okres Senec</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Karina Szutyányiová</t>
+          <t>Ružinov Štrkovec</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -2183,17 +2183,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Senec, okres Senec</t>
+          <t>Bernolákova, Nová Dedinka, okres Senec</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>RD RD</t>
+          <t>Karina Szutyányiová</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -2205,12 +2205,12 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Školská, Rovinka, okres Senec</t>
+          <t>Senec, okres Senec</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Alena Alena</t>
+          <t>RD RD</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -2227,17 +2227,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Školská, Rovinka, okres Senec</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lukas Novosiadly </t>
+          <t>Alena Alena</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -2249,17 +2249,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Hany Zelinovej, Senec, okres Senec</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Peter Veselsky</t>
+          <t xml:space="preserve">Lukas Novosiadly </t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -2271,17 +2271,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Dunajská, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Hany Zelinovej, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Tatiana B</t>
+          <t>Peter Veselsky</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>5+ izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -2293,17 +2293,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Malacky, okres Malacky</t>
+          <t>Dunajská, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Martin Jendek</t>
+          <t>Tatiana B</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>5+ izbový byt</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -2315,12 +2315,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Antolská, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Peter K</t>
+          <t>Martin Jendek</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2337,17 +2337,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Zidiny 11, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Antolská, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Vratislav Jurica</t>
+          <t>Peter K</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -2359,17 +2359,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Čulenova 5, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Zidiny 11, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Martin Martin</t>
+          <t>Vratislav Jurica</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -2381,17 +2381,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Betliarska, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Čulenova 5, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Hana Habartova</t>
+          <t>Martin Martin</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Zmiešaná zóna</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -2403,17 +2403,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Sliačska 13903, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Betliarska, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Jan Syč</t>
+          <t>Hana Habartova</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Zmiešaná zóna</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -2425,17 +2425,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Sliačska 13903, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Denisa Slančová</t>
+          <t>Jan Syč</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -2447,17 +2447,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Dúbravčická, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Jakub Brondoš</t>
+          <t>Denisa Slančová</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Rekreačný pozemok</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -2469,17 +2469,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Miletičova 5A, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Dúbravčická, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Kristián Németh</t>
+          <t>Jakub Brondoš</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rekreačný pozemok</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -2491,12 +2491,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Vrabčia, Senec, okres Senec</t>
+          <t>Miletičova 5A, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Katarína Lattová</t>
+          <t>Kristián Németh</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -2513,17 +2513,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Lipová ulica, Hrubá Borša, okres Senec</t>
+          <t>Vrabčia, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Štefan Hencel</t>
+          <t>Katarína Lattová</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -2535,12 +2535,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Šenkvice, okres Pezinok</t>
+          <t>Lipová ulica, Hrubá Borša, okres Senec</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Jaro Jaro</t>
+          <t>Štefan Hencel</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -2557,17 +2557,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Ota Holúska, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
+          <t>Šenkvice, okres Pezinok</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Nikola Mináčová</t>
+          <t>Jaro Jaro</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
@@ -2579,17 +2579,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Plachého, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Ota Holúska, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Alojz Hančin</t>
+          <t>Nikola Mináčová</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Other object for housing</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -2601,17 +2601,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Bebravská, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Plachého, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARZE MARZE </t>
+          <t>Alojz Hančin</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Other object for housing</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
@@ -2623,17 +2623,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Banskobystrická, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bebravská, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Jozef Novák</t>
+          <t xml:space="preserve">MARZE MARZE </t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -2645,17 +2645,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Banskobystrická, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>RD RD</t>
+          <t>Jozef Novák</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
@@ -2667,17 +2667,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Peter Szell</t>
+          <t>RD RD</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Iný priestor</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -2689,17 +2689,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Albrechtova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARZE MARZE </t>
+          <t>Peter Szell</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Iný priestor</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
@@ -2711,17 +2711,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Geologická, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Albrechtova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Elena Raucinova</t>
+          <t xml:space="preserve">MARZE MARZE </t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -2733,12 +2733,12 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Ružová dolina, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Geologická, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Michal Sadloň</t>
+          <t>Elena Raucinova</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -2755,17 +2755,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Okružná ulica, Tomášov, okres Senec</t>
+          <t>Ružová dolina, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>D P</t>
+          <t>Michal Sadloň</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
@@ -2777,12 +2777,12 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Bratislava-Vajnory, okres Bratislava III</t>
+          <t>Okružná ulica, Tomášov, okres Senec</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Radoslav Totkovic</t>
+          <t>D P</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -2799,17 +2799,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Rudroffova, Bratislava-Rača, okres Bratislava III</t>
+          <t>Bratislava-Vajnory, okres Bratislava III</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Ján Vlk</t>
+          <t>Radoslav Totkovic</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
@@ -2821,17 +2821,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Krížna 1, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Rudroffova, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Hadi Beheshti</t>
+          <t>Ján Vlk</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
@@ -2843,17 +2843,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Dostojevského rad, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Krížna 1, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Lara Ondrejková</t>
+          <t>Hadi Beheshti</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
@@ -2865,17 +2865,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Vysoká pri Morave, okres Malacky</t>
+          <t>Dostojevského rad, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Dalibor Švihla</t>
+          <t>Lara Ondrejková</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Mobilný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
@@ -2887,17 +2887,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Bernolákovská, Ivanka pri Dunaji, okres Senec</t>
+          <t>Vysoká pri Morave, okres Malacky</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Oľga Šimáková</t>
+          <t>Dalibor Švihla</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Mobilný dom</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
@@ -2909,17 +2909,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Miletičova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bernolákovská, Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Lubo Stransky</t>
+          <t>Oľga Šimáková</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
@@ -2931,17 +2931,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Segnerova, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Miletičova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Samuel Kovalčík</t>
+          <t>Lubo Stransky</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
@@ -2953,17 +2953,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Jánošíkova, Malacky, okres Malacky</t>
+          <t>Segnerova, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Viliam Pavelka</t>
+          <t>Samuel Kovalčík</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
@@ -2975,17 +2975,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Bartoškova, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Jánošíkova, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Tibor S</t>
+          <t>Viliam Pavelka</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
@@ -2997,17 +2997,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>D. Skuteckého 1650, Malacky, okres Malacky</t>
+          <t>Bartoškova, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Mario Kral</t>
+          <t>Tibor S</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Double studio apartment</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
@@ -3019,17 +3019,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Dukelská, Modra, okres Pezinok</t>
+          <t>D. Skuteckého 1650, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Maroš Németh</t>
+          <t>Mario Kral</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Double studio apartment</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
@@ -3041,12 +3041,12 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Tajovského, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Dukelská, Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Martin Gažo</t>
+          <t>Maroš Németh</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -3063,17 +3063,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Tajovského, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Tomas Riegel</t>
+          <t>Martin Gažo</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
@@ -6143,17 +6143,17 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Ulica Svornosti, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Pri vinohradoch 142, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Matuš  Žemlička</t>
+          <t>Ľuboš Čmelko</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Zmiešaná zóna</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D259" s="4" t="inlineStr">
@@ -6165,17 +6165,17 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Košická 10, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Ulica Svornosti, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>David A</t>
+          <t>Matuš  Žemlička</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Zmiešaná zóna</t>
         </is>
       </c>
       <c r="D260" s="4" t="inlineStr">
@@ -6187,17 +6187,17 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>Zlatý Karas, Nová Dedinka, okres Senec</t>
+          <t>Košická 10, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Vincent Durbak</t>
+          <t>David A</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D261" s="4" t="inlineStr">
@@ -6209,17 +6209,17 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Zlatý Karas, Nová Dedinka, okres Senec</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Edmund Edmund</t>
+          <t>Vincent Durbak</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D262" s="4" t="inlineStr">
@@ -6231,17 +6231,17 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>Jedľová ulica, Zohor, okres Malacky</t>
+          <t>Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Andrea Bencová</t>
+          <t>Edmund Edmund</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D263" s="4" t="inlineStr">
@@ -6253,17 +6253,17 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Plavecký Štvrtok, okres Malacky</t>
+          <t>Jedľová ulica, Zohor, okres Malacky</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Sisi Belo</t>
+          <t>Andrea Bencová</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D264" s="4" t="inlineStr">
@@ -6275,17 +6275,17 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Baltská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Plavecký Štvrtok, okres Malacky</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>L M</t>
+          <t>Sisi Belo</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D265" s="4" t="inlineStr">
@@ -6297,12 +6297,12 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Trnavská cesta, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Baltská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>LEX vision</t>
+          <t>L M</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
@@ -6319,17 +6319,17 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Male Pole 111, Vištuk, okres Pezinok</t>
+          <t>Trnavská cesta, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Frantisek Krasnansky</t>
+          <t>LEX vision</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D267" s="4" t="inlineStr">
@@ -6341,17 +6341,17 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>Uránová, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Male Pole 111, Vištuk, okres Pezinok</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Erik Varchol</t>
+          <t>Frantisek Krasnansky</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D268" s="4" t="inlineStr">
@@ -6363,17 +6363,17 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Andreja Mráza 3160, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Uránová, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Michal Ruš</t>
+          <t>Erik Varchol</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D269" s="4" t="inlineStr">
@@ -6385,17 +6385,17 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Hlavná 10E, Nová Dedinka, okres Senec</t>
+          <t>Andreja Mráza 3160, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>Miroslava Magulova</t>
+          <t>Michal Ruš</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D270" s="4" t="inlineStr">
@@ -6407,17 +6407,17 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Veľké Leváre, okres Malacky</t>
+          <t>Hlavná 10E, Nová Dedinka, okres Senec</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>Denis  Klempa</t>
+          <t>Miroslava Magulova</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D271" s="4" t="inlineStr">
@@ -6429,12 +6429,12 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Plavecký Štvrtok, okres Malacky</t>
+          <t>Veľké Leváre, okres Malacky</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Peter J</t>
+          <t>Denis  Klempa</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
@@ -6451,17 +6451,17 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>Cementárenská, Stupava, okres Malacky</t>
+          <t>Plavecký Štvrtok, okres Malacky</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Peter Haco</t>
+          <t>Peter J</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>Polyfunkčná budova</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D273" s="4" t="inlineStr">
@@ -6473,17 +6473,17 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>Sama Chalúpku, Malacky, okres Malacky</t>
+          <t>Cementárenská, Stupava, okres Malacky</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Boris Cambalik</t>
+          <t>Peter Haco</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Polyfunkčná budova</t>
         </is>
       </c>
       <c r="D274" s="4" t="inlineStr">
@@ -6495,17 +6495,17 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Bieloruská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Sama Chalúpku, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Richard Macko</t>
+          <t>Boris Cambalik</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D275" s="4" t="inlineStr">
@@ -6517,17 +6517,17 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Cyprichova 2, Bratislava-Rača, okres Bratislava III</t>
+          <t>Bieloruská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Anna Boríková</t>
+          <t>Richard Macko</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
         <is>
-          <t>Reštauračné priestory</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D276" s="4" t="inlineStr">
@@ -6539,17 +6539,17 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Cyprichova 2, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Lucia Danišová</t>
+          <t>Anna Boríková</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Reštauračné priestory</t>
         </is>
       </c>
       <c r="D277" s="4" t="inlineStr">
@@ -6561,17 +6561,17 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Karloveské rameno, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Pavol Bak</t>
+          <t>Lucia Danišová</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Pozemok pre bytovú výstavbu</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D278" s="4" t="inlineStr">
@@ -6593,7 +6593,7 @@
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>Bytový dom</t>
+          <t>Pozemok pre bytovú výstavbu</t>
         </is>
       </c>
       <c r="D279" s="4" t="inlineStr">
@@ -6605,17 +6605,17 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Karloveské rameno, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Nova Rekonštrukcia</t>
+          <t>Pavol Bak</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Bytový dom</t>
         </is>
       </c>
       <c r="D280" s="4" t="inlineStr">
@@ -6627,17 +6627,17 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Studená, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Byt Studena</t>
+          <t>Nova Rekonštrukcia</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D281" s="4" t="inlineStr">
@@ -6649,17 +6649,17 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Krížna 1, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Studená, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>martina busova</t>
+          <t>Byt Studena</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D282" s="4" t="inlineStr">
@@ -6671,12 +6671,12 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Fedákova, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Krížna 1, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Magdaléna Helísek</t>
+          <t>martina busova</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
@@ -6693,17 +6693,17 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Hany Meličkovej, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Fedákova, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Viera Peterkova</t>
+          <t>Magdaléna Helísek</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D284" s="4" t="inlineStr">
@@ -6715,12 +6715,12 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Haburská, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Hany Meličkovej, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>M Žitňanská</t>
+          <t>Viera Peterkova</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
@@ -6737,17 +6737,17 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Bratislava-Lamač, okres Bratislava IV</t>
+          <t>Haburská, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>E S</t>
+          <t>M Žitňanská</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D286" s="4" t="inlineStr">
@@ -6759,17 +6759,17 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Hamuliakovo, okres Senec</t>
+          <t>Bratislava-Lamač, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Sebastian Bognár</t>
+          <t>E S</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D287" s="4" t="inlineStr">
@@ -6781,12 +6781,12 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Senec, okres Senec</t>
+          <t>Hamuliakovo, okres Senec</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Jana Muhlova</t>
+          <t>Sebastian Bognár</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
@@ -6803,17 +6803,17 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>Košická, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Senec, okres Senec</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>Timea Henry</t>
+          <t>Jana Muhlova</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D289" s="4" t="inlineStr">
@@ -6835,7 +6835,7 @@
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D290" s="4" t="inlineStr">
@@ -6847,17 +6847,17 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>Jantárová, Bratislava-Jarovce, okres Bratislava V</t>
+          <t>Košická, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Monika Szocsova</t>
+          <t>Timea Henry</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D291" s="4" t="inlineStr">
@@ -6869,17 +6869,17 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>Západný rad, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Jantárová, Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Iveta Kopecká</t>
+          <t>Monika Szocsova</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D292" s="4" t="inlineStr">
@@ -6891,7 +6891,7 @@
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>Gaštanová 9, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Západný rad, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B293" t="inlineStr">
@@ -6901,7 +6901,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D293" s="4" t="inlineStr">
@@ -6913,17 +6913,17 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>Jána L.Bellu (Lužianky), Senec, okres Senec</t>
+          <t>Gaštanová 9, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Marian Mičko</t>
+          <t>Iveta Kopecká</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D294" s="4" t="inlineStr">
@@ -6935,17 +6935,17 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Modra, okres Pezinok</t>
+          <t>Jána L.Bellu (Lužianky), Senec, okres Senec</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Jozef súkromná osoba</t>
+          <t>Marian Mičko</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Hotel / penzión</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D295" s="4" t="inlineStr">
@@ -6957,17 +6957,17 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Dunajská, Most pri Bratislave, okres Senec</t>
+          <t>Stavbárska 5177, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
         <is>
-          <t>Ľuboš Štvrtecký</t>
+          <t>Adriana D</t>
         </is>
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D296" s="4" t="inlineStr">
@@ -6979,17 +6979,17 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>Pionierska, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Peter Nagy</t>
+          <t>Jozef súkromná osoba</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Hotel / penzión</t>
         </is>
       </c>
       <c r="D297" s="4" t="inlineStr">
@@ -7001,17 +7001,17 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>Koniarková, Bratislava-Vajnory, okres Bratislava III</t>
+          <t>Dunajská, Most pri Bratislave, okres Senec</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Daniela Kiniková</t>
+          <t>Ľuboš Štvrtecký</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D298" s="4" t="inlineStr">
@@ -7023,17 +7023,17 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>Opálová, Bratislava-Jarovce, okres Bratislava V</t>
+          <t>Pionierska, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Jana Malisova</t>
+          <t>Peter Nagy</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D299" s="4" t="inlineStr">
@@ -7045,12 +7045,12 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>Hydinárska 9617, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Koniarková, Bratislava-Vajnory, okres Bratislava III</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Alex Medek</t>
+          <t>Daniela Kiniková</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -7067,17 +7067,17 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>Slnečné jazerá, Senec, okres Senec</t>
+          <t>Opálová, Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Filip Lečko</t>
+          <t>Jana Malisova</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D301" s="4" t="inlineStr">
@@ -7089,12 +7089,12 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>Pekná 1061, Veľké Leváre, okres Malacky</t>
+          <t>Hydinárska 9617, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Valéria Micháleková</t>
+          <t>Alex Medek</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
@@ -7111,17 +7111,17 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>Banšelova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Slnečné jazerá, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Ivan Beňo</t>
+          <t>Filip Lečko</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D303" s="4" t="inlineStr">
@@ -7133,12 +7133,12 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Avanárska, Rohožník, okres Malacky</t>
+          <t>Pekná 1061, Veľké Leváre, okres Malacky</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Julius Bohunsky</t>
+          <t>Valéria Micháleková</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
@@ -7155,12 +7155,12 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Dlhé diely, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Banšelova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Matusk Tomas</t>
+          <t>Ivan Beňo</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -7177,12 +7177,12 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Jozefa Kubinu, Malacky, okres Malacky</t>
+          <t>Avanárska, Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Martina Hlubocká</t>
+          <t>Julius Bohunsky</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
@@ -7199,17 +7199,17 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Markova 7, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Dlhé diely, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Martin Číž</t>
+          <t>Matusk Tomas</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D307" s="4" t="inlineStr">
@@ -7221,17 +7221,17 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Jozefa Kubinu, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Peter Kovár</t>
+          <t>Martina Hlubocká</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D308" s="4" t="inlineStr">
@@ -7243,17 +7243,17 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>Steinov dvor, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Markova 7, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Ing Šalátová Zuzana</t>
+          <t>Martin Číž</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D309" s="4" t="inlineStr">
@@ -7265,17 +7265,17 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>Svätý Martin, Senec, okres Senec</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Stanislav Sakac</t>
+          <t>Peter Kovár</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D310" s="4" t="inlineStr">
@@ -7287,17 +7287,17 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Steinov dvor, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Sandra zahradnikova</t>
+          <t>Ing Šalátová Zuzana</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D311" s="4" t="inlineStr">
@@ -7309,17 +7309,17 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>Žižkova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Svätý Martin, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Denisa Slančová</t>
+          <t>Stanislav Sakac</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D312" s="4" t="inlineStr">
@@ -7331,17 +7331,17 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>Strmý vŕšok 164, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
+          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Tereza Adámyová</t>
+          <t>Sandra zahradnikova</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D313" s="4" t="inlineStr">
@@ -7353,17 +7353,17 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>Lackova, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Žižkova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Predaj Bytu</t>
+          <t>Denisa Slančová</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D314" s="4" t="inlineStr">
@@ -7375,12 +7375,12 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Rohožník, okres Malacky</t>
+          <t>Strmý vŕšok 164, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Tatiana B</t>
+          <t>Tereza Adámyová</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -7397,12 +7397,12 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Nevädzová 6, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Lackova, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Daniel l</t>
+          <t>Predaj Bytu</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -7419,17 +7419,17 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Makovického, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Predaj Nehnutelosti</t>
+          <t>Tatiana B</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D317" s="4" t="inlineStr">
@@ -7441,17 +7441,17 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Čsl. parašutistov, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Nevädzová 6, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Tomáš Tóth</t>
+          <t>Daniel l</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D318" s="4" t="inlineStr">
@@ -7463,17 +7463,17 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>Holíčska 9, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Makovického, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Zuzana Pišteková</t>
+          <t>Predaj Nehnutelosti</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D319" s="4" t="inlineStr">
@@ -7485,17 +7485,17 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>Talihov dvor, Pezinok, okres Pezinok</t>
+          <t>Čsl. parašutistov, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Marian Virgovič</t>
+          <t>Tomáš Tóth</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>Záhrada</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D320" s="4" t="inlineStr">
@@ -7507,17 +7507,17 @@
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>Račianska 64, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Holíčska 9, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t>Roman Miškulynets</t>
+          <t>Zuzana Pišteková</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D321" s="4" t="inlineStr">
@@ -7529,17 +7529,17 @@
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>Suchý vrch, Limbach, okres Pezinok</t>
+          <t>Talihov dvor, Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t>Miloslav Moravec</t>
+          <t>Marian Virgovič</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
         <is>
-          <t>Zrub / chalupa</t>
+          <t>Záhrada</t>
         </is>
       </c>
       <c r="D322" s="4" t="inlineStr">
@@ -7551,17 +7551,17 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>Ružová dolina 16, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Račianska 64, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t>Ľuboš Ľahký</t>
+          <t>Roman Miškulynets</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D323" s="4" t="inlineStr">
@@ -7573,17 +7573,17 @@
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>Na vrátkach, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Suchý vrch, Limbach, okres Pezinok</t>
         </is>
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t>Roland Samek</t>
+          <t>Miloslav Moravec</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Zrub / chalupa</t>
         </is>
       </c>
       <c r="D324" s="4" t="inlineStr">
@@ -7595,17 +7595,17 @@
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>Námestie 1. mája 3866, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Ružová dolina 16, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t>Oleksiy Namestie</t>
+          <t>Ľuboš Ľahký</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
         <is>
-          <t>Polyfunkčná budova</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D325" s="4" t="inlineStr">
@@ -7617,17 +7617,17 @@
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>Nejedlého 3394, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Na vrátkach, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t>Vladimír Žiga</t>
+          <t>Roland Samek</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D326" s="4" t="inlineStr">
@@ -7639,17 +7639,17 @@
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>Kristy Bendovej, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Námestie 1. mája 3866, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t>Jana Gottstein</t>
+          <t>Oleksiy Namestie</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Polyfunkčná budova</t>
         </is>
       </c>
       <c r="D327" s="4" t="inlineStr">
@@ -7661,17 +7661,17 @@
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>Sklenárova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Nejedlého 3394, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t>Dagmar Ivanová</t>
+          <t>Vladimír Žiga</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D328" s="4" t="inlineStr">
@@ -7683,17 +7683,17 @@
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>Pod vŕškom, Stupava, okres Malacky</t>
+          <t>Kristy Bendovej, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t>Lenka Višňovská</t>
+          <t>Jana Gottstein</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D329" s="4" t="inlineStr">
@@ -7705,17 +7705,17 @@
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>Galbavého 1, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Sklenárova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t>Denisa Lukačovičová</t>
+          <t>Dagmar Ivanová</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
         <is>
-          <t>Obchodné priestory</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D330" s="4" t="inlineStr">
@@ -7727,17 +7727,17 @@
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>Vážska, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Pod vŕškom, Stupava, okres Malacky</t>
         </is>
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t>Kristína Erazmusová</t>
+          <t>Lenka Višňovská</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D331" s="4" t="inlineStr">
@@ -7749,17 +7749,17 @@
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>Stromová 25, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Galbavého 1, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t>Michal Rusek</t>
+          <t>Denisa Lukačovičová</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Obchodné priestory</t>
         </is>
       </c>
       <c r="D332" s="4" t="inlineStr">
@@ -7771,17 +7771,17 @@
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>Chatová rekreačná oblasť, Rohožník, okres Malacky</t>
+          <t>Vážska, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t>M J</t>
+          <t>Kristína Erazmusová</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
         <is>
-          <t>Zrub / chalupa</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D333" s="4" t="inlineStr">
@@ -7793,17 +7793,17 @@
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>Hagarova, Bratislava-Rača, okres Bratislava III</t>
+          <t>Stromová 25, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t>Pavol Kusenda</t>
+          <t>Michal Rusek</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D334" s="4" t="inlineStr">
@@ -7815,17 +7815,17 @@
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Chatová rekreačná oblasť, Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t>L G</t>
+          <t>M J</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Zrub / chalupa</t>
         </is>
       </c>
       <c r="D335" s="4" t="inlineStr">
@@ -7837,17 +7837,17 @@
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>Malacky, okres Malacky</t>
+          <t>Hagarova, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t>Pán Budkovsky</t>
+          <t>Pavol Kusenda</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D336" s="4" t="inlineStr">
@@ -7859,17 +7859,17 @@
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>Námestie Hraničiarov, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t>predaj nehnutelnosti</t>
+          <t>L G</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D337" s="4" t="inlineStr">
@@ -7881,17 +7881,17 @@
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>Chotárna, Bratislava-Jarovce, okres Bratislava V</t>
+          <t>Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t>Tomáš Stolárik</t>
+          <t>Pán Budkovsky</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D338" s="4" t="inlineStr">
@@ -7903,17 +7903,17 @@
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>Vavrinecká, Limbach, okres Pezinok</t>
+          <t>Námestie Hraničiarov, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t>Peter Petrina</t>
+          <t>predaj nehnutelnosti</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D339" s="4" t="inlineStr">
@@ -7925,17 +7925,17 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>Komenského 2, Modra, okres Pezinok</t>
+          <t>Chotárna, Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Andrej B</t>
+          <t>Tomáš Stolárik</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D340" s="4" t="inlineStr">
@@ -7947,17 +7947,17 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>Bratislava-Jarovce, okres Bratislava V</t>
+          <t>Vavrinecká, Limbach, okres Pezinok</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Soňa Slobodníková</t>
+          <t>Peter Petrina</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D341" s="4" t="inlineStr">
@@ -7969,17 +7969,17 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>Na Revíne 19, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Komenského 2, Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Dušan Cintula</t>
+          <t>Andrej B</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D342" s="4" t="inlineStr">
@@ -7991,17 +7991,17 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>Hrušková 44H, Bratislava-Rača, okres Bratislava III</t>
+          <t>Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Jasna Rumanková</t>
+          <t>Soňa Slobodníková</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D343" s="4" t="inlineStr">
@@ -8013,17 +8013,17 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>Martina Granca, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Na Revíne 19, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Michal Michal</t>
+          <t>Dušan Cintula</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D344" s="4" t="inlineStr">
@@ -8035,17 +8035,17 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>Konventná 5, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Hrušková 44H, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Vladimir Taraba</t>
+          <t>Jasna Rumanková</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D345" s="4" t="inlineStr">
@@ -8057,17 +8057,17 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>Pezinok, okres Pezinok</t>
+          <t>Martina Granca, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Tomáš Machciník</t>
+          <t>Michal Michal</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D346" s="4" t="inlineStr">
@@ -8079,17 +8079,17 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>Malokarpatská 1, Svätý Jur, okres Pezinok</t>
+          <t>Konventná 5, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Jana Zárecká</t>
+          <t>Vladimir Taraba</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D347" s="4" t="inlineStr">
@@ -8101,17 +8101,17 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>Panónska cesta, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Oliver Práznovský</t>
+          <t>Tomáš Machciník</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D348" s="4" t="inlineStr">
@@ -8123,17 +8123,17 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>Mariánska cesta, Svätý Jur, okres Pezinok</t>
+          <t>Malokarpatská 1, Svätý Jur, okres Pezinok</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Marian Machalek</t>
+          <t>Jana Zárecká</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>Rekreačný pozemok</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D349" s="4" t="inlineStr">
@@ -8145,17 +8145,17 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>Homolova, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Panónska cesta, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Jaroslav Janco</t>
+          <t>Oliver Práznovský</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D350" s="4" t="inlineStr">
@@ -8167,17 +8167,17 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>Potočná, Bratislava-Rača, okres Bratislava III</t>
+          <t>Mariánska cesta, Svätý Jur, okres Pezinok</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Pavol Beblavy</t>
+          <t>Marian Machalek</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Rekreačný pozemok</t>
         </is>
       </c>
       <c r="D351" s="4" t="inlineStr">
@@ -8189,17 +8189,17 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>Pezinok, okres Pezinok</t>
+          <t>Homolova, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Peter Urban</t>
+          <t>Jaroslav Janco</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D352" s="4" t="inlineStr">
@@ -8211,17 +8211,17 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>Miletičova 60, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Potočná, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Michael Kollár</t>
+          <t>Pavol Beblavy</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D353" s="4" t="inlineStr">
@@ -8233,17 +8233,17 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>Svätovavrinecká, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Katarína Rusňáková</t>
+          <t>Peter Urban</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>5+ izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D354" s="4" t="inlineStr">
@@ -8255,27 +8255,71 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
+          <t>Miletičova 60, Bratislava-Ružinov, okres Bratislava II</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Michael Kollár</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>2-izbový byt</t>
+        </is>
+      </c>
+      <c r="D355" s="4" t="inlineStr">
+        <is>
+          <t>otvoriť ponuku</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>Svätovavrinecká, Bratislava-Nové Mesto, okres Bratislava III</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Katarína Rusňáková</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>5+ izbový byt</t>
+        </is>
+      </c>
+      <c r="D356" s="4" t="inlineStr">
+        <is>
+          <t>otvoriť ponuku</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
           <t>Hraničiarska, Vysoká pri Morave, okres Malacky</t>
         </is>
       </c>
-      <c r="B355" t="inlineStr">
+      <c r="B357" t="inlineStr">
         <is>
           <t>Andrea Bencová</t>
         </is>
       </c>
-      <c r="C355" t="inlineStr">
+      <c r="C357" t="inlineStr">
         <is>
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D355" s="4" t="inlineStr">
+      <c r="D357" s="4" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D355"/>
+  <autoFilter ref="A1:D357"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -8631,6 +8675,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D353" r:id="rId352"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D354" r:id="rId353"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D355" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D356" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D357" r:id="rId356"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8663,7 +8709,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>354</v>
+        <v>356</v>
       </c>
     </row>
     <row r="4">
@@ -8674,7 +8720,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>28.09.2026 11:59</t>
+          <t>28.09.2026 22:43</t>
         </is>
       </c>
     </row>
@@ -8704,7 +8750,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9">
@@ -8714,33 +8760,33 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>okres Bratislava V</t>
+          <t>okres Senec</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>okres Senec</t>
+          <t>okres Bratislava IV</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>okres Bratislava IV</t>
+          <t>okres Bratislava V</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -8754,7 +8800,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14">
@@ -8803,7 +8849,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="20">
@@ -8813,7 +8859,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="21">
@@ -8853,7 +8899,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
Aktualizácia ponúk – 2026-10-03 10:36 UTC
</commit_message>
<xml_diff>
--- a/public/ponuky.xlsx
+++ b/public/ponuky.xlsx
@@ -1015,22 +1015,22 @@
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Miletičova 35, Bratislava-Ružinov, okres Bratislava II</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Lubo Lajos</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Drobného, Bratislava-Dúbravka, okres Bratislava IV</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Gabriela Cermakova</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
         <is>
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="D26" s="4" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1039,12 +1039,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Ulica Svornosti, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Miletičova 35, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Marek Bacik</t>
+          <t>Lubo Lajos</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1061,17 +1061,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Jungmannova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Ulica Svornosti, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Vaso Bratislava</t>
+          <t>Marek Bacik</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -1083,17 +1083,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Brusnicová 13, Chorvátsky Grob, okres Senec</t>
+          <t>Jungmannova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Dušan Pokoš</t>
+          <t>Vaso Bratislava</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -1105,17 +1105,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Gavlovičova, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Brusnicová 13, Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Michal K</t>
+          <t>Dušan Pokoš</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -1127,17 +1127,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Vlčie hrdlo 85, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Gavlovičova, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Natalia Kubicova</t>
+          <t>Michal K</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -1149,12 +1149,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Hrachová 16C, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Vlčie hrdlo 85, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Dušan Pokoš</t>
+          <t>Natalia Kubicova</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1171,17 +1171,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Družstevná, Bernolákovo, okres Senec</t>
+          <t>Hrachová 16C, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Michaela Jancek</t>
+          <t>Dušan Pokoš</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -1193,12 +1193,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Planét, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Družstevná, Bernolákovo, okres Senec</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Július Július</t>
+          <t>Michaela Jancek</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1215,12 +1215,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Skalná, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Planét, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>katarina sekerka</t>
+          <t>Július Július</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1237,17 +1237,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Heyrovského, Bratislava-Lamač, okres Bratislava IV</t>
+          <t>Skalná, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Maros Palik</t>
+          <t>katarina sekerka</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -1259,17 +1259,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Oravská 2, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Heyrovského, Bratislava-Lamač, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Zdena Bartošová</t>
+          <t>Maros Palik</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -1281,17 +1281,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Jarabinková 2, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Oravská 2, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Michael Kollár</t>
+          <t>Zdena Bartošová</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -1303,7 +1303,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Miletičova 60, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Jarabinková 2, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -1325,12 +1325,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Bernolákova 2, Senec, okres Senec</t>
+          <t>Miletičova 60, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Šimon Klúčik</t>
+          <t>Michael Kollár</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1347,17 +1347,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Rovinka, okres Senec</t>
+          <t>Bernolákova 2, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Petra Sárkány</t>
+          <t>Šimon Klúčik</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -1369,17 +1369,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>J. Holčeka, Budmerice, okres Pezinok</t>
+          <t>Rovinka, okres Senec</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Ondrej Kolciter</t>
+          <t>Petra Sárkány</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -1413,17 +1413,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Chorvátsky Grob, okres Senec</t>
+          <t>J. Holčeka, Budmerice, okres Pezinok</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Dada Garajova</t>
+          <t>Ondrej Kolciter</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -1435,17 +1435,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Bajkalská 45C, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Eva Valáriková</t>
+          <t>Dada Garajova</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -1457,17 +1457,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Trebišovská, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bajkalská 45C, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Ružinov Štrkovec</t>
+          <t>Eva Valáriková</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -1479,17 +1479,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Rohožník, okres Malacky</t>
+          <t>Trebišovská, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Sukromna Osoba</t>
+          <t>Ružinov Štrkovec</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -1501,17 +1501,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Senec, okres Senec</t>
+          <t>Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Jakub Králik</t>
+          <t>Sukromna Osoba</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -1523,17 +1523,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Malacky, okres Malacky</t>
+          <t>Senec, okres Senec</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Elena Straznicka</t>
+          <t>Jakub Králik</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -1545,12 +1545,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Holubia, Senec, okres Senec</t>
+          <t>Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Marko Klúčik</t>
+          <t>Elena Straznicka</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1567,17 +1567,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>1mája, Pezinok, okres Pezinok</t>
+          <t>Holubia, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Ladislav Ružek</t>
+          <t>Marko Klúčik</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -1589,17 +1589,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>1mája, Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Lukas Durinak</t>
+          <t>Ladislav Ružek</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -1611,17 +1611,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Okružná 47, Senec, okres Senec</t>
+          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Roman Gazdik</t>
+          <t>Lukas Durinak</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -1633,12 +1633,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Slovenský Grob, okres Pezinok</t>
+          <t>Okružná 47, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Igor Šramka</t>
+          <t>Roman Gazdik</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2709,22 +2709,22 @@
       </c>
     </row>
     <row r="103">
-      <c r="A103" s="3" t="inlineStr">
+      <c r="A103" t="inlineStr">
         <is>
           <t>Saratovská 14, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
-      <c r="B103" s="3" t="inlineStr">
+      <c r="B103" t="inlineStr">
         <is>
           <t>Michal Podlucký</t>
         </is>
       </c>
-      <c r="C103" s="3" t="inlineStr">
+      <c r="C103" t="inlineStr">
         <is>
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D103" s="4" t="inlineStr">
+      <c r="D103" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3349,17 +3349,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Albrechtova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Geologická, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARZE MARZE </t>
+          <t>Elena Raucinova</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D132" s="2" t="inlineStr">
@@ -3371,12 +3371,12 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Geologická, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Ružová dolina, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Elena Raucinova</t>
+          <t>Michal Sadloň</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -3393,17 +3393,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Ružová dolina, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Okružná ulica, Tomášov, okres Senec</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Michal Sadloň</t>
+          <t>D P</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D134" s="2" t="inlineStr">
@@ -3415,17 +3415,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Okružná ulica, Tomášov, okres Senec</t>
+          <t>Rudroffova, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>D P</t>
+          <t>Ján Vlk</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D135" s="2" t="inlineStr">
@@ -3437,17 +3437,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Rudroffova, Bratislava-Rača, okres Bratislava III</t>
+          <t>Krížna 1, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Ján Vlk</t>
+          <t>Hadi Beheshti</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D136" s="2" t="inlineStr">
@@ -3459,17 +3459,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Krížna 1, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Dostojevského rad, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Hadi Beheshti</t>
+          <t>Lara Ondrejková</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D137" s="2" t="inlineStr">
@@ -3481,17 +3481,17 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Dostojevského rad, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bernolákovská, Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Lara Ondrejková</t>
+          <t>Oľga Šimáková</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D138" s="2" t="inlineStr">
@@ -3503,17 +3503,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Bernolákovská, Ivanka pri Dunaji, okres Senec</t>
+          <t>Miletičova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Oľga Šimáková</t>
+          <t>Lubo Stransky</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D139" s="2" t="inlineStr">
@@ -3525,17 +3525,17 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Miletičova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Segnerova, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Lubo Stransky</t>
+          <t>Samuel Kovalčík</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D140" s="2" t="inlineStr">
@@ -3547,17 +3547,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>Segnerova, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Jánošíkova, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Samuel Kovalčík</t>
+          <t>Viliam Pavelka</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D141" s="2" t="inlineStr">
@@ -3569,17 +3569,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Jánošíkova, Malacky, okres Malacky</t>
+          <t>Bartoškova, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Viliam Pavelka</t>
+          <t>Tibor S</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D142" s="2" t="inlineStr">
@@ -3591,17 +3591,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Bartoškova, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>D. Skuteckého 1650, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Tibor S</t>
+          <t>Mario Kral</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Double studio apartment</t>
         </is>
       </c>
       <c r="D143" s="2" t="inlineStr">
@@ -3613,17 +3613,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>D. Skuteckého 1650, Malacky, okres Malacky</t>
+          <t>Tajovského, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Mario Kral</t>
+          <t>Martin Gažo</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Double studio apartment</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D144" s="2" t="inlineStr">
@@ -3635,17 +3635,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Tajovského, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Kpt. Jána Rašu, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Martin Gažo</t>
+          <t>Monika Manova</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D145" s="2" t="inlineStr">
@@ -3657,17 +3657,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Kpt. Jána Rašu, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Monika Manova</t>
+          <t>Viliam Červenka</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D146" s="2" t="inlineStr">
@@ -3679,17 +3679,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Chorvátsky Grob, okres Senec</t>
+          <t>Budatínska 22, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Viliam Červenka</t>
+          <t>Martin Hraboš</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D147" s="2" t="inlineStr">
@@ -3701,12 +3701,12 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Budatínska 22, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Studenohorská, Bratislava-Lamač, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Martin Hraboš</t>
+          <t>Richard Remeník</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -3723,17 +3723,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Studenohorská, Bratislava-Lamač, okres Bratislava IV</t>
+          <t>Žltá 2A, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Richard Remeník</t>
+          <t>Peter Slánský</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D149" s="2" t="inlineStr">
@@ -3745,17 +3745,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Žltá 2A, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Banšelova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Peter Slánský</t>
+          <t>Miroslava Mihalikova</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D150" s="2" t="inlineStr">
@@ -3767,17 +3767,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Banšelova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Máchova 11, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Miroslava Mihalikova</t>
+          <t>Marian Varga</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D151" s="2" t="inlineStr">
@@ -3789,12 +3789,12 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Máchova 11, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Bratislava-Rusovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Marian Varga</t>
+          <t>Milan Dzilsky</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -3811,17 +3811,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Bratislava-Rusovce, okres Bratislava V</t>
+          <t>Rozvodná, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Milan Dzilsky</t>
+          <t>Daniela Súkromná osoba</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D153" s="2" t="inlineStr">
@@ -3833,17 +3833,17 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Rozvodná, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Daniela Súkromná osoba</t>
+          <t>Michal POLÁČEK</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D154" s="2" t="inlineStr">
@@ -3855,17 +3855,17 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
+          <t>Športová, Limbach, okres Pezinok</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Michal POLÁČEK</t>
+          <t>Michal Mravec</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D155" s="2" t="inlineStr">
@@ -3877,17 +3877,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Športová, Limbach, okres Pezinok</t>
+          <t>Železničiarska, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Michal Mravec</t>
+          <t>Dávid Uličný</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D156" s="2" t="inlineStr">
@@ -3899,17 +3899,17 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Železničiarska, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Balkánska 67, Bratislava-Rusovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Dávid Uličný</t>
+          <t>Peter Kalas</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D157" s="2" t="inlineStr">
@@ -3921,12 +3921,12 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Balkánska 67, Bratislava-Rusovce, okres Bratislava V</t>
+          <t>Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Peter Kalas</t>
+          <t>pán Budkovský</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -3943,17 +3943,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Malacky, okres Malacky</t>
+          <t>Horská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>pán Budkovský</t>
+          <t>Michaela Weberova</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Mezonet</t>
         </is>
       </c>
       <c r="D159" s="2" t="inlineStr">
@@ -3975,7 +3975,7 @@
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Mezonet</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D160" s="2" t="inlineStr">
@@ -3987,17 +3987,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Horská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Tallerova 4, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Michaela Weberova</t>
+          <t>Daniela Ondriašová</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D161" s="2" t="inlineStr">
@@ -4009,17 +4009,17 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Tallerova 4, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bernolákova ulica, Miloslavov, okres Senec</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Daniela Ondriašová</t>
+          <t>Erik Mihok</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D162" s="2" t="inlineStr">
@@ -4031,17 +4031,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Bernolákova ulica, Miloslavov, okres Senec</t>
+          <t>Východná, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Erik Mihok</t>
+          <t>Marek Vodička</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D163" s="2" t="inlineStr">
@@ -4053,17 +4053,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Východná, Bratislava-Rača, okres Bratislava III</t>
+          <t>Bratislava-Rusovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Marek Vodička</t>
+          <t>Alexandra Belašičová</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D164" s="2" t="inlineStr">
@@ -4075,17 +4075,17 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Bratislava-Rusovce, okres Bratislava V</t>
+          <t>L. Novomeského, Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Alexandra Belašičová</t>
+          <t>Stefan PASTVA</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D165" s="2" t="inlineStr">
@@ -4097,17 +4097,17 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>L. Novomeského, Pezinok, okres Pezinok</t>
+          <t>Pri Pálenici, Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Stefan PASTVA</t>
+          <t>Dominika Ševčíková</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D166" s="2" t="inlineStr">
@@ -4119,17 +4119,17 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Pri Pálenici, Ivanka pri Dunaji, okres Senec</t>
+          <t>Vyšehradská, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Dominika Ševčíková</t>
+          <t>Anna Zábrelová</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D167" s="2" t="inlineStr">
@@ -4141,17 +4141,17 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Vyšehradská, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Vígľašská, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Anna Zábrelová</t>
+          <t>Kristína Gatyášová</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D168" s="2" t="inlineStr">
@@ -4163,17 +4163,17 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Vígľašská, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Zidiny, Bratislava-Lamač, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Kristína Gatyášová</t>
+          <t>Vratislav Jurica</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D169" s="2" t="inlineStr">
@@ -4185,12 +4185,12 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Zidiny, Bratislava-Lamač, okres Bratislava IV</t>
+          <t>Opálová ulica, Miloslavov, okres Senec</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Vratislav Jurica</t>
+          <t>Michal Farsky</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -4207,17 +4207,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Opálová ulica, Miloslavov, okres Senec</t>
+          <t>Hrachová 73, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Michal Farsky</t>
+          <t>Patrik Písečný</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D171" s="2" t="inlineStr">
@@ -4229,12 +4229,12 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Hrachová 73, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Rovniankova 4, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Patrik Písečný</t>
+          <t>Ján Čeman</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -4251,17 +4251,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Rovniankova 4, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Čsl. tankistov, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Ján Čeman</t>
+          <t>Viliam Kulacs</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D173" s="2" t="inlineStr">
@@ -4273,17 +4273,17 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Čsl. tankistov, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
+          <t>Palárikova 3, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Viliam Kulacs</t>
+          <t>Michal Michal</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D174" s="2" t="inlineStr">
@@ -4295,17 +4295,17 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Palárikova 3, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Záhradnícka, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Michal Michal</t>
+          <t>Marta Onova</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D175" s="2" t="inlineStr">
@@ -4317,17 +4317,17 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Záhradnícka, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Janka Kráľa, Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Marta Onova</t>
+          <t>Ivana Poláková</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D176" s="2" t="inlineStr">
@@ -4339,17 +4339,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Janka Kráľa, Chorvátsky Grob, okres Senec</t>
+          <t>Hronská 10, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Ivana Poláková</t>
+          <t>Radoslav Cifra</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D177" s="2" t="inlineStr">
@@ -4361,12 +4361,12 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Hronská 10, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Rezedová, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Radoslav Cifra</t>
+          <t>Andrea SJ</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -4383,17 +4383,17 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Rezedová, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Andrea SJ</t>
+          <t>Peter Fusek</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D179" s="2" t="inlineStr">
@@ -4405,17 +4405,17 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Potočná 9, Limbach, okres Pezinok</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Peter Fusek</t>
+          <t>Miroslav Gavalec</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D180" s="2" t="inlineStr">
@@ -4427,17 +4427,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Potočná 9, Limbach, okres Pezinok</t>
+          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Miroslav Gavalec</t>
+          <t>Daniela Ondriašová</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D181" s="2" t="inlineStr">
@@ -4449,17 +4449,17 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Drotárska cesta, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Daniela Ondriašová</t>
+          <t>Petra Hager</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D182" s="2" t="inlineStr">
@@ -4471,17 +4471,17 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Drotárska cesta, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Petra Hager</t>
+          <t>Peter Pezinok</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D183" s="2" t="inlineStr">
@@ -4493,17 +4493,17 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Pezinok, okres Pezinok</t>
+          <t>Zuzany Chalupovej 10B, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Peter Pezinok</t>
+          <t>Pavol Trembuľak</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D184" s="2" t="inlineStr">
@@ -4515,17 +4515,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej 10B, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Karadžičova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Pavol Trembuľak</t>
+          <t>Tatiana B</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D185" s="2" t="inlineStr">
@@ -4537,17 +4537,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Karadžičova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Tatiana B</t>
+          <t>Peter Kollar</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Reštauračné priestory</t>
         </is>
       </c>
       <c r="D186" s="2" t="inlineStr">
@@ -4559,17 +4559,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Nejedlého 20, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Peter Kollar</t>
+          <t>Marian Placko</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Reštauračné priestory</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D187" s="2" t="inlineStr">
@@ -4581,17 +4581,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Nejedlého 20, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Jána L. Bellu, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Marian Placko</t>
+          <t>Michal Sadloň</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D188" s="2" t="inlineStr">
@@ -4603,17 +4603,17 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Jána L. Bellu, Senec, okres Senec</t>
+          <t>Pri kríži, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Michal Sadloň</t>
+          <t>Denisa Brozmannova</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D189" s="2" t="inlineStr">
@@ -4625,17 +4625,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Pri kríži, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Mesačná 9, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Denisa Brozmannova</t>
+          <t>Eva Valáriková</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D190" s="2" t="inlineStr">
@@ -4647,17 +4647,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Mesačná 9, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Sedmokrásková 3, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Eva Valáriková</t>
+          <t>Lekáreň Sedmokráska</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Obchodné priestory</t>
         </is>
       </c>
       <c r="D191" s="2" t="inlineStr">
@@ -4669,17 +4669,17 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Sedmokrásková 3, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Triblavinská, Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Lekáreň Sedmokráska</t>
+          <t>Robert Manak</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>Obchodné priestory</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D192" s="2" t="inlineStr">
@@ -4691,17 +4691,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>Triblavinská, Chorvátsky Grob, okres Senec</t>
+          <t>Antolská, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Robert Manak</t>
+          <t>Peter Petovsky</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D193" s="2" t="inlineStr">
@@ -4713,17 +4713,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Antolská, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Svätý Jur, okres Pezinok</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Peter Petovsky</t>
+          <t>Martin Kratochvíl</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Záhrada</t>
         </is>
       </c>
       <c r="D194" s="2" t="inlineStr">
@@ -4735,17 +4735,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Svätý Jur, okres Pezinok</t>
+          <t>Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Martin Kratochvíl</t>
+          <t>Vaše Bývanie</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Záhrada</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D195" s="2" t="inlineStr">
@@ -4757,17 +4757,17 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
+          <t>Ševčenkova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Vaše Bývanie</t>
+          <t>Pavol Zlacký</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D196" s="2" t="inlineStr">
@@ -4779,12 +4779,12 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Ševčenkova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Mlynské nivy, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Pavol Zlacký</t>
+          <t>Viktória Rybáriková</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -4801,17 +4801,17 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Mlynské nivy, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bieloruská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Viktória Rybáriková</t>
+          <t>Veronika L</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D198" s="2" t="inlineStr">
@@ -4823,17 +4823,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Bieloruská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Mickiewiczova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Veronika L</t>
+          <t>Lubica Šuleková</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Iný priestor</t>
         </is>
       </c>
       <c r="D199" s="2" t="inlineStr">
@@ -4845,17 +4845,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Mickiewiczova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Závod, okres Malacky</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Lubica Šuleková</t>
+          <t>Peter Peter</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>Iný priestor</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D200" s="2" t="inlineStr">
@@ -4867,17 +4867,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Závod, okres Malacky</t>
+          <t>Zuzany Chalupovej 11A, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Peter Peter</t>
+          <t>David slnecnice</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D201" s="2" t="inlineStr">
@@ -4889,17 +4889,17 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej 11A, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Devínska cesta, Bratislava-Devín, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>David slnecnice</t>
+          <t>Július Július</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Záhradná chatka</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
@@ -4911,17 +4911,17 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Devínska cesta, Bratislava-Devín, okres Bratislava IV</t>
+          <t>Tureň, okres Senec</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Július Július</t>
+          <t>Maroš Szighardt</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>Záhradná chatka</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D203" s="2" t="inlineStr">
@@ -4933,12 +4933,12 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Tureň, okres Senec</t>
+          <t>Hamuliakovo, okres Senec</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Maroš Szighardt</t>
+          <t>Peter Košút</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -4955,17 +4955,17 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Hamuliakovo, okres Senec</t>
+          <t>Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Peter Košút</t>
+          <t>Jan L</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D205" s="2" t="inlineStr">
@@ -4977,17 +4977,17 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
+          <t>Eduarda Wenzla, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Jan L</t>
+          <t xml:space="preserve">Miroslav O  </t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D206" s="2" t="inlineStr">
@@ -4999,12 +4999,12 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Eduarda Wenzla, Bratislava-Rača, okres Bratislava III</t>
+          <t>Bajkalská 9B, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t xml:space="preserve">Miroslav O  </t>
+          <t>gianluca de vecchi</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -5021,17 +5021,17 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Bajkalská 9B, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Dulovo námestie, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>gianluca de vecchi</t>
+          <t>Martin Griga</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D208" s="2" t="inlineStr">
@@ -5043,17 +5043,17 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Dulovo námestie, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Cyprichova, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Martin Griga</t>
+          <t>Anton K</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D209" s="2" t="inlineStr">
@@ -5065,17 +5065,17 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Cyprichova, Bratislava-Rača, okres Bratislava III</t>
+          <t>Dvojkrížna, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Anton K</t>
+          <t>Ladislav Sipos</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D210" s="2" t="inlineStr">
@@ -5087,17 +5087,17 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Dvojkrížna, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Na varte, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Ladislav Sipos</t>
+          <t>Alexander Milly</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D211" s="2" t="inlineStr">
@@ -5109,17 +5109,17 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Na varte, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Malé Leváre, okres Malacky</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Alexander Milly</t>
+          <t>Victoria Ivanová</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D212" s="2" t="inlineStr">
@@ -5131,17 +5131,17 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Malé Leváre, okres Malacky</t>
+          <t>Nejedlého 20, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Victoria Ivanová</t>
+          <t>Mojmír Gaško</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D213" s="2" t="inlineStr">
@@ -5153,17 +5153,17 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Nejedlého 20, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Veltlínska, Svätý Jur, okres Pezinok</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Mojmír Gaško</t>
+          <t>Jaroslav Š</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D214" s="2" t="inlineStr">
@@ -5175,17 +5175,17 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Veltlínska, Svätý Jur, okres Pezinok</t>
+          <t>Riazanská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Jaroslav Š</t>
+          <t>Ivan Beňo</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D215" s="2" t="inlineStr">
@@ -5197,17 +5197,17 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Riazanská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Višňová, Bernolákovo, okres Senec</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Ivan Beňo</t>
+          <t>Juraj Várady</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D216" s="2" t="inlineStr">
@@ -5219,12 +5219,12 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>Višňová, Bernolákovo, okres Senec</t>
+          <t>Dunajská Lužná, okres Senec</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Juraj Várady</t>
+          <t>Kristína Gatyášová</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -5241,12 +5241,12 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Dunajská Lužná, okres Senec</t>
+          <t>Karasová 68, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Kristína Gatyášová</t>
+          <t>Juraj Várady</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -5263,12 +5263,12 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Karasová 68, Senec, okres Senec</t>
+          <t>Oblačná 7155, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Juraj Várady</t>
+          <t>Roman R</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -5285,17 +5285,17 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>Oblačná 7155, Bratislava-Rača, okres Bratislava III</t>
+          <t>Novohorská, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Roman R</t>
+          <t>Martin Klaučo</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D220" s="2" t="inlineStr">
@@ -5307,17 +5307,17 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>Novohorská, Bratislava-Rača, okres Bratislava III</t>
+          <t>Zuzany Chalupovej 3981, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Martin Klaučo</t>
+          <t>Karol Jurčik</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D221" s="2" t="inlineStr">
@@ -5329,17 +5329,17 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej 3981, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Rusovská cesta, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>Karol Jurčik</t>
+          <t>Mgr Jarmila Somolányiová</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D222" s="2" t="inlineStr">
@@ -5351,12 +5351,12 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>Rusovská cesta, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Nobelova, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Mgr Jarmila Somolányiová</t>
+          <t>Ondrej R</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -5373,17 +5373,17 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>Nobelova, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Kukučínova, Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Ondrej R</t>
+          <t>Jaro Hanzel</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D224" s="2" t="inlineStr">
@@ -5395,17 +5395,17 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Kukučínova, Ivanka pri Dunaji, okres Senec</t>
+          <t>Železničná ulica, Miloslavov, okres Senec</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Jaro Hanzel</t>
+          <t>Jan Holko</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D225" s="2" t="inlineStr">
@@ -5417,17 +5417,17 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>Železničná ulica, Miloslavov, okres Senec</t>
+          <t>Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>Jan Holko</t>
+          <t>jana Lieskovska</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D226" s="2" t="inlineStr">
@@ -5439,17 +5439,17 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Pri vinohradoch 6179, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>jana Lieskovska</t>
+          <t>Tibor Tokár</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D227" s="2" t="inlineStr">
@@ -5461,17 +5461,17 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>Pri vinohradoch 6179, Bratislava-Rača, okres Bratislava III</t>
+          <t>Bratislava-Rusovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Tibor Tokár</t>
+          <t>petra svetik</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D228" s="2" t="inlineStr">
@@ -5483,17 +5483,17 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Bratislava-Rusovce, okres Bratislava V</t>
+          <t>Mikulášska 1B, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>petra svetik</t>
+          <t>Martin Mančík</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D229" s="2" t="inlineStr">
@@ -5505,17 +5505,17 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>Mikulášska 1B, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bélu Bartóka 9, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Martin Mančík</t>
+          <t>Igor Gottgeisl</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D230" s="2" t="inlineStr">
@@ -5527,17 +5527,17 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>Bélu Bartóka 9, Senec, okres Senec</t>
+          <t>Bernolákovo, okres Senec</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Igor Gottgeisl</t>
+          <t>Lucia Tacovska</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Záhrada</t>
         </is>
       </c>
       <c r="D231" s="2" t="inlineStr">
@@ -5549,17 +5549,17 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Bernolákovo, okres Senec</t>
+          <t>Bezručova 5, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Lucia Tacovska</t>
+          <t>Peter Moravcik</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Záhrada</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D232" s="2" t="inlineStr">
@@ -5571,17 +5571,17 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Bezručova 5, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Čsl. tankistov, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Peter Moravcik</t>
+          <t>Ing Štefan Paľov</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D233" s="2" t="inlineStr">
@@ -5593,17 +5593,17 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>Čsl. tankistov, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
+          <t>Na pasekách, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Ing Štefan Paľov</t>
+          <t>Jaroslav Babik</t>
         </is>
       </c>
       <c r="C234" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D234" s="2" t="inlineStr">
@@ -5615,17 +5615,17 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>Na pasekách, Bratislava-Rača, okres Bratislava III</t>
+          <t>Západný rad, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Jaroslav Babik</t>
+          <t>Iveta Kopecká</t>
         </is>
       </c>
       <c r="C235" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D235" s="2" t="inlineStr">
@@ -5637,17 +5637,17 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>Západný rad, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Lachova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Iveta Kopecká</t>
+          <t>Veronika Mich</t>
         </is>
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D236" s="2" t="inlineStr">
@@ -5659,17 +5659,17 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>Lachova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Dlhá 8/D, Stupava, okres Malacky</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Veronika Mich</t>
+          <t>Jaroslav Timko</t>
         </is>
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D237" s="2" t="inlineStr">
@@ -5681,17 +5681,17 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>Dlhá 8/D, Stupava, okres Malacky</t>
+          <t>Ožvoldíkova, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Jaroslav Timko</t>
+          <t>Marek Riesz</t>
         </is>
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D238" s="2" t="inlineStr">
@@ -5703,17 +5703,17 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>Ožvoldíkova, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Miloslavov, okres Senec</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Marek Riesz</t>
+          <t>Roman Pavelka</t>
         </is>
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D239" s="2" t="inlineStr">
@@ -5725,12 +5725,12 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>Miloslavov, okres Senec</t>
+          <t>Jablonec, okres Pezinok</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Roman Pavelka</t>
+          <t>Martin Chudoba</t>
         </is>
       </c>
       <c r="C240" t="inlineStr">
@@ -5747,12 +5747,12 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>Jablonec, okres Pezinok</t>
+          <t>Borská, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Martin Chudoba</t>
+          <t>Jan Kuna</t>
         </is>
       </c>
       <c r="C241" t="inlineStr">
@@ -5769,17 +5769,17 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>Borská, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Vilová, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Jan Kuna</t>
+          <t xml:space="preserve">Terézia Laurincová </t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D242" s="2" t="inlineStr">
@@ -5791,17 +5791,17 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>Vilová, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Ožvoldíkova, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t xml:space="preserve">Terézia Laurincová </t>
+          <t>Samuel Kovalčík</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D243" s="2" t="inlineStr">
@@ -5813,17 +5813,17 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>Ožvoldíkova, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Žabí majer, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Samuel Kovalčík</t>
+          <t>Marcel Buttko</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Mobilný dom</t>
         </is>
       </c>
       <c r="D244" s="2" t="inlineStr">
@@ -5835,17 +5835,17 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>Žabí majer, Bratislava-Rača, okres Bratislava III</t>
+          <t>Ulica Sauberg, Svätý Jur, okres Pezinok</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Marcel Buttko</t>
+          <t>Boris Haviar</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Mobilný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D245" s="2" t="inlineStr">
@@ -5857,17 +5857,17 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>Ulica Sauberg, Svätý Jur, okres Pezinok</t>
+          <t>Frankovská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Boris Haviar</t>
+          <t>Michal Klempai</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D246" s="2" t="inlineStr">
@@ -5879,17 +5879,17 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>Frankovská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Žilinská 1, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Michal Klempai</t>
+          <t>Mat Nav</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Obchodné priestory</t>
         </is>
       </c>
       <c r="D247" s="2" t="inlineStr">
@@ -5901,17 +5901,17 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>Žilinská 1, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Mat Nav</t>
+          <t>Zuzana Farbulová</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Obchodné priestory</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D248" s="2" t="inlineStr">
@@ -5923,17 +5923,17 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>Pezinok, okres Pezinok</t>
+          <t>Kuklovská, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Zuzana Farbulová</t>
+          <t>Ra Fa</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D249" s="2" t="inlineStr">
@@ -5945,17 +5945,17 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>Kuklovská, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Podhradie 68, Svätý Jur, okres Pezinok</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Ra Fa</t>
+          <t>Dávid Boháč</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D250" s="2" t="inlineStr">
@@ -5967,17 +5967,17 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>Podhradie 68, Svätý Jur, okres Pezinok</t>
+          <t>Schengenská, Bratislava-Čunovo, okres Bratislava V</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Dávid Boháč</t>
+          <t>Ľudovít Braniš</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Rekreačný pozemok</t>
         </is>
       </c>
       <c r="D251" s="2" t="inlineStr">
@@ -5989,17 +5989,17 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>Schengenská, Bratislava-Čunovo, okres Bratislava V</t>
+          <t>Železničná 43, Bernolákovo, okres Senec</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Ľudovít Braniš</t>
+          <t>Tomáš Tenczer</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Rekreačný pozemok</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D252" s="2" t="inlineStr">
@@ -6011,17 +6011,17 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>Železničná 43, Bernolákovo, okres Senec</t>
+          <t>Antolská 6, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Tomáš Tenczer</t>
+          <t>Rudolf Lachkovic</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D253" s="2" t="inlineStr">
@@ -6033,17 +6033,17 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>Antolská 6, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Lovinského 35, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Rudolf Lachkovic</t>
+          <t xml:space="preserve">Pavol Kupec </t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Administratívna budova</t>
         </is>
       </c>
       <c r="D254" s="2" t="inlineStr">
@@ -6055,17 +6055,17 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>Lovinského 35, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pavol Kupec </t>
+          <t>Peter J</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Administratívna budova</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D255" s="2" t="inlineStr">
@@ -6077,17 +6077,17 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>Malacky, okres Malacky</t>
+          <t>Černyševského 12, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Peter J</t>
+          <t>Vladimir Jagr</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D256" s="2" t="inlineStr">
@@ -6099,17 +6099,17 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>Černyševského 12, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Fedinova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Vladimir Jagr</t>
+          <t>Tomáš  Vizina</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D257" s="2" t="inlineStr">
@@ -6121,17 +6121,17 @@
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>Fedinova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Hlavná 244, Záhorská Ves, okres Malacky</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Tomáš  Vizina</t>
+          <t>Alexander Horvath</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D258" s="2" t="inlineStr">
@@ -6143,17 +6143,17 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>Hlavná 244, Záhorská Ves, okres Malacky</t>
+          <t>Ulica 29. augusta 23, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Alexander Horvath</t>
+          <t>Anna Privrelová</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D259" s="2" t="inlineStr">
@@ -6165,17 +6165,17 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>Ulica 29. augusta 23, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Záhradná 51, Limbach, okres Pezinok</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Anna Privrelová</t>
+          <t>Taras Baca</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D260" s="2" t="inlineStr">
@@ -6187,17 +6187,17 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>Záhradná 51, Limbach, okres Pezinok</t>
+          <t>Jána Jonáša, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Taras Baca</t>
+          <t>Katarína Kachmanová</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D261" s="2" t="inlineStr">
@@ -6209,17 +6209,17 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>Jána Jonáša, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
+          <t>Pri vinohradoch 142, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Katarína Kachmanová</t>
+          <t>Ľuboš Čmelko</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D262" s="2" t="inlineStr">
@@ -6231,17 +6231,17 @@
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>Pri vinohradoch 142, Bratislava-Rača, okres Bratislava III</t>
+          <t>Ulica Svornosti, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Ľuboš Čmelko</t>
+          <t>Matuš  Žemlička</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Zmiešaná zóna</t>
         </is>
       </c>
       <c r="D263" s="2" t="inlineStr">
@@ -6253,17 +6253,17 @@
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>Ulica Svornosti, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Košická 10, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Matuš  Žemlička</t>
+          <t>David A</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Zmiešaná zóna</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D264" s="2" t="inlineStr">
@@ -6275,17 +6275,17 @@
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>Košická 10, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Zlatý Karas, Nová Dedinka, okres Senec</t>
         </is>
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>David A</t>
+          <t>Vincent Durbak</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D265" s="2" t="inlineStr">
@@ -6297,17 +6297,17 @@
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>Zlatý Karas, Nová Dedinka, okres Senec</t>
+          <t>Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Vincent Durbak</t>
+          <t>Edmund Edmund</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D266" s="2" t="inlineStr">
@@ -6319,17 +6319,17 @@
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Plavecký Štvrtok, okres Malacky</t>
         </is>
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Edmund Edmund</t>
+          <t>Sisi Belo</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D267" s="2" t="inlineStr">
@@ -6341,17 +6341,17 @@
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>Jedľová ulica, Zohor, okres Malacky</t>
+          <t>Baltská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B268" t="inlineStr">
         <is>
-          <t>Andrea Bencová</t>
+          <t>L M</t>
         </is>
       </c>
       <c r="C268" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D268" s="2" t="inlineStr">
@@ -6363,17 +6363,17 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>Plavecký Štvrtok, okres Malacky</t>
+          <t>Trnavská cesta, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B269" t="inlineStr">
         <is>
-          <t>Sisi Belo</t>
+          <t>LEX vision</t>
         </is>
       </c>
       <c r="C269" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D269" s="2" t="inlineStr">
@@ -6385,17 +6385,17 @@
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>Baltská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Male Pole 111, Vištuk, okres Pezinok</t>
         </is>
       </c>
       <c r="B270" t="inlineStr">
         <is>
-          <t>L M</t>
+          <t>Frantisek Krasnansky</t>
         </is>
       </c>
       <c r="C270" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D270" s="2" t="inlineStr">
@@ -6407,17 +6407,17 @@
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>Trnavská cesta, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Uránová, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B271" t="inlineStr">
         <is>
-          <t>LEX vision</t>
+          <t>Erik Varchol</t>
         </is>
       </c>
       <c r="C271" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D271" s="2" t="inlineStr">
@@ -6429,17 +6429,17 @@
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>Male Pole 111, Vištuk, okres Pezinok</t>
+          <t>Hlavná 10E, Nová Dedinka, okres Senec</t>
         </is>
       </c>
       <c r="B272" t="inlineStr">
         <is>
-          <t>Frantisek Krasnansky</t>
+          <t>Miroslava Magulova</t>
         </is>
       </c>
       <c r="C272" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D272" s="2" t="inlineStr">
@@ -6451,17 +6451,17 @@
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>Uránová, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Veľké Leváre, okres Malacky</t>
         </is>
       </c>
       <c r="B273" t="inlineStr">
         <is>
-          <t>Erik Varchol</t>
+          <t>Denis  Klempa</t>
         </is>
       </c>
       <c r="C273" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D273" s="2" t="inlineStr">
@@ -6473,17 +6473,17 @@
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>Hlavná 10E, Nová Dedinka, okres Senec</t>
+          <t>Plavecký Štvrtok, okres Malacky</t>
         </is>
       </c>
       <c r="B274" t="inlineStr">
         <is>
-          <t>Miroslava Magulova</t>
+          <t>Peter J</t>
         </is>
       </c>
       <c r="C274" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D274" s="2" t="inlineStr">
@@ -6495,17 +6495,17 @@
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>Veľké Leváre, okres Malacky</t>
+          <t>Cementárenská, Stupava, okres Malacky</t>
         </is>
       </c>
       <c r="B275" t="inlineStr">
         <is>
-          <t>Denis  Klempa</t>
+          <t>Peter Haco</t>
         </is>
       </c>
       <c r="C275" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Polyfunkčná budova</t>
         </is>
       </c>
       <c r="D275" s="2" t="inlineStr">
@@ -6517,12 +6517,12 @@
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>Plavecký Štvrtok, okres Malacky</t>
+          <t>Sama Chalúpku, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B276" t="inlineStr">
         <is>
-          <t>Peter J</t>
+          <t>Boris Cambalik</t>
         </is>
       </c>
       <c r="C276" t="inlineStr">
@@ -6539,17 +6539,17 @@
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>Cementárenská, Stupava, okres Malacky</t>
+          <t>Bieloruská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B277" t="inlineStr">
         <is>
-          <t>Peter Haco</t>
+          <t>Richard Macko</t>
         </is>
       </c>
       <c r="C277" t="inlineStr">
         <is>
-          <t>Polyfunkčná budova</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D277" s="2" t="inlineStr">
@@ -6561,17 +6561,17 @@
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>Sama Chalúpku, Malacky, okres Malacky</t>
+          <t>Cyprichova 2, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B278" t="inlineStr">
         <is>
-          <t>Boris Cambalik</t>
+          <t>Anna Boríková</t>
         </is>
       </c>
       <c r="C278" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Reštauračné priestory</t>
         </is>
       </c>
       <c r="D278" s="2" t="inlineStr">
@@ -6583,17 +6583,17 @@
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>Bieloruská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>Richard Macko</t>
+          <t>Lucia Danišová</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D279" s="2" t="inlineStr">
@@ -6605,17 +6605,17 @@
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>Cyprichova 2, Bratislava-Rača, okres Bratislava III</t>
+          <t>Karloveské rameno, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>Anna Boríková</t>
+          <t>Pavol Bak</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
         <is>
-          <t>Reštauračné priestory</t>
+          <t>Pozemok pre bytovú výstavbu</t>
         </is>
       </c>
       <c r="D280" s="2" t="inlineStr">
@@ -6627,17 +6627,17 @@
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Karloveské rameno, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>Lucia Danišová</t>
+          <t>Pavol Bak</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Bytový dom</t>
         </is>
       </c>
       <c r="D281" s="2" t="inlineStr">
@@ -6649,17 +6649,17 @@
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>Karloveské rameno, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Kľak, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>Pavol Bak</t>
+          <t>Miroslav  Pinka</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
         <is>
-          <t>Pozemok pre bytovú výstavbu</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D282" s="2" t="inlineStr">
@@ -6671,17 +6671,17 @@
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>Karloveské rameno, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B283" t="inlineStr">
         <is>
-          <t>Pavol Bak</t>
+          <t>Nova Rekonštrukcia</t>
         </is>
       </c>
       <c r="C283" t="inlineStr">
         <is>
-          <t>Bytový dom</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D283" s="2" t="inlineStr">
@@ -6693,17 +6693,17 @@
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Studená, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B284" t="inlineStr">
         <is>
-          <t>Nova Rekonštrukcia</t>
+          <t>Byt Studena</t>
         </is>
       </c>
       <c r="C284" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D284" s="2" t="inlineStr">
@@ -6715,17 +6715,17 @@
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>Studená, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Krížna 1, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B285" t="inlineStr">
         <is>
-          <t>Byt Studena</t>
+          <t>martina busova</t>
         </is>
       </c>
       <c r="C285" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D285" s="2" t="inlineStr">
@@ -6737,12 +6737,12 @@
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>Krížna 1, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Fedákova, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B286" t="inlineStr">
         <is>
-          <t>martina busova</t>
+          <t>Magdaléna Helísek</t>
         </is>
       </c>
       <c r="C286" t="inlineStr">
@@ -6759,17 +6759,17 @@
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>Fedákova, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Hany Meličkovej, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B287" t="inlineStr">
         <is>
-          <t>Magdaléna Helísek</t>
+          <t>Viera Peterkova</t>
         </is>
       </c>
       <c r="C287" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D287" s="2" t="inlineStr">
@@ -6781,17 +6781,17 @@
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>Hany Meličkovej, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Bratislava-Lamač, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B288" t="inlineStr">
         <is>
-          <t>Viera Peterkova</t>
+          <t>E S</t>
         </is>
       </c>
       <c r="C288" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D288" s="2" t="inlineStr">
@@ -6803,17 +6803,17 @@
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>Bratislava-Lamač, okres Bratislava IV</t>
+          <t>Topoľčianska 12, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B289" t="inlineStr">
         <is>
-          <t>E S</t>
+          <t>Gabriel Mészáros</t>
         </is>
       </c>
       <c r="C289" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Double studio apartment</t>
         </is>
       </c>
       <c r="D289" s="2" t="inlineStr">
@@ -6825,17 +6825,17 @@
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>Topoľčianska 12, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Hamuliakovo, okres Senec</t>
         </is>
       </c>
       <c r="B290" t="inlineStr">
         <is>
-          <t>Gabriel Mészáros</t>
+          <t>Sebastian Bognár</t>
         </is>
       </c>
       <c r="C290" t="inlineStr">
         <is>
-          <t>Double studio apartment</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D290" s="2" t="inlineStr">
@@ -6847,12 +6847,12 @@
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>Hamuliakovo, okres Senec</t>
+          <t>Senec, okres Senec</t>
         </is>
       </c>
       <c r="B291" t="inlineStr">
         <is>
-          <t>Sebastian Bognár</t>
+          <t>Jana Muhlova</t>
         </is>
       </c>
       <c r="C291" t="inlineStr">
@@ -6869,17 +6869,17 @@
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>Senec, okres Senec</t>
+          <t>Košická, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B292" t="inlineStr">
         <is>
-          <t>Jana Muhlova</t>
+          <t>Timea Henry</t>
         </is>
       </c>
       <c r="C292" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D292" s="2" t="inlineStr">
@@ -6901,7 +6901,7 @@
       </c>
       <c r="C293" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D293" s="2" t="inlineStr">
@@ -6913,17 +6913,17 @@
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>Košická, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Jantárová, Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B294" t="inlineStr">
         <is>
-          <t>Timea Henry</t>
+          <t>Monika Szocsova</t>
         </is>
       </c>
       <c r="C294" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D294" s="2" t="inlineStr">
@@ -6935,17 +6935,17 @@
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>Jantárová, Bratislava-Jarovce, okres Bratislava V</t>
+          <t>Západný rad, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B295" t="inlineStr">
         <is>
-          <t>Monika Szocsova</t>
+          <t>Iveta Kopecká</t>
         </is>
       </c>
       <c r="C295" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D295" s="2" t="inlineStr">
@@ -6957,7 +6957,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Západný rad, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Gaštanová 9, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -6967,7 +6967,7 @@
       </c>
       <c r="C296" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D296" s="2" t="inlineStr">
@@ -6979,17 +6979,17 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>Gaštanová 9, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Jána L.Bellu (Lužianky), Senec, okres Senec</t>
         </is>
       </c>
       <c r="B297" t="inlineStr">
         <is>
-          <t>Iveta Kopecká</t>
+          <t>Marian Mičko</t>
         </is>
       </c>
       <c r="C297" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D297" s="2" t="inlineStr">
@@ -7001,17 +7001,17 @@
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>Jána L.Bellu (Lužianky), Senec, okres Senec</t>
+          <t>Stavbárska 5177, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B298" t="inlineStr">
         <is>
-          <t>Marian Mičko</t>
+          <t>Adriana D</t>
         </is>
       </c>
       <c r="C298" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D298" s="2" t="inlineStr">
@@ -7023,17 +7023,17 @@
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>Stavbárska 5177, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>Adriana D</t>
+          <t>Jozef súkromná osoba</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Hotel / penzión</t>
         </is>
       </c>
       <c r="D299" s="2" t="inlineStr">
@@ -7045,17 +7045,17 @@
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>Modra, okres Pezinok</t>
+          <t>Dunajská, Most pri Bratislave, okres Senec</t>
         </is>
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>Jozef súkromná osoba</t>
+          <t>Ľuboš Štvrtecký</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
         <is>
-          <t>Hotel / penzión</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D300" s="2" t="inlineStr">
@@ -7067,17 +7067,17 @@
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>Dunajská, Most pri Bratislave, okres Senec</t>
+          <t>Pionierska, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>Ľuboš Štvrtecký</t>
+          <t>Peter Nagy</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D301" s="2" t="inlineStr">
@@ -7089,17 +7089,17 @@
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>Pionierska, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Koniarková, Bratislava-Vajnory, okres Bratislava III</t>
         </is>
       </c>
       <c r="B302" t="inlineStr">
         <is>
-          <t>Peter Nagy</t>
+          <t>Daniela Kiniková</t>
         </is>
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D302" s="2" t="inlineStr">
@@ -7111,17 +7111,17 @@
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>Koniarková, Bratislava-Vajnory, okres Bratislava III</t>
+          <t>Opálová, Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B303" t="inlineStr">
         <is>
-          <t>Daniela Kiniková</t>
+          <t>Jana Malisova</t>
         </is>
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D303" s="2" t="inlineStr">
@@ -7133,17 +7133,17 @@
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>Opálová, Bratislava-Jarovce, okres Bratislava V</t>
+          <t>Hydinárska 9617, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B304" t="inlineStr">
         <is>
-          <t>Jana Malisova</t>
+          <t>Alex Medek</t>
         </is>
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D304" s="2" t="inlineStr">
@@ -7155,12 +7155,12 @@
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>Hydinárska 9617, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Slnečné jazerá, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B305" t="inlineStr">
         <is>
-          <t>Alex Medek</t>
+          <t>Filip Lečko</t>
         </is>
       </c>
       <c r="C305" t="inlineStr">
@@ -7177,17 +7177,17 @@
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>Slnečné jazerá, Senec, okres Senec</t>
+          <t>Banšelova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B306" t="inlineStr">
         <is>
-          <t>Filip Lečko</t>
+          <t>Ivan Beňo</t>
         </is>
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D306" s="2" t="inlineStr">
@@ -7199,17 +7199,17 @@
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>Banšelova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Avanárska, Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B307" t="inlineStr">
         <is>
-          <t>Ivan Beňo</t>
+          <t>Julius Bohunsky</t>
         </is>
       </c>
       <c r="C307" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D307" s="2" t="inlineStr">
@@ -7221,17 +7221,17 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>Avanárska, Rohožník, okres Malacky</t>
+          <t>Dlhé diely, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B308" t="inlineStr">
         <is>
-          <t>Julius Bohunsky</t>
+          <t>Matusk Tomas</t>
         </is>
       </c>
       <c r="C308" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D308" s="2" t="inlineStr">
@@ -7243,17 +7243,17 @@
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>Dlhé diely, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Jozefa Kubinu, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B309" t="inlineStr">
         <is>
-          <t>Matusk Tomas</t>
+          <t>Martina Hlubocká</t>
         </is>
       </c>
       <c r="C309" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D309" s="2" t="inlineStr">
@@ -7265,17 +7265,17 @@
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>Jozefa Kubinu, Malacky, okres Malacky</t>
+          <t>Markova 7, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B310" t="inlineStr">
         <is>
-          <t>Martina Hlubocká</t>
+          <t>Martin Číž</t>
         </is>
       </c>
       <c r="C310" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D310" s="2" t="inlineStr">
@@ -7287,17 +7287,17 @@
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>Markova 7, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B311" t="inlineStr">
         <is>
-          <t>Martin Číž</t>
+          <t>Peter Kovár</t>
         </is>
       </c>
       <c r="C311" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D311" s="2" t="inlineStr">
@@ -7309,17 +7309,17 @@
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Steinov dvor, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B312" t="inlineStr">
         <is>
-          <t>Peter Kovár</t>
+          <t>Ing Šalátová Zuzana</t>
         </is>
       </c>
       <c r="C312" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D312" s="2" t="inlineStr">
@@ -7331,17 +7331,17 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>Steinov dvor, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Svätý Martin, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B313" t="inlineStr">
         <is>
-          <t>Ing Šalátová Zuzana</t>
+          <t>Stanislav Sakac</t>
         </is>
       </c>
       <c r="C313" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D313" s="2" t="inlineStr">
@@ -7353,17 +7353,17 @@
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>Svätý Martin, Senec, okres Senec</t>
+          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t>Stanislav Sakac</t>
+          <t>Sandra zahradnikova</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D314" s="2" t="inlineStr">
@@ -7375,17 +7375,17 @@
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Žižkova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t>Sandra zahradnikova</t>
+          <t>Denisa Slančová</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D315" s="2" t="inlineStr">
@@ -7397,17 +7397,17 @@
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>Žižkova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Strmý vŕšok 164, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t>Denisa Slančová</t>
+          <t>Tereza Adámyová</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D316" s="2" t="inlineStr">
@@ -7419,17 +7419,17 @@
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>Strmý vŕšok 164, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
+          <t>Lackova, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t>Tereza Adámyová</t>
+          <t>Predaj Bytu</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D317" s="2" t="inlineStr">
@@ -7441,17 +7441,17 @@
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>Lackova, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t>Predaj Bytu</t>
+          <t>Tatiana B</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D318" s="2" t="inlineStr">
@@ -7463,17 +7463,17 @@
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>Rohožník, okres Malacky</t>
+          <t>Nevädzová 6, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t>Tatiana B</t>
+          <t>Daniel l</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D319" s="2" t="inlineStr">
@@ -7485,17 +7485,17 @@
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>Nevädzová 6, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Máchova, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t>Daniel l</t>
+          <t>Marian V</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D320" s="2" t="inlineStr">
@@ -8651,7 +8651,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>02.10.2026 21:30</t>
+          <t>03.10.2026 10:36</t>
         </is>
       </c>
     </row>
@@ -8711,7 +8711,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12">
@@ -8731,7 +8731,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="14">
@@ -8741,7 +8741,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="15">
@@ -8751,7 +8751,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17">
@@ -8780,7 +8780,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20">
@@ -8790,7 +8790,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="21">
@@ -8810,7 +8810,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="23">
@@ -8830,7 +8830,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="25">

</xml_diff>

<commit_message>
Aktualizácia ponúk – 2026-10-04 11:25 UTC
</commit_message>
<xml_diff>
--- a/public/ponuky.xlsx
+++ b/public/ponuky.xlsx
@@ -489,64 +489,64 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Most pri Bratislave, okres Senec</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Milan Martinka</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Rodinný dom</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>otvoriť ponuku</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>Táborská 10, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>vladimir cagan</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>otvoriť ponuku</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Hany Meličkovej, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Artur Y</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Obchodné priestory</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Peter Peter</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>2-izbový byt</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -555,17 +555,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Most pri Bratislave, okres Senec</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Maryna Rieznykova</t>
+          <t>Peter Peter</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -577,17 +577,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Kvetná, Rovinka, okres Senec</t>
+          <t>Most pri Bratislave, okres Senec</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Petra Janosikova</t>
+          <t>Maryna Rieznykova</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -599,12 +599,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Ondrejovova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Kvetná, Rovinka, okres Senec</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Martin Fried</t>
+          <t>Petra Janosikova</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -621,17 +621,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Ondrejovova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Tomáš Lehocký</t>
+          <t>Martin Fried</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -643,12 +643,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Landererova 6, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Mat Nav</t>
+          <t>Tomáš Lehocký</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -665,17 +665,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Mierová 200, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Landererova 6, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Richard Velky</t>
+          <t>Mat Nav</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Pozemok pre bytovú výstavbu</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -687,17 +687,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Rovinka, okres Senec</t>
+          <t>Mierová 200, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lenka B</t>
+          <t>Richard Velky</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre bytovú výstavbu</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -709,17 +709,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Rovinka, okres Senec</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Dominika Ševčíková</t>
+          <t>Lenka B</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -731,17 +731,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Sabinovská, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Zuzana Papánková</t>
+          <t>Dominika Ševčíková</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -753,17 +753,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Bajkalská 45C, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Sabinovská, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Nina Labudová</t>
+          <t>Zuzana Papánková</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -775,17 +775,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Nad Vinohradmi, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
+          <t>Bajkalská 45C, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Yury Makarov</t>
+          <t>Nina Labudová</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -797,17 +797,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Vajnorská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Nad Vinohradmi, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Dominika Koháryová</t>
+          <t>Yury Makarov</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -819,17 +819,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Cyprichova 40, Bratislava-Rača, okres Bratislava III</t>
+          <t>Vajnorská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Tomáš Samuhel</t>
+          <t>Peter Smiček</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -841,17 +841,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Miletičova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Cyprichova 40, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Tomas L</t>
+          <t>Tomáš Samuhel</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -863,17 +863,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Bebravská, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Miletičova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARZE MARZE </t>
+          <t>Tomas L</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -885,17 +885,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Devínska cesta, Bratislava-Devín, okres Bratislava IV</t>
+          <t>Bebravská, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Jana Filípková</t>
+          <t xml:space="preserve">MARZE MARZE </t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Záhrada</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -907,17 +907,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Albrechtova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Devínska cesta, Bratislava-Devín, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARZE MARZE </t>
+          <t>Jana Filípková</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Záhrada</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -929,17 +929,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Malé Vinice, Chorvátsky Grob, okres Senec</t>
+          <t>Albrechtova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Eva Husarová</t>
+          <t xml:space="preserve">MARZE MARZE </t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -951,17 +951,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Kuchyňa, okres Malacky</t>
+          <t>Malé Vinice, Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Lucia Lučanská</t>
+          <t>Eva Husarová</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -973,17 +973,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Arménska, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Kuchyňa, okres Malacky</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BYT ARMÉNSKA</t>
+          <t>Lucia Lučanská</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -995,17 +995,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Košická, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Arménska, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Filip Jandura</t>
+          <t>BYT ARMÉNSKA</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1017,17 +1017,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Domkárska, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Košická, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Peter Baláž</t>
+          <t>Filip Jandura</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1039,17 +1039,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Riazanská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Domkárska, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Marián Petráš</t>
+          <t>Peter Baláž</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1061,17 +1061,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Burgundská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Riazanská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>IGS real Ivan</t>
+          <t>Marián Petráš</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -1083,17 +1083,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Sokolská, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Burgundská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Sona Pircova</t>
+          <t>IGS real Ivan</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1105,17 +1105,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Štúrova, Marianka, okres Malacky</t>
+          <t>Sokolská, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>borisfkovac Kovac</t>
+          <t>Sona Pircova</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -1127,17 +1127,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Školská, Chorvátsky Grob, okres Senec</t>
+          <t>Štúrova, Marianka, okres Malacky</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Denis Zamocky</t>
+          <t>borisfkovac Kovac</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1149,17 +1149,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mlynské nivy 57, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Školská, Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Stefan Niznik</t>
+          <t>Denis Zamocky</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -1171,12 +1171,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Drobného, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Mlynské nivy 57, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Gabriela Cermakova</t>
+          <t>Stefan Niznik</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1193,12 +1193,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Miletičova 35, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Drobného, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Lubo Lajos</t>
+          <t>Gabriela Cermakova</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1215,12 +1215,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Ulica Svornosti, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Miletičova 35, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Marek Bacik</t>
+          <t>Lubo Lajos</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1237,17 +1237,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jungmannova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Ulica Svornosti, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Vaso Bratislava</t>
+          <t>Marek Bacik</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -1259,17 +1259,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Brusnicová 13, Chorvátsky Grob, okres Senec</t>
+          <t>Jungmannova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Dušan Pokoš</t>
+          <t>Vaso Bratislava</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -1281,17 +1281,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Gavlovičova, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Brusnicová 13, Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Michal K</t>
+          <t>Dušan Pokoš</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -1303,17 +1303,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Vlčie hrdlo 85, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Gavlovičova, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Natalia Kubicova</t>
+          <t>Michal K</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -1325,12 +1325,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Hrachová 16C, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Vlčie hrdlo 85, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Dušan Pokoš</t>
+          <t>Natalia Kubicova</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1347,17 +1347,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Planét, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Hrachová 16C, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Július Július</t>
+          <t>Dušan Pokoš</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -1369,12 +1369,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Skalná, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Planét, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>katarina sekerka</t>
+          <t>Július Július</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1391,17 +1391,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Heyrovského, Bratislava-Lamač, okres Bratislava IV</t>
+          <t>Skalná, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Maros Palik</t>
+          <t>katarina sekerka</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -1413,17 +1413,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Oravská 2, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Heyrovského, Bratislava-Lamač, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Zdena Bartošová</t>
+          <t>Maros Palik</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -1435,17 +1435,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Jarabinková 2, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Oravská 2, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Michael Kollár</t>
+          <t>Zdena Bartošová</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -1457,7 +1457,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Miletičova 60, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Jarabinková 2, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1467,7 +1467,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -1479,12 +1479,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Bernolákova 2, Senec, okres Senec</t>
+          <t>Miletičova 60, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Šimon Klúčik</t>
+          <t>Michael Kollár</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1501,17 +1501,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Rovinka, okres Senec</t>
+          <t>Bernolákova 2, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Petra Sárkány</t>
+          <t>Šimon Klúčik</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -1523,17 +1523,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>J. Holčeka, Budmerice, okres Pezinok</t>
+          <t>Rovinka, okres Senec</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Ondrej Kolciter</t>
+          <t>Petra Sárkány</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -1567,17 +1567,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Chorvátsky Grob, okres Senec</t>
+          <t>J. Holčeka, Budmerice, okres Pezinok</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Dada Garajova</t>
+          <t>Ondrej Kolciter</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -1589,17 +1589,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Bajkalská 45C, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Eva Valáriková</t>
+          <t>Dada Garajova</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -1611,17 +1611,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Trebišovská, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bajkalská 45C, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Ružinov Štrkovec</t>
+          <t>Eva Valáriková</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -1633,17 +1633,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Rohožník, okres Malacky</t>
+          <t>Trebišovská, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Sukromna Osoba</t>
+          <t>Ružinov Štrkovec</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -1655,17 +1655,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Senec, okres Senec</t>
+          <t>Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Jakub Králik</t>
+          <t>Sukromna Osoba</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -1677,17 +1677,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Malacky, okres Malacky</t>
+          <t>Senec, okres Senec</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Elena Straznicka</t>
+          <t>Jakub Králik</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -1699,12 +1699,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Holubia, Senec, okres Senec</t>
+          <t>Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Marko Klúčik</t>
+          <t>Elena Straznicka</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -1721,17 +1721,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>1mája, Pezinok, okres Pezinok</t>
+          <t>Holubia, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Ladislav Ružek</t>
+          <t>Marko Klúčik</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -1743,17 +1743,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>1mája, Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Lukas Durinak</t>
+          <t>Ladislav Ružek</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -1765,17 +1765,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Okružná 47, Senec, okres Senec</t>
+          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Roman Gazdik</t>
+          <t>Lukas Durinak</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -1787,17 +1787,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Kozia, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Okružná 47, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Ľubor Mendel</t>
+          <t>Roman Gazdik</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -1809,17 +1809,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Dopravná 23, Bratislava-Rača, okres Bratislava III</t>
+          <t>Kozia, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Peter Pipiš</t>
+          <t>Ľubor Mendel</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -1831,17 +1831,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Šalviová, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Dopravná 23, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Juraj Valašťan</t>
+          <t>Peter Pipiš</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -1853,12 +1853,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Agátová, Ivanka pri Dunaji, okres Senec</t>
+          <t>Šalviová, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Viktória Krupová</t>
+          <t>Juraj Valašťan</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -1875,17 +1875,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Kaplinská 7, Bratislava-Rača, okres Bratislava III</t>
+          <t>Agátová, Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Eva Žíhlavníková</t>
+          <t>Viktória Krupová</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -1897,17 +1897,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Repašského 1, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Kaplinská 7, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Michal Weismann</t>
+          <t>Eva Žíhlavníková</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -1929,7 +1929,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -1941,17 +1941,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Repašského 1, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Alexander Kernaševič</t>
+          <t>Michal Weismann</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Mobile cells and stands</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -1963,17 +1963,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Landererova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Simona Kourdi</t>
+          <t>Alexander Kernaševič</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Mobile cells and stands</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -1985,17 +1985,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>167, Borinka, okres Malacky</t>
+          <t>Landererova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Kamil Semeš</t>
+          <t>Simona Kourdi</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -2007,17 +2007,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Gregorovej, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>167, Borinka, okres Malacky</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Andrej Miko</t>
+          <t>Kamil Semeš</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -2029,17 +2029,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Jablonec, okres Pezinok</t>
+          <t>Gregorovej, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Andrea Valentová</t>
+          <t>Andrej Miko</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -2051,17 +2051,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Ivanka pri Dunaji, okres Senec</t>
+          <t>Jablonec, okres Pezinok</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Andrea Bášková</t>
+          <t>Andrea Valentová</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -2073,12 +2073,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Katarína Rusňáková</t>
+          <t>Andrea Bášková</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -2095,12 +2095,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Ulica 8. mája 22A, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Vladimír Mitrík</t>
+          <t>Katarína Rusňáková</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -2117,17 +2117,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Partizánska 1081, Malacky, okres Malacky</t>
+          <t>Ulica 8. mája 22A, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Peter Ondrovič</t>
+          <t>Vladimír Mitrík</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -2139,12 +2139,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Čulenova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Partizánska 1081, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>M I</t>
+          <t>Peter Ondrovič</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2161,17 +2161,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Lachova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Čulenova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Zuzana V</t>
+          <t>M I</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -2183,17 +2183,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Drobného, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Lachova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Peter Chovanec</t>
+          <t>Zuzana V</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -2205,17 +2205,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Vysoká pri Morave, okres Malacky</t>
+          <t>Drobného, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Miroslav Vojkovic</t>
+          <t>Peter Chovanec</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -2227,12 +2227,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Vinárska, Modra, okres Pezinok</t>
+          <t>Vysoká pri Morave, okres Malacky</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>marek rozic</t>
+          <t>Miroslav Vojkovic</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2249,17 +2249,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Vinárska, Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Anton K</t>
+          <t>marek rozic</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -2271,17 +2271,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Tupolevova 18, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Ivan Hargas</t>
+          <t>Anton K</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -2293,12 +2293,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Stavbárska 4, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Tupolevova 18, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Jaroslav Valus</t>
+          <t>Ivan Hargas</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2315,17 +2315,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Bratislava-Vajnory, okres Bratislava III</t>
+          <t>Stavbárska 4, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Juraj Varacka</t>
+          <t>Jaroslav Valus</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
@@ -2337,17 +2337,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Papraďová, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Vajnory, okres Bratislava III</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Jana Zemanova</t>
+          <t>Juraj Varacka</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -2359,17 +2359,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Papraďová, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Juraj Litomerický</t>
+          <t>Jana Zemanova</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -2381,17 +2381,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Vyšehradská 16, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Juraj Kovašich</t>
+          <t>Juraj Litomerický</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -2403,17 +2403,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Grösslingova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Vyšehradská 16, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Viktor Riegel</t>
+          <t>Juraj Kovašich</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -2425,17 +2425,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Sekurisova, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Grösslingova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Matej Kohucik</t>
+          <t>Viktor Riegel</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -2447,17 +2447,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Ipeľská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Sekurisova, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>David Ivanov</t>
+          <t>Matej Kohucik</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -2469,17 +2469,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Karloveské rameno, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Ipeľská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Boris Emrich</t>
+          <t>David Ivanov</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -2491,17 +2491,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Malokrasňanská 8, Bratislava-Rača, okres Bratislava III</t>
+          <t>Karloveské rameno, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Paula Baranová</t>
+          <t>Boris Emrich</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -2513,17 +2513,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Tomášikova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Malokrasňanská 8, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>BaTom P</t>
+          <t>Paula Baranová</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -2535,17 +2535,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Krížna, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Tomášikova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Peter Valenta</t>
+          <t>BaTom P</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Kancelárie</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
@@ -2557,17 +2557,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Námestie Slobody, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Krížna, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Martin Gažo</t>
+          <t>Peter Valenta</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Kancelárie</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
@@ -2579,17 +2579,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Bratislava-Rusovce, okres Bratislava V</t>
+          <t>Námestie Slobody, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Milan Dzilsky</t>
+          <t>Martin Gažo</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -2601,17 +2601,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Rovniankova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Bratislava-Rusovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Roman N</t>
+          <t>Milan Dzilsky</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
@@ -2623,17 +2623,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Rovniankova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Martin Chamko</t>
+          <t>Roman N</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -2645,17 +2645,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Jaskový rad 47, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Angela Brinzova</t>
+          <t>Martin Chamko</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
@@ -2667,17 +2667,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Podjavorinskej 13, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Jaskový rad 47, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Tomáš Čitbaj</t>
+          <t>Angela Brinzova</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -2689,17 +2689,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Krušpánová, Bratislava-Čunovo, okres Bratislava V</t>
+          <t>Podjavorinskej 13, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Alena Horváthová</t>
+          <t>Tomáš Čitbaj</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
@@ -2711,17 +2711,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Šancová 37, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Krušpánová, Bratislava-Čunovo, okres Bratislava V</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Frantisek Manduch</t>
+          <t>Alena Horváthová</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -2733,17 +2733,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Malé Leváre, okres Malacky</t>
+          <t>Šancová 37, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Michal Fajták</t>
+          <t>Frantisek Manduch</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
@@ -2755,17 +2755,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Komenského, Modra, okres Pezinok</t>
+          <t>Malé Leváre, okres Malacky</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Richard Baranovic</t>
+          <t>Michal Fajták</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
@@ -2777,17 +2777,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Markova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Komenského, Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Peter Novotný</t>
+          <t>Richard Baranovic</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
@@ -2799,12 +2799,12 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Hornádska 28, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Markova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Miro Kralovic</t>
+          <t>Peter Novotný</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -2821,12 +2821,12 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Plzenská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Hornádska 28, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Peter Kubica</t>
+          <t>Miro Kralovic</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -2843,17 +2843,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Saratovská 14, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Plzenská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Michal Podlucký</t>
+          <t>Peter Kubica</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
@@ -2865,17 +2865,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Saratovská 14, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Lukáš K</t>
+          <t>Michal Podlucký</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
@@ -2887,17 +2887,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Hattalova, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Šťastný  Vlastník</t>
+          <t>Lukáš K</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
@@ -2909,17 +2909,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Slovenský Grob, okres Pezinok</t>
+          <t>Hattalova, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Jozef Brom</t>
+          <t>Šťastný  Vlastník</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
@@ -2931,17 +2931,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Slovenský Grob, okres Pezinok</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>MM victory</t>
+          <t>Jozef Brom</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
@@ -2953,17 +2953,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Bernolákova, Nová Dedinka, okres Senec</t>
+          <t>Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Karina Szutyányiová</t>
+          <t>MM victory</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
@@ -2975,17 +2975,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Senec, okres Senec</t>
+          <t>Bernolákova, Nová Dedinka, okres Senec</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>RD RD</t>
+          <t>Karina Szutyányiová</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
@@ -2997,12 +2997,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Školská, Rovinka, okres Senec</t>
+          <t>Senec, okres Senec</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Alena Alena</t>
+          <t>RD RD</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -3019,17 +3019,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Školská, Rovinka, okres Senec</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Lukas Novosiadly </t>
+          <t>Alena Alena</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
@@ -3041,17 +3041,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Hany Zelinovej, Senec, okres Senec</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Peter Veselsky</t>
+          <t xml:space="preserve">Lukas Novosiadly </t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
@@ -3063,17 +3063,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Dunajská, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Hany Zelinovej, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Tatiana B</t>
+          <t>Peter Veselsky</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>5+ izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
@@ -3085,17 +3085,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Malacky, okres Malacky</t>
+          <t>Dunajská, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Martin Jendek</t>
+          <t>Tatiana B</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>5+ izbový byt</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
@@ -8605,7 +8605,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>03.10.2026 20:06</t>
+          <t>04.10.2026 11:25</t>
         </is>
       </c>
     </row>
@@ -8651,17 +8651,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>okres Bratislava IV</t>
+          <t>okres Senec</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>okres Senec</t>
+          <t>okres Bratislava IV</t>
         </is>
       </c>
       <c r="B11" t="n">
@@ -8691,7 +8691,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>okres Malacky</t>
+          <t>okres Pezinok</t>
         </is>
       </c>
       <c r="B14" t="n">
@@ -8701,11 +8701,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>okres Pezinok</t>
+          <t>okres Malacky</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="17">
@@ -8730,21 +8730,21 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Aktualizácia ponúk – 2026-10-11 11:38 UTC
</commit_message>
<xml_diff>
--- a/public/ponuky.xlsx
+++ b/public/ponuky.xlsx
@@ -489,64 +489,64 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Nobelovo nám., Bratislava-Petržalka, okres Bratislava V</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Michal Weismann</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>2-izbový byt</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>otvoriť ponuku</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>Odborárska 3, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>J D</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>otvoriť ponuku</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Ivan Styk</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>Bratislava-Jarovce, okres Bratislava V</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Ivan Styk</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Pozemok pre rodinný dom</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="4" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -555,17 +555,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Mýtna 50, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bratislava-Jarovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Miloš Roško</t>
+          <t>Ivan Styk</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -577,17 +577,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Frankovská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Mýtna 50, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Michal Klempai</t>
+          <t>Miloš Roško</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -599,17 +599,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Nobelova 12C, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Frankovská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Radovan Hýbl</t>
+          <t>Michal Klempai</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -621,42 +621,42 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Pri Šajbách, Bratislava-Rača, okres Bratislava III</t>
+          <t>Nobelova 12C, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Andrea Peciarova</t>
+          <t>Radovan Hýbl</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>2-izbový byt</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>otvoriť ponuku</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Na Grunte, Bratislava-Nové Mesto, okres Bratislava III</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Katarina K</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Malacky, okres Malacky</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Viliam Pavelka</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>Rodinný dom</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -665,12 +665,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Nábrežie arm. gen. Ludvíka Svobodu 20, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Pri Šajbách, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Marek  MV MV</t>
+          <t>Andrea Peciarova</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -687,17 +687,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Martin Číž</t>
+          <t>Viliam Pavelka</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -709,17 +709,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Jarabinková 2C, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Nábrežie arm. gen. Ludvíka Svobodu 20, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Jozef Border</t>
+          <t>Marek  MV MV</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -753,17 +753,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Blagoevova 16, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Jarabinková 2C, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Marek Chudý</t>
+          <t>Jozef Border</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Double studio apartment</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -775,17 +775,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Pod Kopcami, Stupava, okres Malacky</t>
+          <t>Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Peter Glasa</t>
+          <t>Martin Číž</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -797,17 +797,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Plavecký Štvrtok, okres Malacky</t>
+          <t>Blagoevova 16, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Bianka Chmelová</t>
+          <t>Marek Chudý</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Double studio apartment</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -819,17 +819,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Nechtíková ulica, Rovinka, okres Senec</t>
+          <t>Pod Kopcami, Stupava, okres Malacky</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Marcel Polák</t>
+          <t>Peter Glasa</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -841,17 +841,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Malacky, okres Malacky</t>
+          <t>Plavecký Štvrtok, okres Malacky</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Lucia Blažeková</t>
+          <t>Bianka Chmelová</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -863,12 +863,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>497, Plavecký Štvrtok, okres Malacky</t>
+          <t>Nechtíková ulica, Rovinka, okres Senec</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Lucia Blažeková</t>
+          <t>Marcel Polák</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -885,17 +885,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Vysoká 9, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Partner Technic</t>
+          <t>Lucia Blažeková</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -907,17 +907,17 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ondavská, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>497, Plavecký Štvrtok, okres Malacky</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Jakub Peťko</t>
+          <t>Lucia Blažeková</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
@@ -929,17 +929,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Jurigovo nám., Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Vysoká 9, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Roman Babiar</t>
+          <t>Partner Technic</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -951,12 +951,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Legerského 8, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Ondavská, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Michal Rajter</t>
+          <t>Jakub Peťko</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -973,17 +973,17 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Podunajská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Jurigovo nám., Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Martin Mašata</t>
+          <t>Roman Babiar</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Polyfunkčná budova</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
@@ -995,17 +995,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Kostolná pri Dunaji, okres Senec</t>
+          <t>Legerského 8, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Michal P</t>
+          <t>Michal Rajter</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1017,17 +1017,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Šenkvice, okres Pezinok</t>
+          <t>Podunajská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Marek Kakalik</t>
+          <t>Martin Mašata</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Orná pôda</t>
+          <t>Polyfunkčná budova</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1039,17 +1039,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Galvaniho, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Kostolná pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Kristína Mizeráková</t>
+          <t>Michal P</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1061,17 +1061,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Za kostolom, Kostolište, okres Malacky</t>
+          <t>Šenkvice, okres Pezinok</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Ferdinand Havlík</t>
+          <t>Marek Kakalik</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Orná pôda</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -1083,17 +1083,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Kyjevská 2, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Galvaniho, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Monika Faltinová</t>
+          <t>Kristína Mizeráková</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -1105,17 +1105,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Za kostolom, Kostolište, okres Malacky</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Iveta Škubová</t>
+          <t>Ferdinand Havlík</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -1127,17 +1127,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Koceľova 21, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Kyjevská 2, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Eva Valáriková</t>
+          <t>Monika Faltinová</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1149,17 +1149,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mečíková 5823, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
+          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Jana Varga Bitova</t>
+          <t>Iveta Škubová</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -1171,17 +1171,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Koceľova 21, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Jan Plch</t>
+          <t>Eva Valáriková</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -1193,17 +1193,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Mečíková 5823, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Zuzana Vlková</t>
+          <t>Jana Varga Bitova</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -1215,17 +1215,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Palisády, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Alexandra Litecka</t>
+          <t>Jan Plch</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>5+ izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -1237,17 +1237,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Černyševského, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Vladimir Jagr</t>
+          <t>Zuzana Vlková</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -1259,17 +1259,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Žabí majer, Bratislava-Rača, okres Bratislava III</t>
+          <t>Palisády, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Lydia Hentekova</t>
+          <t>Alexandra Litecka</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Záhrada</t>
+          <t>5+ izbový byt</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -1281,17 +1281,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Smikova, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Černyševského, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Kamil Vrabeľ</t>
+          <t>Vladimir Jagr</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -1303,17 +1303,17 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Šancová 74, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Žabí majer, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Juraj Jediný</t>
+          <t>Lydia Hentekova</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Záhrada</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -1325,17 +1325,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Somolického 6, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Smikova, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Viktória Peniaková</t>
+          <t>Kamil Vrabeľ</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -1347,17 +1347,17 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Šancová 74, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>R K</t>
+          <t>Juraj Jediný</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
@@ -1369,17 +1369,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Somolického 6, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Zuzana Vreckova</t>
+          <t>Viktória Peniaková</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -1391,17 +1391,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>14050, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Dominika Bachrata</t>
+          <t>R K</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -1413,7 +1413,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1423,7 +1423,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -1435,17 +1435,17 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Harmónia, Modra, okres Pezinok</t>
+          <t>14050, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Silvia Papugová</t>
+          <t>Dominika Bachrata</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
@@ -1457,17 +1457,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Štefánikova 82, Modra, okres Pezinok</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Peter Juran</t>
+          <t>Zuzana Vreckova</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -1479,17 +1479,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Gregorovej, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Harmónia, Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Dadka Kesjar</t>
+          <t>Silvia Papugová</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -1501,17 +1501,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Most pri Bratislave, okres Senec</t>
+          <t>Štefánikova 82, Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Zahrada Most</t>
+          <t>Peter Juran</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Záhradná chatka</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -1523,17 +1523,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>521, Borinka, okres Malacky</t>
+          <t>Gregorovej, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Miroslav Hollý</t>
+          <t>Dadka Kesjar</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
@@ -1545,17 +1545,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Most pri Bratislave, okres Senec</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Dagmar Semrisová</t>
+          <t>Zahrada Most</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Záhradná chatka</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -1567,12 +1567,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Most pri Bratislave, okres Senec</t>
+          <t>521, Borinka, okres Malacky</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Milan Martinka</t>
+          <t>Miroslav Hollý</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -1589,17 +1589,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Táborská 10, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>vladimir cagan</t>
+          <t>Dagmar Semrisová</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -1611,17 +1611,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Hany Meličkovej, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Most pri Bratislave, okres Senec</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Artur Y</t>
+          <t>Milan Martinka</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Obchodné priestory</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -1633,17 +1633,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Táborská 10, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Peter Peter</t>
+          <t>vladimir cagan</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -1655,17 +1655,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Most pri Bratislave, okres Senec</t>
+          <t>Hany Meličkovej, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Maryna Rieznykova</t>
+          <t>Artur Y</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Obchodné priestory</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -1677,17 +1677,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Kvetná, Rovinka, okres Senec</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Petra Janosikova</t>
+          <t>Peter Peter</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -1699,17 +1699,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Ondrejovova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Most pri Bratislave, okres Senec</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Martin Fried</t>
+          <t>Maryna Rieznykova</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -1721,17 +1721,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Kvetná, Rovinka, okres Senec</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Tomáš Lehocký</t>
+          <t>Petra Janosikova</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -1743,17 +1743,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Uzbecká, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Ondrejovova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Mária Mériová</t>
+          <t>Martin Fried</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Other type of apartment</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -1765,12 +1765,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Landererova 6, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Mat Nav</t>
+          <t>Tomáš Lehocký</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -1787,17 +1787,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Mierová 200, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Uzbecká, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Richard Velky</t>
+          <t>Mária Mériová</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Pozemok pre bytovú výstavbu</t>
+          <t>Other type of apartment</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -1809,17 +1809,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Rovinka, okres Senec</t>
+          <t>Landererova 6, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Lenka B</t>
+          <t>Mat Nav</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -1831,17 +1831,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Mierová 200, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Dominika Ševčíková</t>
+          <t>Richard Velky</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre bytovú výstavbu</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
@@ -1853,17 +1853,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Sabinovská, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Rovinka, okres Senec</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Zuzana Papánková</t>
+          <t>Lenka B</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -1875,17 +1875,17 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Bajkalská 45C, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Nina Labudová</t>
+          <t>Dominika Ševčíková</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -1897,17 +1897,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Nad Vinohradmi, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
+          <t>Sabinovská, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Yury Makarov</t>
+          <t>Zuzana Papánková</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -1919,17 +1919,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Vajnorská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Bajkalská 45C, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Peter Smiček</t>
+          <t>Nina Labudová</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -1941,17 +1941,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Cyprichova 40, Bratislava-Rača, okres Bratislava III</t>
+          <t>Nad Vinohradmi, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Tomáš Samuhel</t>
+          <t>Yury Makarov</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -1963,12 +1963,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Miletičova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Vajnorská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Tomas L</t>
+          <t>Peter Smiček</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -1985,17 +1985,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Bebravská, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Cyprichova 40, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARZE MARZE </t>
+          <t>Tomáš Samuhel</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -2007,17 +2007,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Devínska cesta, Bratislava-Devín, okres Bratislava IV</t>
+          <t>Miletičova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Jana Filípková</t>
+          <t>Tomas L</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Záhrada</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -2029,7 +2029,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Albrechtova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bebravská, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -2051,17 +2051,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Malé Vinice, Chorvátsky Grob, okres Senec</t>
+          <t>Devínska cesta, Bratislava-Devín, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Eva Husarová</t>
+          <t>Jana Filípková</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Záhrada</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -2073,17 +2073,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Kuchyňa, okres Malacky</t>
+          <t>Albrechtova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Lucia Lučanská</t>
+          <t xml:space="preserve">MARZE MARZE </t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
@@ -2095,17 +2095,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Arménska, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Malé Vinice, Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>BYT ARMÉNSKA</t>
+          <t>Eva Husarová</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -2117,17 +2117,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Košická, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Kuchyňa, okres Malacky</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Filip Jandura</t>
+          <t>Lucia Lučanská</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -2139,12 +2139,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Domkárska, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Arménska, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Peter Baláž</t>
+          <t>BYT ARMÉNSKA</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2161,17 +2161,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Riazanská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Košická, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Marián Petráš</t>
+          <t>Filip Jandura</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -2183,17 +2183,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Burgundská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Domkárska, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>IGS real Ivan</t>
+          <t>Peter Baláž</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -2205,17 +2205,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Štúrova, Marianka, okres Malacky</t>
+          <t>Riazanská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>borisfkovac Kovac</t>
+          <t>Marián Petráš</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -2227,12 +2227,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Školská, Chorvátsky Grob, okres Senec</t>
+          <t>Burgundská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Denis Zamocky</t>
+          <t>IGS real Ivan</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -2249,17 +2249,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Mlynské nivy 57, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Štúrova, Marianka, okres Malacky</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Stefan Niznik</t>
+          <t>borisfkovac Kovac</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -2271,17 +2271,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Drobného, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Školská, Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Gabriela Cermakova</t>
+          <t>Denis Zamocky</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -2293,12 +2293,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Miletičova 35, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Mlynské nivy 57, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Lubo Lajos</t>
+          <t>Stefan Niznik</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -2315,12 +2315,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Ulica Svornosti, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Drobného, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Marek Bacik</t>
+          <t>Gabriela Cermakova</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2337,17 +2337,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Jungmannova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Miletičova 35, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Vaso Bratislava</t>
+          <t>Lubo Lajos</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -2359,17 +2359,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Brusnicová 13, Chorvátsky Grob, okres Senec</t>
+          <t>Ulica Svornosti, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Dušan Pokoš</t>
+          <t>Marek Bacik</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -2381,17 +2381,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Gavlovičova, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Jungmannova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Michal K</t>
+          <t>Vaso Bratislava</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -2403,17 +2403,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Vlčie hrdlo 85, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Brusnicová 13, Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Natalia Kubicova</t>
+          <t>Dušan Pokoš</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -2425,17 +2425,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Hrachová 16C, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Gavlovičova, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Dušan Pokoš</t>
+          <t>Michal K</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -2447,17 +2447,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Planét, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Vlčie hrdlo 85, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Július Július</t>
+          <t>Natalia Kubicova</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -2469,17 +2469,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Skalná, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Hrachová 16C, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>katarina sekerka</t>
+          <t>Dušan Pokoš</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -2491,17 +2491,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Heyrovského, Bratislava-Lamač, okres Bratislava IV</t>
+          <t>Planét, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Maros Palik</t>
+          <t>Július Július</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -2513,12 +2513,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Oravská 2, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Skalná, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Zdena Bartošová</t>
+          <t>katarina sekerka</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -2535,17 +2535,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Jarabinková 2, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Heyrovského, Bratislava-Lamač, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Michael Kollár</t>
+          <t>Maros Palik</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
@@ -2557,17 +2557,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Miletičova 60, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Oravská 2, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Michael Kollár</t>
+          <t>Zdena Bartošová</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
@@ -2579,17 +2579,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Rovinka, okres Senec</t>
+          <t>Jarabinková 2, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Petra Sárkány</t>
+          <t>Michael Kollár</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -2601,17 +2601,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>J. Holčeka, Budmerice, okres Pezinok</t>
+          <t>Miletičova 60, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Ondrej Kolciter</t>
+          <t>Michael Kollár</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
@@ -2623,17 +2623,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>J. Holčeka, Budmerice, okres Pezinok</t>
+          <t>Rovinka, okres Senec</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Ondrej Kolciter</t>
+          <t>Petra Sárkány</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -2645,17 +2645,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Chorvátsky Grob, okres Senec</t>
+          <t>J. Holčeka, Budmerice, okres Pezinok</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Dada Garajova</t>
+          <t>Ondrej Kolciter</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
@@ -2667,17 +2667,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Bajkalská 45C, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>J. Holčeka, Budmerice, okres Pezinok</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Eva Valáriková</t>
+          <t>Ondrej Kolciter</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -2689,12 +2689,12 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Senec, okres Senec</t>
+          <t>Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Jakub Králik</t>
+          <t>Dada Garajova</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -2711,12 +2711,12 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Malacky, okres Malacky</t>
+          <t>Bajkalská 45C, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Elena Straznicka</t>
+          <t>Eva Valáriková</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -2733,17 +2733,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Holubia, Senec, okres Senec</t>
+          <t>Senec, okres Senec</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Marko Klúčik</t>
+          <t>Jakub Králik</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
@@ -2755,12 +2755,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Jelačičova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Lara Kristi</t>
+          <t>Elena Straznicka</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -2777,17 +2777,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>1mája, Pezinok, okres Pezinok</t>
+          <t>Holubia, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Ladislav Ružek</t>
+          <t>Marko Klúčik</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
@@ -2799,17 +2799,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Okružná 47, Senec, okres Senec</t>
+          <t>Jelačičova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Roman Gazdik</t>
+          <t>Lara Kristi</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
@@ -2821,17 +2821,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Kozia, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>1mája, Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Ľubor Mendel</t>
+          <t>Ladislav Ružek</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
@@ -2843,17 +2843,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Šalviová, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Okružná 47, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Juraj Valašťan</t>
+          <t>Roman Gazdik</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
@@ -2865,17 +2865,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Rovinka, okres Senec</t>
+          <t>Kozia, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Miroslav Vancik</t>
+          <t>Ľubor Mendel</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
@@ -2887,12 +2887,12 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Agátová, Ivanka pri Dunaji, okres Senec</t>
+          <t>Šalviová, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Viktória Krupová</t>
+          <t>Juraj Valašťan</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -2909,17 +2909,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Kaplinská 7, Bratislava-Rača, okres Bratislava III</t>
+          <t>Rovinka, okres Senec</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Eva Žíhlavníková</t>
+          <t>Miroslav Vancik</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
@@ -2931,17 +2931,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Repašského 1, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Agátová, Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Michal Weismann</t>
+          <t>Viktória Krupová</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
@@ -2953,17 +2953,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Repašského 1, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Kaplinská 7, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Michal Weismann</t>
+          <t>Eva Žíhlavníková</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
@@ -4515,17 +4515,17 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Športová, Limbach, okres Pezinok</t>
+          <t>Častá, okres Pezinok</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Michal Mravec</t>
+          <t>Monika Zatkalíková</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Záhradná chatka</t>
         </is>
       </c>
       <c r="D185" s="4" t="inlineStr">
@@ -4537,17 +4537,17 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>Železničiarska, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Športová, Limbach, okres Pezinok</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Dávid Uličný</t>
+          <t>Michal Mravec</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D186" s="4" t="inlineStr">
@@ -4559,17 +4559,17 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Balkánska 67, Bratislava-Rusovce, okres Bratislava V</t>
+          <t>Železničiarska, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Peter Kalas</t>
+          <t>Dávid Uličný</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D187" s="4" t="inlineStr">
@@ -4581,17 +4581,17 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Horská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Balkánska 67, Bratislava-Rusovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Michaela Weberova</t>
+          <t>Peter Kalas</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>Mezonet</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D188" s="4" t="inlineStr">
@@ -4613,7 +4613,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Mezonet</t>
         </is>
       </c>
       <c r="D189" s="4" t="inlineStr">
@@ -4625,17 +4625,17 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Tallerova 4, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Horská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>Daniela Ondriašová</t>
+          <t>Michaela Weberova</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D190" s="4" t="inlineStr">
@@ -4647,17 +4647,17 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Bernolákova ulica, Miloslavov, okres Senec</t>
+          <t>Tallerova 4, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>Erik Mihok</t>
+          <t>Daniela Ondriašová</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D191" s="4" t="inlineStr">
@@ -4669,12 +4669,12 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Bratislava-Rusovce, okres Bratislava V</t>
+          <t>Bernolákova ulica, Miloslavov, okres Senec</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>Alexandra Belašičová</t>
+          <t>Erik Mihok</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -4691,17 +4691,17 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>L. Novomeského, Pezinok, okres Pezinok</t>
+          <t>Bratislava-Rusovce, okres Bratislava V</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>Stefan PASTVA</t>
+          <t>Alexandra Belašičová</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D193" s="4" t="inlineStr">
@@ -4713,17 +4713,17 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Vyšehradská, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>L. Novomeského, Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>Anna Zábrelová</t>
+          <t>Stefan PASTVA</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D194" s="4" t="inlineStr">
@@ -4735,17 +4735,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Zidiny, Bratislava-Lamač, okres Bratislava IV</t>
+          <t>Vyšehradská, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>Vratislav Jurica</t>
+          <t>Anna Zábrelová</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D195" s="4" t="inlineStr">
@@ -4757,12 +4757,12 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Opálová ulica, Miloslavov, okres Senec</t>
+          <t>Zidiny, Bratislava-Lamač, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>Michal Farsky</t>
+          <t>Vratislav Jurica</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -4779,17 +4779,17 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>Hrachová 73, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Opálová ulica, Miloslavov, okres Senec</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>Patrik Písečný</t>
+          <t>Michal Farsky</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D197" s="4" t="inlineStr">
@@ -4801,12 +4801,12 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Rovniankova 4, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Hrachová 73, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>Ján Čeman</t>
+          <t>Patrik Písečný</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -4823,17 +4823,17 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Čsl. tankistov, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
+          <t>Rovniankova 4, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>Viliam Kulacs</t>
+          <t>Ján Čeman</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D199" s="4" t="inlineStr">
@@ -4845,17 +4845,17 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Palárikova 3, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Čsl. tankistov, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>Michal Michal</t>
+          <t>Viliam Kulacs</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D200" s="4" t="inlineStr">
@@ -4867,17 +4867,17 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Záhradnícka, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Palárikova 3, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>Marta Onova</t>
+          <t>Michal Michal</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D201" s="4" t="inlineStr">
@@ -4889,17 +4889,17 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Janka Kráľa, Chorvátsky Grob, okres Senec</t>
+          <t>Záhradnícka, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>Ivana Poláková</t>
+          <t>Marta Onova</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D202" s="4" t="inlineStr">
@@ -4911,17 +4911,17 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Račianska 65, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Janka Kráľa, Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>Michal Baláž</t>
+          <t>Ivana Poláková</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D203" s="4" t="inlineStr">
@@ -4933,17 +4933,17 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Potočná 9, Limbach, okres Pezinok</t>
+          <t>Račianska 65, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>Miroslav Gavalec</t>
+          <t>Michal Baláž</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D204" s="4" t="inlineStr">
@@ -4955,17 +4955,17 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Potočná 9, Limbach, okres Pezinok</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>Daniela Ondriašová</t>
+          <t>Miroslav Gavalec</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D205" s="4" t="inlineStr">
@@ -4977,17 +4977,17 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>Drotárska cesta, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>Petra Hager</t>
+          <t>Daniela Ondriašová</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D206" s="4" t="inlineStr">
@@ -4999,17 +4999,17 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>Pezinok, okres Pezinok</t>
+          <t>Drotárska cesta, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>Peter Pezinok</t>
+          <t>Petra Hager</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D207" s="4" t="inlineStr">
@@ -5021,17 +5021,17 @@
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>Karadžičova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>Tatiana B</t>
+          <t>Peter Pezinok</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D208" s="4" t="inlineStr">
@@ -5043,17 +5043,17 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Karadžičova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>Peter Kollar</t>
+          <t>Tatiana B</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Reštauračné priestory</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D209" s="4" t="inlineStr">
@@ -5065,17 +5065,17 @@
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>Bartoškova, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>Miroslav S</t>
+          <t>Peter Kollar</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Reštauračné priestory</t>
         </is>
       </c>
       <c r="D210" s="4" t="inlineStr">
@@ -5087,12 +5087,12 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>Nejedlého 20, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Bartoškova, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>Marian Placko</t>
+          <t>Miroslav S</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -5109,17 +5109,17 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>Jána L. Bellu, Senec, okres Senec</t>
+          <t>Nejedlého 20, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>Michal Sadloň</t>
+          <t>Marian Placko</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D212" s="4" t="inlineStr">
@@ -5131,17 +5131,17 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>Pri kríži, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Jána L. Bellu, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>Denisa Brozmannova</t>
+          <t>Michal Sadloň</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D213" s="4" t="inlineStr">
@@ -5153,17 +5153,17 @@
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>Sedmokrásková 3, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Pri kríži, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>Lekáreň Sedmokráska</t>
+          <t>Denisa Brozmannova</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
         <is>
-          <t>Obchodné priestory</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D214" s="4" t="inlineStr">
@@ -5175,17 +5175,17 @@
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>Svätý Jur, okres Pezinok</t>
+          <t>Sedmokrásková 3, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>Martin Kratochvíl</t>
+          <t>Lekáreň Sedmokráska</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
         <is>
-          <t>Záhrada</t>
+          <t>Obchodné priestory</t>
         </is>
       </c>
       <c r="D215" s="4" t="inlineStr">
@@ -5197,17 +5197,17 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
+          <t>Svätý Jur, okres Pezinok</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>Vaše Bývanie</t>
+          <t>Martin Kratochvíl</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Záhrada</t>
         </is>
       </c>
       <c r="D216" s="4" t="inlineStr">
@@ -5219,17 +5219,17 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>Ševčenkova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>Pavol Zlacký</t>
+          <t>Vaše Bývanie</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D217" s="4" t="inlineStr">
@@ -5241,12 +5241,12 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>Mlynské nivy, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Ševčenkova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>Viktória Rybáriková</t>
+          <t>Pavol Zlacký</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -5263,17 +5263,17 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>Bieloruská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Mlynské nivy, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>Veronika L</t>
+          <t>Viktória Rybáriková</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D219" s="4" t="inlineStr">
@@ -5285,17 +5285,17 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>Mickiewiczova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bieloruská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>Lubica Šuleková</t>
+          <t>Veronika L</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>Iný priestor</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D220" s="4" t="inlineStr">
@@ -5307,17 +5307,17 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>Závod, okres Malacky</t>
+          <t>Mickiewiczova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>Peter Peter</t>
+          <t>Lubica Šuleková</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Iný priestor</t>
         </is>
       </c>
       <c r="D221" s="4" t="inlineStr">
@@ -5329,17 +5329,17 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej 11A, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Závod, okres Malacky</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>David slnecnice</t>
+          <t>Peter Peter</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D222" s="4" t="inlineStr">
@@ -5351,17 +5351,17 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>Tureň, okres Senec</t>
+          <t>Zuzany Chalupovej 11A, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>Maroš Szighardt</t>
+          <t>David slnecnice</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D223" s="4" t="inlineStr">
@@ -5373,12 +5373,12 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>Hamuliakovo, okres Senec</t>
+          <t>Tureň, okres Senec</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>Peter Košút</t>
+          <t>Maroš Szighardt</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -5395,17 +5395,17 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
+          <t>Hamuliakovo, okres Senec</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>Jan L</t>
+          <t>Peter Košút</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D225" s="4" t="inlineStr">
@@ -5417,17 +5417,17 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>Eduarda Wenzla, Bratislava-Rača, okres Bratislava III</t>
+          <t>Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Miroslav O  </t>
+          <t>Jan L</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D226" s="4" t="inlineStr">
@@ -5439,12 +5439,12 @@
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>Bajkalská 9B, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Eduarda Wenzla, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>gianluca de vecchi</t>
+          <t xml:space="preserve">Miroslav O  </t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -5461,17 +5461,17 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>Dulovo námestie, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bajkalská 9B, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Martin Griga</t>
+          <t>gianluca de vecchi</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D228" s="4" t="inlineStr">
@@ -5483,17 +5483,17 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>Cyprichova, Bratislava-Rača, okres Bratislava III</t>
+          <t>Dulovo námestie, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Anton K</t>
+          <t>Martin Griga</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D229" s="4" t="inlineStr">
@@ -5505,17 +5505,17 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>Na varte, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Cyprichova, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Alexander Milly</t>
+          <t>Anton K</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D230" s="4" t="inlineStr">
@@ -5527,17 +5527,17 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>Malé Leváre, okres Malacky</t>
+          <t>Na varte, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Victoria Ivanová</t>
+          <t>Alexander Milly</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D231" s="4" t="inlineStr">
@@ -5549,17 +5549,17 @@
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>Nejedlého 20, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Malé Leváre, okres Malacky</t>
         </is>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Mojmír Gaško</t>
+          <t>Victoria Ivanová</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D232" s="4" t="inlineStr">
@@ -5571,17 +5571,17 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>Veltlínska, Svätý Jur, okres Pezinok</t>
+          <t>Nejedlého 20, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Jaroslav Š</t>
+          <t>Mojmír Gaško</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D233" s="4" t="inlineStr">
@@ -6957,7 +6957,7 @@
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>Kľak, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>obec Kľak, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B296" t="inlineStr">
@@ -8651,7 +8651,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10.10.2026 20:55</t>
+          <t>11.10.2026 11:38</t>
         </is>
       </c>
     </row>
@@ -8691,7 +8691,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="10">
@@ -8711,13 +8711,13 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>okres Bratislava I</t>
+          <t>okres Bratislava V</t>
         </is>
       </c>
       <c r="B12" t="n">
@@ -8727,11 +8727,11 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>okres Bratislava V</t>
+          <t>okres Bratislava I</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14">
@@ -8790,7 +8790,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21">
@@ -8800,7 +8800,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
     <row r="22">
@@ -8820,7 +8820,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="24">
@@ -8840,7 +8840,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="26">
@@ -8916,7 +8916,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Pozemok pre bytovú výstavbu</t>
+          <t>Záhradná chatka</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -8926,7 +8926,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Iný priestor</t>
+          <t>Pozemok pre bytovú výstavbu</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -8936,7 +8936,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Reštauračné priestory</t>
+          <t>Iný priestor</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -8946,7 +8946,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Zrub / chalupa</t>
+          <t>Reštauračné priestory</t>
         </is>
       </c>
       <c r="B36" t="n">
@@ -8956,17 +8956,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Orná pôda</t>
+          <t>Zrub / chalupa</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Záhradná chatka</t>
+          <t>Orná pôda</t>
         </is>
       </c>
       <c r="B38" t="n">

</xml_diff>

<commit_message>
Aktualizácia ponúk – 2026-10-17 09:27 UTC
</commit_message>
<xml_diff>
--- a/public/ponuky.xlsx
+++ b/public/ponuky.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Prehľad" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ponuky'!$A$1:$D$366</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Ponuky'!$A$1:$D$364</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -455,7 +455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D366"/>
+  <dimension ref="A1:D364"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -489,42 +489,42 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Pezinská, Senec, okres Senec</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Aneta Štefanovská</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Rodinný dom</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>otvoriť ponuku</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>Cesta na Kamzík, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>erik erik</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Cesta na Kamzík, Bratislava-Nové Mesto, okres Bratislava III</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>erik erik</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Rodinný dom</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -533,17 +533,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Šustekova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Cesta na Kamzík, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Martin Uher</t>
+          <t>erik erik</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -555,17 +555,17 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Ivanka pri Dunaji, okres Senec</t>
+          <t>Šustekova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Andrea Bášková</t>
+          <t>Martin Uher</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -577,12 +577,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Studienka 778, Studienka, okres Malacky</t>
+          <t>Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Peter J</t>
+          <t>Andrea Bášková</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -599,17 +599,17 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Studienka 778, Studienka, okres Malacky</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Jozef Hurny</t>
+          <t>Peter J</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Kancelárie</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -621,17 +621,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Záhradnícka, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Jozef Klimo</t>
+          <t>Jozef Hurny</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Kancelárie</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -643,17 +643,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Markova 3, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Záhradnícka, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Lukas Buna</t>
+          <t>Jozef Klimo</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -665,17 +665,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Šancová, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Markova 3, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Ondrej Fabrici</t>
+          <t>Lukas Buna</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -687,17 +687,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Petra Jilemnického, Malacky, okres Malacky</t>
+          <t>Šancová, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Adriana Gašparec</t>
+          <t>Ondrej Fabrici</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -709,12 +709,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Svetlá, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Petra Jilemnického, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Blanka Čorná</t>
+          <t>Adriana Gašparec</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -731,17 +731,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Metodova 6, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Svetlá, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Michal Komačka</t>
+          <t>Blanka Čorná</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Obchodné priestory</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -753,17 +753,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Tomislava P. Kolakoviča, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
+          <t>Metodova 6, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Peter Orlický</t>
+          <t>Michal Komačka</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Obchodné priestory</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -775,12 +775,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Grösslingova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Tomislava P. Kolakoviča, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Andrea Brejkova</t>
+          <t>Peter Orlický</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -797,17 +797,17 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej 18A, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Grösslingova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Martin Gyimesi</t>
+          <t>Andrea Brejkova</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -819,17 +819,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Černockého 9, Bratislava-Rača, okres Bratislava III</t>
+          <t>Zuzany Chalupovej 18A, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Marcel Blanárik</t>
+          <t>Martin Gyimesi</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -841,17 +841,17 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Pavla Horova, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
+          <t>Černockého 9, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Daniela Laurenčíková</t>
+          <t>Marcel Blanárik</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -863,17 +863,17 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Pavla Horova, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Veronika Kubovičová</t>
+          <t>Daniela Laurenčíková</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -885,42 +885,42 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>Bratislava-Dúbravka, okres Bratislava IV</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Veronika Kubovičová</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>4-izbový byt</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>otvoriť ponuku</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
           <t>Žabotova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Pavol Lazar</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Reštaurácia</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Špitálska, Bratislava-Staré Mesto, okres Bratislava I</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>Alexandra Horvathova</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>3-izbový byt</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="inlineStr">
+      <c r="D21" s="4" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -929,17 +929,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Uránová, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Špitálska, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Erik Varchol</t>
+          <t>Alexandra Horvathova</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -951,17 +951,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Landererova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Uránová, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Anton K</t>
+          <t>Erik Varchol</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
@@ -973,12 +973,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Segnerova, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Landererova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Marian Placko</t>
+          <t>Anton K</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -995,17 +995,17 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Segnerova, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Stanislav Blaško</t>
+          <t>Marian Placko</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -1017,17 +1017,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Andrej Oravec</t>
+          <t>Stanislav Blaško</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -1039,17 +1039,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Jánošíkova, Senec, okres Senec</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Attila Kulcsar</t>
+          <t>Andrej Oravec</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Pozemok pre bytovú výstavbu</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
@@ -1061,17 +1061,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Šancová, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Jánošíkova, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Tomas Gajdos</t>
+          <t>Attila Kulcsar</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre bytovú výstavbu</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
@@ -1083,12 +1083,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Jarabinková, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Šancová, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Alica Pongráczová</t>
+          <t>Tomas Gajdos</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1105,17 +1105,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Obilná, Bernolákovo, okres Senec</t>
+          <t>Jarabinková, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>petra wolfert</t>
+          <t>Alica Pongráczová</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -1127,17 +1127,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej 17, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Obilná, Bernolákovo, okres Senec</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Martin Krivosik</t>
+          <t>petra wolfert</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -1149,17 +1149,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Tupolevova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Zuzany Chalupovej 17, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>katarina uhrinova</t>
+          <t>Martin Krivosik</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -1171,17 +1171,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Hálova 12, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Tupolevova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>STEFAN MARTINKA</t>
+          <t>katarina uhrinova</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -1193,17 +1193,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Kasárenská 511, Záhorská Ves, okres Malacky</t>
+          <t>Hálova 12, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Lucia Blažeková</t>
+          <t>STEFAN MARTINKA</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -1215,17 +1215,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Nad Výhonom, Malacky, okres Malacky</t>
+          <t>Kasárenská 511, Záhorská Ves, okres Malacky</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Tibor Kováč</t>
+          <t>Lucia Blažeková</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Záhradná chatka</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -1565,22 +1565,22 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Frankovská, Bratislava-Nové Mesto, okres Bratislava III</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Michal Klempai</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>4-izbový byt</t>
-        </is>
-      </c>
-      <c r="D51" s="4" t="inlineStr">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>Cajlanská, Pezinok, okres Pezinok</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>Lenka Franova</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>Rodinný dom</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1589,17 +1589,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Nobelova 12C, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Frankovská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Radovan Hýbl</t>
+          <t>Michal Klempai</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -1611,17 +1611,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Na Grunte, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Nobelova 12C, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Katarina K</t>
+          <t>Radovan Hýbl</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -1633,12 +1633,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Pri Šajbách, Bratislava-Rača, okres Bratislava III</t>
+          <t>Na Grunte, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Andrea Peciarova</t>
+          <t>Katarina K</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1655,17 +1655,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Malacky, okres Malacky</t>
+          <t>Pri Šajbách, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Viliam Pavelka</t>
+          <t>Andrea Peciarova</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -1677,17 +1677,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Nábrežie arm. gen. Ludvíka Svobodu 20, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Marek  MV MV</t>
+          <t>Viliam Pavelka</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -1699,17 +1699,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Nábrežie arm. gen. Ludvíka Svobodu 20, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Martin Číž</t>
+          <t>Marek  MV MV</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -1721,17 +1721,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Jarabinková 2C, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Jozef Border</t>
+          <t>Martin Číž</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -1743,17 +1743,17 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Jarabinková 2C, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Martin Číž</t>
+          <t>Jozef Border</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -1765,17 +1765,17 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Blagoevova 16, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Marek Chudý</t>
+          <t>Martin Číž</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Double studio apartment</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -1787,17 +1787,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Pod Kopcami, Stupava, okres Malacky</t>
+          <t>Blagoevova 16, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Peter Glasa</t>
+          <t>Marek Chudý</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Double studio apartment</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
@@ -1809,17 +1809,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Plavecký Štvrtok, okres Malacky</t>
+          <t>Pod Kopcami, Stupava, okres Malacky</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Bianka Chmelová</t>
+          <t>Peter Glasa</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
@@ -1831,12 +1831,12 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Nechtíková ulica, Rovinka, okres Senec</t>
+          <t>Plavecký Štvrtok, okres Malacky</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Marcel Polák</t>
+          <t>Bianka Chmelová</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -1853,17 +1853,17 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Malacky, okres Malacky</t>
+          <t>Nechtíková ulica, Rovinka, okres Senec</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Lucia Blažeková</t>
+          <t>Marcel Polák</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
@@ -1875,7 +1875,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>497, Plavecký Štvrtok, okres Malacky</t>
+          <t>Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
@@ -1897,17 +1897,17 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Vysoká 9, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>497, Plavecký Štvrtok, okres Malacky</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Partner Technic</t>
+          <t>Lucia Blažeková</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
@@ -1919,17 +1919,17 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Ondavská, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Vysoká 9, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Jakub Peťko</t>
+          <t>Partner Technic</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
@@ -1941,17 +1941,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Jurigovo nám., Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Ondavská, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Roman Babiar</t>
+          <t>Jakub Peťko</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
@@ -1963,17 +1963,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Legerského 8, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Jurigovo nám., Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Michal Rajter</t>
+          <t>Roman Babiar</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
@@ -1985,17 +1985,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Podunajská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Legerského 8, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Martin Mašata</t>
+          <t>Michal Rajter</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Polyfunkčná budova</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
@@ -2007,17 +2007,17 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Kostolná pri Dunaji, okres Senec</t>
+          <t>Podunajská, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Michal P</t>
+          <t>Martin Mašata</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>Polyfunkčná budova</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
@@ -2029,17 +2029,17 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Šenkvice, okres Pezinok</t>
+          <t>Kostolná pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Marek Kakalik</t>
+          <t>Michal P</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Orná pôda</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
@@ -2051,17 +2051,17 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Galvaniho, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Šenkvice, okres Pezinok</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Kristína Mizeráková</t>
+          <t>Marek Kakalik</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Orná pôda</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
@@ -2073,17 +2073,17 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Za kostolom, Kostolište, okres Malacky</t>
+          <t>Galvaniho, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Ferdinand Havlík</t>
+          <t>Kristína Mizeráková</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
@@ -2095,17 +2095,17 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Kyjevská 2, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Za kostolom, Kostolište, okres Malacky</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Monika Faltinová</t>
+          <t>Ferdinand Havlík</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
@@ -2117,17 +2117,17 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Kyjevská 2, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Iveta Škubová</t>
+          <t>Monika Faltinová</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
@@ -2139,17 +2139,17 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Mečíková 5823, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
+          <t>Zuzany Chalupovej, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Jana Varga Bitova</t>
+          <t>Iveta Škubová</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
@@ -2161,17 +2161,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Mečíková 5823, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Jan Plch</t>
+          <t>Jana Varga Bitova</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
@@ -2183,17 +2183,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Zuzana Vlková</t>
+          <t>Jan Plch</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
@@ -2205,17 +2205,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Horská, Bratislava-Rača, okres Bratislava III</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Peter Széll</t>
+          <t>Zuzana Vlková</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Iný priestor</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
@@ -2227,17 +2227,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Palisády, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Horská, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Alexandra Litecka</t>
+          <t>Peter Széll</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>5+ izbový byt</t>
+          <t>Iný priestor</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
@@ -2249,17 +2249,17 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Černyševského, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Palisády, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Vladimir Jagr</t>
+          <t>Alexandra Litecka</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>5+ izbový byt</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
@@ -2271,17 +2271,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Žabí majer, Bratislava-Rača, okres Bratislava III</t>
+          <t>Černyševského, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Lydia Hentekova</t>
+          <t>Vladimir Jagr</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Záhrada</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
@@ -2293,17 +2293,17 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Smikova, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Žabí majer, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Kamil Vrabeľ</t>
+          <t>Lydia Hentekova</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Záhrada</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
@@ -2315,12 +2315,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Šancová 74, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Smikova, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Juraj Jediný</t>
+          <t>Kamil Vrabeľ</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -2337,17 +2337,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Somolického 6, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Šancová 74, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Viktória Peniaková</t>
+          <t>Juraj Jediný</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
@@ -2359,17 +2359,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Somolického 6, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>R K</t>
+          <t>Viktória Peniaková</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
@@ -2381,17 +2381,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Zuzana Vreckova</t>
+          <t>R K</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
@@ -2403,17 +2403,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>14050, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Dominika Bachrata</t>
+          <t>Zuzana Vreckova</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
@@ -2425,17 +2425,17 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>14050, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Zuzana Vreckova</t>
+          <t>Dominika Bachrata</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
@@ -2447,17 +2447,17 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Harmónia, Modra, okres Pezinok</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Silvia Papugová</t>
+          <t>Zuzana Vreckova</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
@@ -2469,17 +2469,17 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Štefánikova 82, Modra, okres Pezinok</t>
+          <t>Harmónia, Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Peter Juran</t>
+          <t>Silvia Papugová</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
@@ -2491,17 +2491,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Gregorovej, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Štefánikova 82, Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Dadka Kesjar</t>
+          <t>Peter Juran</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
@@ -2513,17 +2513,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Most pri Bratislave, okres Senec</t>
+          <t>Gregorovej, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Zahrada Most</t>
+          <t>Dadka Kesjar</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Záhradná chatka</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
@@ -2535,17 +2535,17 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>521, Borinka, okres Malacky</t>
+          <t>Most pri Bratislave, okres Senec</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Miroslav Hollý</t>
+          <t>Zahrada Most</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Záhradná chatka</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
@@ -2557,17 +2557,17 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>521, Borinka, okres Malacky</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Dagmar Semrisová</t>
+          <t>Miroslav Hollý</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
@@ -2579,17 +2579,17 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Most pri Bratislave, okres Senec</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Milan M</t>
+          <t>Dagmar Semrisová</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
@@ -2601,17 +2601,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Táborská 10, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Most pri Bratislave, okres Senec</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>vladimir cagan</t>
+          <t>Milan M</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
@@ -2623,17 +2623,17 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Hany Meličkovej, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Táborská 10, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Artur Y</t>
+          <t>vladimir cagan</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Obchodné priestory</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
@@ -2645,17 +2645,17 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Hany Meličkovej, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Peter Peter</t>
+          <t>Artur Y</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Obchodné priestory</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
@@ -2667,17 +2667,17 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Most pri Bratislave, okres Senec</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Maryna Rieznykova</t>
+          <t>Peter Peter</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
@@ -2689,17 +2689,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Ondrejovova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Most pri Bratislave, okres Senec</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Martin Fried</t>
+          <t>Maryna Rieznykova</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
@@ -2711,17 +2711,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Ondrejovova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Tomáš Lehocký</t>
+          <t>Martin Fried</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
@@ -2733,17 +2733,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Uzbecká, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Mária Mériová</t>
+          <t>Tomáš Lehocký</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Other type of apartment</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
@@ -2755,17 +2755,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Landererova 6, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Uzbecká, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Mat Nav</t>
+          <t>Mária Mériová</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Other type of apartment</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
@@ -2777,17 +2777,17 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Mierová 200, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Landererova 6, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Richard Velky</t>
+          <t>Mat Nav</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Pozemok pre bytovú výstavbu</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
@@ -2799,17 +2799,17 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Mierová 200, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Dominika Ševčíková</t>
+          <t>Richard Velky</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre bytovú výstavbu</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
@@ -2821,17 +2821,17 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Nad Vinohradmi, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
+          <t>Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Yury Makarov</t>
+          <t>Dominika Ševčíková</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
@@ -2843,17 +2843,17 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Vajnorská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Nad Vinohradmi, Bratislava-Devínska Nová Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Peter Smiček</t>
+          <t>Yury Makarov</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
@@ -2865,17 +2865,17 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Cyprichova 40, Bratislava-Rača, okres Bratislava III</t>
+          <t>Vajnorská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Tomáš Samuhel</t>
+          <t>Peter Smiček</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
@@ -2887,17 +2887,17 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Miletičova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Cyprichova 40, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Tomas L</t>
+          <t>Tomáš Samuhel</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
@@ -2909,17 +2909,17 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Bebravská, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Miletičova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARZE MARZE </t>
+          <t>Tomas L</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Garsónka</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
@@ -2931,17 +2931,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Devínska cesta, Bratislava-Devín, okres Bratislava IV</t>
+          <t>Bebravská, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Jana Filípková</t>
+          <t xml:space="preserve">MARZE MARZE </t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Záhrada</t>
+          <t>Garsónka</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
@@ -2953,17 +2953,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Albrechtova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Devínska cesta, Bratislava-Devín, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t xml:space="preserve">MARZE MARZE </t>
+          <t>Jana Filípková</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Záhrada</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
@@ -2975,17 +2975,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Malé Vinice, Chorvátsky Grob, okres Senec</t>
+          <t>Albrechtova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Eva Husarová</t>
+          <t xml:space="preserve">MARZE MARZE </t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
@@ -2997,17 +2997,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Arménska, Bratislava-Vrakuňa, okres Bratislava II</t>
+          <t>Malé Vinice, Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>BYT ARMÉNSKA</t>
+          <t>Eva Husarová</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
@@ -3019,17 +3019,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Košická, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Arménska, Bratislava-Vrakuňa, okres Bratislava II</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Filip Jandura</t>
+          <t>BYT ARMÉNSKA</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
@@ -3041,17 +3041,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Domkárska, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Košická, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Peter Baláž</t>
+          <t>Filip Jandura</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
@@ -3063,17 +3063,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Riazanská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Domkárska, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Marián Petráš</t>
+          <t>Peter Baláž</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
@@ -3085,17 +3085,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Burgundská, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Riazanská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>IGS real Ivan</t>
+          <t>Marián Petráš</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
@@ -3107,17 +3107,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Štúrova, Marianka, okres Malacky</t>
+          <t>Burgundská, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>borisfkovac Kovac</t>
+          <t>IGS real Ivan</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
@@ -3129,17 +3129,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Školská, Chorvátsky Grob, okres Senec</t>
+          <t>Štúrova, Marianka, okres Malacky</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Denis Zamocky</t>
+          <t>borisfkovac Kovac</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D122" s="4" t="inlineStr">
@@ -3151,17 +3151,17 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Mlynské nivy 57, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Školská, Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Stefan Niznik</t>
+          <t>Denis Zamocky</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D123" s="4" t="inlineStr">
@@ -3173,12 +3173,12 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Drobného, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Mlynské nivy 57, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Gabriela Cermakova</t>
+          <t>Stefan Niznik</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -3195,12 +3195,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Miletičova 35, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Drobného, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Lubo Lajos</t>
+          <t>Gabriela Cermakova</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -3217,12 +3217,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Ulica Svornosti, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Miletičova 35, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Marek Bacik</t>
+          <t>Lubo Lajos</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -3239,17 +3239,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Jungmannova, Bratislava-Petržalka, okres Bratislava V</t>
+          <t>Ulica Svornosti, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Vaso Bratislava</t>
+          <t>Marek Bacik</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
@@ -3261,17 +3261,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Brusnicová 13, Chorvátsky Grob, okres Senec</t>
+          <t>Jungmannova, Bratislava-Petržalka, okres Bratislava V</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Dušan Pokoš</t>
+          <t>Vaso Bratislava</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D128" s="4" t="inlineStr">
@@ -3283,17 +3283,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Vlčie hrdlo 85, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Brusnicová 13, Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Natalia Kubicova</t>
+          <t>Dušan Pokoš</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
@@ -3305,12 +3305,12 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Hrachová 16C, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Vlčie hrdlo 85, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Dušan Pokoš</t>
+          <t>Natalia Kubicova</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -3327,17 +3327,17 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Planét, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Hrachová 16C, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Július S</t>
+          <t>Dušan Pokoš</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
@@ -3349,12 +3349,12 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Skalná, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Planét, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>katarina sekerka</t>
+          <t>Július S</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -3371,17 +3371,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Heyrovského, Bratislava-Lamač, okres Bratislava IV</t>
+          <t>Skalná, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Maros Palik</t>
+          <t>katarina sekerka</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
@@ -3393,17 +3393,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Oravská 2, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Heyrovského, Bratislava-Lamač, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Zdena Bartošová</t>
+          <t>Maros Palik</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D134" s="4" t="inlineStr">
@@ -3415,17 +3415,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Jarabinková 2, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Oravská 2, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Eva Franzen</t>
+          <t>Zdena Bartošová</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
@@ -3437,17 +3437,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Miletičova 60, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Jarabinková 2, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Michael Kollár</t>
+          <t>Eva Franzen</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D136" s="4" t="inlineStr">
@@ -3459,17 +3459,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Chorvátsky Grob, okres Senec</t>
+          <t>Miletičova 60, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Dada Garajova</t>
+          <t>Michael Kollár</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D137" s="4" t="inlineStr">
@@ -3481,12 +3481,12 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Senec, okres Senec</t>
+          <t>Chorvátsky Grob, okres Senec</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Jakub Králik</t>
+          <t>Dada Garajova</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -3503,17 +3503,17 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Holubia, Senec, okres Senec</t>
+          <t>Senec, okres Senec</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>Marko Klúčik</t>
+          <t>Jakub Králik</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D139" s="4" t="inlineStr">
@@ -3525,12 +3525,12 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Jelačičova, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Holubia, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>Lara Kristi</t>
+          <t>Marko Klúčik</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -3547,17 +3547,17 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>1mája, Pezinok, okres Pezinok</t>
+          <t>Jelačičova, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>Ladislav Ružek</t>
+          <t>Lara Kristi</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Samostatná garáž</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D141" s="4" t="inlineStr">
@@ -3569,17 +3569,17 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Okružná 47, Senec, okres Senec</t>
+          <t>1mája, Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>Roman Gazdik</t>
+          <t>Ladislav Ružek</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Samostatná garáž</t>
         </is>
       </c>
       <c r="D142" s="4" t="inlineStr">
@@ -3591,17 +3591,17 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Kozia, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Okružná 47, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>Ľubor Mendel</t>
+          <t>Roman Gazdik</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D143" s="4" t="inlineStr">
@@ -3613,17 +3613,17 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Šalviová, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Kozia, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Juraj Valašťan</t>
+          <t>Ľubor Mendel</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D144" s="4" t="inlineStr">
@@ -3635,17 +3635,17 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Rovinka, okres Senec</t>
+          <t>Šalviová, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>Miroslav Vancik</t>
+          <t>Juraj Valašťan</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D145" s="4" t="inlineStr">
@@ -3657,17 +3657,17 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Agátová, Ivanka pri Dunaji, okres Senec</t>
+          <t>Rovinka, okres Senec</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Viktória Krupová</t>
+          <t>Miroslav Vancik</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D146" s="4" t="inlineStr">
@@ -3679,17 +3679,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Kaplinská 7, Bratislava-Rača, okres Bratislava III</t>
+          <t>Agátová, Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Eva Žíhlavníková</t>
+          <t>Viktória Krupová</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D147" s="4" t="inlineStr">
@@ -3701,17 +3701,17 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Kaplinská 7, Bratislava-Rača, okres Bratislava III</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Alexander Kernaševič</t>
+          <t>Eva Žíhlavníková</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Mobile cells and stands</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D148" s="4" t="inlineStr">
@@ -3723,17 +3723,17 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Landererova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Simona Kourdi</t>
+          <t>Alexander Kernaševič</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Mobile cells and stands</t>
         </is>
       </c>
       <c r="D149" s="4" t="inlineStr">
@@ -3745,17 +3745,17 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>167, Borinka, okres Malacky</t>
+          <t>Landererova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Kamil Semeš</t>
+          <t>Simona Kourdi</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Chata / rekreačný dom</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D150" s="4" t="inlineStr">
@@ -3767,17 +3767,17 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Gregorovej, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>167, Borinka, okres Malacky</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Andrej Miko</t>
+          <t>Kamil Semeš</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Chata / rekreačný dom</t>
         </is>
       </c>
       <c r="D151" s="4" t="inlineStr">
@@ -3789,17 +3789,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Jablonec, okres Pezinok</t>
+          <t>Gregorovej, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Andrea Valentová</t>
+          <t>Andrej Miko</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Pozemok pre rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D152" s="4" t="inlineStr">
@@ -3811,17 +3811,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Ivanka pri Dunaji, okres Senec</t>
+          <t>Jablonec, okres Pezinok</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Andrea Bášková</t>
+          <t>Andrea Valentová</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D153" s="4" t="inlineStr">
@@ -3833,12 +3833,12 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Ivanka pri Dunaji, okres Senec</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Katarína Rusňáková</t>
+          <t>Andrea Bášková</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -3855,12 +3855,12 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Ulica 8. mája 22A, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Vladimír Mitrík</t>
+          <t>Katarína Rusňáková</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -3877,17 +3877,17 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Partizánska 1081, Malacky, okres Malacky</t>
+          <t>Ulica 8. mája 22A, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Peter Ondrovič</t>
+          <t>Vladimír Mitrík</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D156" s="4" t="inlineStr">
@@ -3899,12 +3899,12 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Čulenova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Partizánska 1081, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>M I</t>
+          <t>Peter Ondrovič</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -3921,17 +3921,17 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Drobného, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Čulenova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Peter Chovanec</t>
+          <t>M I</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D158" s="4" t="inlineStr">
@@ -3943,17 +3943,17 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Vysoká pri Morave, okres Malacky</t>
+          <t>Drobného, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Miroslav Vojkovic</t>
+          <t>Peter Chovanec</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D159" s="4" t="inlineStr">
@@ -3965,12 +3965,12 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Vinárska, Modra, okres Pezinok</t>
+          <t>Vysoká pri Morave, okres Malacky</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>marek rozic</t>
+          <t>Miroslav Vojkovic</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -3987,17 +3987,17 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Bratislava-Rača, okres Bratislava III</t>
+          <t>Vinárska, Modra, okres Pezinok</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Anton K</t>
+          <t>marek rozic</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D161" s="4" t="inlineStr">
@@ -7925,12 +7925,12 @@
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>Slnečné jazerá, Senec, okres Senec</t>
+          <t>Avanárska, Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t>Filip Lečko</t>
+          <t>Julius Bohunsky</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -7947,17 +7947,17 @@
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>Avanárska, Rohožník, okres Malacky</t>
+          <t>Dlhé diely, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t>Julius Bohunsky</t>
+          <t>Matusk Tomas</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D341" s="4" t="inlineStr">
@@ -7969,17 +7969,17 @@
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>Dlhé diely, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Jozefa Kubinu, Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>Matusk Tomas</t>
+          <t>Martina Hlubocká</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D342" s="4" t="inlineStr">
@@ -7991,17 +7991,17 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>Jozefa Kubinu, Malacky, okres Malacky</t>
+          <t>Steinov dvor, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t>Martina Hlubocká</t>
+          <t>Ing Šalátová Zuzana</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D343" s="4" t="inlineStr">
@@ -8013,17 +8013,17 @@
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>Steinov dvor, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Svätý Martin, Senec, okres Senec</t>
         </is>
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t>Ing Šalátová Zuzana</t>
+          <t>Stanislav Sakac</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D344" s="4" t="inlineStr">
@@ -8035,17 +8035,17 @@
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>Svätý Martin, Senec, okres Senec</t>
+          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t>Stanislav Sakac</t>
+          <t>Sandra zahradnikova</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D345" s="4" t="inlineStr">
@@ -8057,17 +8057,17 @@
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Žižkova, Bratislava-Staré Mesto, okres Bratislava I</t>
         </is>
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t>Sandra zahradnikova</t>
+          <t>Denisa Slančová</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D346" s="4" t="inlineStr">
@@ -8079,17 +8079,17 @@
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>Žižkova, Bratislava-Staré Mesto, okres Bratislava I</t>
+          <t>Strmý vŕšok 164, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t>Denisa Slančová</t>
+          <t>Tereza Adámyová</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D347" s="4" t="inlineStr">
@@ -8101,17 +8101,17 @@
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>Strmý vŕšok 164, Bratislava-Záhorská Bystrica, okres Bratislava IV</t>
+          <t>Lackova, Bratislava-Karlova Ves, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t>Tereza Adámyová</t>
+          <t>Predaj Bytu</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D348" s="4" t="inlineStr">
@@ -8123,17 +8123,17 @@
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>Lackova, Bratislava-Karlova Ves, okres Bratislava IV</t>
+          <t>Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t>Predaj Bytu</t>
+          <t>Tatiana B</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D349" s="4" t="inlineStr">
@@ -8145,17 +8145,17 @@
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>Rohožník, okres Malacky</t>
+          <t>Máchova, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t>Tatiana B</t>
+          <t>Marian V</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D350" s="4" t="inlineStr">
@@ -8167,12 +8167,12 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>Nevädzová 6, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Makovického, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t>Daniel l</t>
+          <t>Predaj Nehnutelosti</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -8189,17 +8189,17 @@
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>Máchova, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
+          <t>Čsl. parašutistov, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t>Marian V</t>
+          <t>Tomáš Tóth</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>1-izbový byt</t>
         </is>
       </c>
       <c r="D352" s="4" t="inlineStr">
@@ -8211,17 +8211,17 @@
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>Makovického, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Račianska 64, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t>Predaj Nehnutelosti</t>
+          <t>Roman Miškulynets</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D353" s="4" t="inlineStr">
@@ -8233,17 +8233,17 @@
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>Čsl. parašutistov, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Suchý vrch, Limbach, okres Pezinok</t>
         </is>
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t>Tomáš Tóth</t>
+          <t>Miloslav Moravec</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
         <is>
-          <t>1-izbový byt</t>
+          <t>Zrub / chalupa</t>
         </is>
       </c>
       <c r="D354" s="4" t="inlineStr">
@@ -8255,17 +8255,17 @@
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>Račianska 64, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Ružová dolina 16, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t>Roman Miškulynets</t>
+          <t>Ľuboš Ľahký</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D355" s="4" t="inlineStr">
@@ -8277,17 +8277,17 @@
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>Suchý vrch, Limbach, okres Pezinok</t>
+          <t>Nejedlého 3394, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t>Miloslav Moravec</t>
+          <t>Vladimír Žiga</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
         <is>
-          <t>Zrub / chalupa</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D356" s="4" t="inlineStr">
@@ -8299,17 +8299,17 @@
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>Ružová dolina 16, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Limbašská cesta, Pezinok, okres Pezinok</t>
         </is>
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t>Ľuboš Ľahký</t>
+          <t>Ganna Naichuk</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>2-izbový byt</t>
         </is>
       </c>
       <c r="D357" s="4" t="inlineStr">
@@ -8321,17 +8321,17 @@
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>Nejedlého 3394, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Kristy Bendovej, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t>Vladimír Žiga</t>
+          <t>Jana Gottstein</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>4-izbový byt</t>
         </is>
       </c>
       <c r="D358" s="4" t="inlineStr">
@@ -8343,17 +8343,17 @@
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>Limbašská cesta, Pezinok, okres Pezinok</t>
+          <t>Pod vŕškom, Stupava, okres Malacky</t>
         </is>
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t>Ganna Naichuk</t>
+          <t>Lenka Višňovská</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
         <is>
-          <t>2-izbový byt</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D359" s="4" t="inlineStr">
@@ -8365,17 +8365,17 @@
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>Kristy Bendovej, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Galbavého 1, Bratislava-Dúbravka, okres Bratislava IV</t>
         </is>
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t>Jana Gottstein</t>
+          <t>Denisa Lukačovičová</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
         <is>
-          <t>4-izbový byt</t>
+          <t>Obchodné priestory</t>
         </is>
       </c>
       <c r="D360" s="4" t="inlineStr">
@@ -8387,17 +8387,17 @@
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>Pod vŕškom, Stupava, okres Malacky</t>
+          <t>Stromová 25, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t>Lenka Višňovská</t>
+          <t>Michal Rusek</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
         <is>
-          <t>Rodinný dom</t>
+          <t>3-izbový byt</t>
         </is>
       </c>
       <c r="D361" s="4" t="inlineStr">
@@ -8409,17 +8409,17 @@
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>Galbavého 1, Bratislava-Dúbravka, okres Bratislava IV</t>
+          <t>Chatová rekreačná oblasť, Rohožník, okres Malacky</t>
         </is>
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t>Denisa Lukačovičová</t>
+          <t>M J</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
         <is>
-          <t>Obchodné priestory</t>
+          <t>Zrub / chalupa</t>
         </is>
       </c>
       <c r="D362" s="4" t="inlineStr">
@@ -8431,17 +8431,17 @@
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>Stromová 25, Bratislava-Nové Mesto, okres Bratislava III</t>
+          <t>Malacky, okres Malacky</t>
         </is>
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t>Michal Rusek</t>
+          <t>Pán Budkovsky</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
         <is>
-          <t>3-izbový byt</t>
+          <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
       <c r="D363" s="4" t="inlineStr">
@@ -8453,17 +8453,17 @@
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>Chatová rekreačná oblasť, Rohožník, okres Malacky</t>
+          <t>Máchova, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
         </is>
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t>M J</t>
+          <t xml:space="preserve">Andrea  Majchráková </t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
         <is>
-          <t>Zrub / chalupa</t>
+          <t>Rodinný dom</t>
         </is>
       </c>
       <c r="D364" s="4" t="inlineStr">
@@ -8472,52 +8472,8 @@
         </is>
       </c>
     </row>
-    <row r="365">
-      <c r="A365" t="inlineStr">
-        <is>
-          <t>Malacky, okres Malacky</t>
-        </is>
-      </c>
-      <c r="B365" t="inlineStr">
-        <is>
-          <t>Pán Budkovsky</t>
-        </is>
-      </c>
-      <c r="C365" t="inlineStr">
-        <is>
-          <t>Pozemok pre rodinný dom</t>
-        </is>
-      </c>
-      <c r="D365" s="4" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
-    <row r="366">
-      <c r="A366" t="inlineStr">
-        <is>
-          <t>Máchova, Bratislava-Podunajské Biskupice, okres Bratislava II</t>
-        </is>
-      </c>
-      <c r="B366" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Andrea  Majchráková </t>
-        </is>
-      </c>
-      <c r="C366" t="inlineStr">
-        <is>
-          <t>Rodinný dom</t>
-        </is>
-      </c>
-      <c r="D366" s="4" t="inlineStr">
-        <is>
-          <t>otvoriť ponuku</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D366"/>
+  <autoFilter ref="A1:D364"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -8882,8 +8838,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D362" r:id="rId361"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D363" r:id="rId362"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D364" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D365" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D366" r:id="rId365"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8916,7 +8870,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>365</v>
+        <v>363</v>
       </c>
     </row>
     <row r="4">
@@ -8927,7 +8881,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>16.10.2026 20:10</t>
+          <t>17.10.2026 09:27</t>
         </is>
       </c>
     </row>
@@ -8957,7 +8911,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9">
@@ -8967,7 +8921,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10">
@@ -9017,7 +8971,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15">
@@ -9027,7 +8981,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="17">
@@ -9056,7 +9010,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20">
@@ -9066,7 +9020,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="21">
@@ -9076,7 +9030,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="22">
@@ -9172,7 +9126,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Záhradná chatka</t>
+          <t>Iný priestor</t>
         </is>
       </c>
       <c r="B31" t="n">
@@ -9182,17 +9136,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Iný priestor</t>
+          <t>Kancelárie</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Kancelárie</t>
+          <t>Double studio apartment</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -9202,7 +9156,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Double studio apartment</t>
+          <t>Polyfunkčná budova</t>
         </is>
       </c>
       <c r="B34" t="n">
@@ -9212,7 +9166,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Polyfunkčná budova</t>
+          <t>5+ izbový byt</t>
         </is>
       </c>
       <c r="B35" t="n">
@@ -9222,7 +9176,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>5+ izbový byt</t>
+          <t>Záhradná chatka</t>
         </is>
       </c>
       <c r="B36" t="n">

</xml_diff>

<commit_message>
Aktualizácia ponúk – 2026-10-23 20:37 UTC
</commit_message>
<xml_diff>
--- a/public/ponuky.xlsx
+++ b/public/ponuky.xlsx
@@ -49,7 +49,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
@@ -59,11 +59,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="0012263F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00E8F5EE"/>
       </patternFill>
     </fill>
   </fills>
@@ -79,13 +74,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -487,88 +480,88 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>Tomášikova 50, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Peter Valentovič</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Iný pozemok</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>Nezábudková 52, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>radovan reis</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>Pod Vtáčnikom, Bratislava-Nové Mesto, okres Bratislava III</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>Henrich Mauritz</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>Malacky, okres Malacky</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Martina Hulmanova</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D5" s="3" t="inlineStr">
+      <c r="D5" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -590,7 +583,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -612,7 +605,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -634,7 +627,7 @@
           <t>Samostatná garáž</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -656,7 +649,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D9" s="4" t="inlineStr">
+      <c r="D9" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -678,7 +671,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D10" s="4" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -700,7 +693,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D11" s="4" t="inlineStr">
+      <c r="D11" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -722,7 +715,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D12" s="4" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -744,7 +737,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D13" s="4" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -766,7 +759,7 @@
           <t>Samostatná garáž</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -788,7 +781,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D15" s="4" t="inlineStr">
+      <c r="D15" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -810,7 +803,7 @@
           <t>Samostatná garáž</t>
         </is>
       </c>
-      <c r="D16" s="4" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -832,7 +825,7 @@
           <t>Samostatná garáž</t>
         </is>
       </c>
-      <c r="D17" s="4" t="inlineStr">
+      <c r="D17" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -854,7 +847,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D18" s="4" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -876,7 +869,7 @@
           <t>Garsónka</t>
         </is>
       </c>
-      <c r="D19" s="4" t="inlineStr">
+      <c r="D19" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -898,7 +891,7 @@
           <t>Samostatná garáž</t>
         </is>
       </c>
-      <c r="D20" s="4" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -920,7 +913,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D21" s="4" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -942,7 +935,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D22" s="4" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -964,7 +957,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D23" s="4" t="inlineStr">
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -986,7 +979,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D24" s="4" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1008,7 +1001,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D25" s="4" t="inlineStr">
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1030,7 +1023,7 @@
           <t>Orná pôda</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1052,7 +1045,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1074,7 +1067,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1096,7 +1089,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D29" s="4" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1118,7 +1111,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1140,7 +1133,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D31" s="4" t="inlineStr">
+      <c r="D31" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1162,7 +1155,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D32" s="4" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1184,7 +1177,7 @@
           <t>Zrub / chalupa</t>
         </is>
       </c>
-      <c r="D33" s="4" t="inlineStr">
+      <c r="D33" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1206,7 +1199,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D34" s="4" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1228,7 +1221,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D35" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1250,7 +1243,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D36" s="4" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1272,7 +1265,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D37" s="4" t="inlineStr">
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1294,7 +1287,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D38" s="4" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1316,7 +1309,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D39" s="4" t="inlineStr">
+      <c r="D39" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1338,7 +1331,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D40" s="4" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1360,7 +1353,7 @@
           <t>Samostatná garáž</t>
         </is>
       </c>
-      <c r="D41" s="4" t="inlineStr">
+      <c r="D41" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1382,7 +1375,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D42" s="4" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1404,7 +1397,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D43" s="4" t="inlineStr">
+      <c r="D43" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1426,7 +1419,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D44" s="4" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1448,7 +1441,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D45" s="4" t="inlineStr">
+      <c r="D45" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1470,7 +1463,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D46" s="4" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1492,7 +1485,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D47" s="4" t="inlineStr">
+      <c r="D47" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1514,7 +1507,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1536,7 +1529,7 @@
           <t>Záhradná chatka</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="D49" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1558,7 +1551,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1580,7 +1573,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D51" s="4" t="inlineStr">
+      <c r="D51" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1602,7 +1595,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D52" s="4" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1624,7 +1617,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D53" s="4" t="inlineStr">
+      <c r="D53" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1646,7 +1639,7 @@
           <t>Chata / rekreačný dom</t>
         </is>
       </c>
-      <c r="D54" s="4" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1668,7 +1661,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D55" s="4" t="inlineStr">
+      <c r="D55" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1690,7 +1683,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D56" s="4" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1712,7 +1705,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D57" s="4" t="inlineStr">
+      <c r="D57" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1734,7 +1727,7 @@
           <t>Samostatná garáž</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1756,7 +1749,7 @@
           <t>Orná pôda</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr">
+      <c r="D59" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1778,7 +1771,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr">
+      <c r="D60" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1800,7 +1793,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D61" s="4" t="inlineStr">
+      <c r="D61" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1822,7 +1815,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D62" s="4" t="inlineStr">
+      <c r="D62" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1844,7 +1837,7 @@
           <t>Garsónka</t>
         </is>
       </c>
-      <c r="D63" s="4" t="inlineStr">
+      <c r="D63" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1866,7 +1859,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D64" s="4" t="inlineStr">
+      <c r="D64" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1888,7 +1881,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D65" s="4" t="inlineStr">
+      <c r="D65" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1910,7 +1903,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D66" s="4" t="inlineStr">
+      <c r="D66" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1932,7 +1925,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D67" s="4" t="inlineStr">
+      <c r="D67" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1954,7 +1947,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D68" s="4" t="inlineStr">
+      <c r="D68" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1976,7 +1969,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D69" s="4" t="inlineStr">
+      <c r="D69" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -1998,7 +1991,7 @@
           <t>Zmiešaná zóna</t>
         </is>
       </c>
-      <c r="D70" s="4" t="inlineStr">
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2020,7 +2013,7 @@
           <t>Samostatná garáž</t>
         </is>
       </c>
-      <c r="D71" s="4" t="inlineStr">
+      <c r="D71" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2042,7 +2035,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D72" s="4" t="inlineStr">
+      <c r="D72" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2064,7 +2057,7 @@
           <t>Zrub / chalupa</t>
         </is>
       </c>
-      <c r="D73" s="4" t="inlineStr">
+      <c r="D73" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2086,7 +2079,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D74" s="4" t="inlineStr">
+      <c r="D74" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2108,7 +2101,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D75" s="4" t="inlineStr">
+      <c r="D75" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2130,7 +2123,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D76" s="4" t="inlineStr">
+      <c r="D76" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2152,7 +2145,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D77" s="4" t="inlineStr">
+      <c r="D77" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2174,7 +2167,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D78" s="4" t="inlineStr">
+      <c r="D78" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2196,7 +2189,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D79" s="4" t="inlineStr">
+      <c r="D79" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2218,7 +2211,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D80" s="4" t="inlineStr">
+      <c r="D80" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2240,7 +2233,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D81" s="4" t="inlineStr">
+      <c r="D81" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2262,7 +2255,7 @@
           <t>Kancelárie</t>
         </is>
       </c>
-      <c r="D82" s="4" t="inlineStr">
+      <c r="D82" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2271,7 +2264,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Záhradnícka, Bratislava-Ružinov, okres Bratislava II</t>
+          <t>Záhradnícka 53, Bratislava-Ružinov, okres Bratislava II</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2284,7 +2277,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D83" s="4" t="inlineStr">
+      <c r="D83" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2306,7 +2299,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D84" s="4" t="inlineStr">
+      <c r="D84" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2328,7 +2321,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D85" s="4" t="inlineStr">
+      <c r="D85" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2350,7 +2343,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D86" s="4" t="inlineStr">
+      <c r="D86" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2372,7 +2365,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D87" s="4" t="inlineStr">
+      <c r="D87" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2394,7 +2387,7 @@
           <t>Obchodné priestory</t>
         </is>
       </c>
-      <c r="D88" s="4" t="inlineStr">
+      <c r="D88" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2416,7 +2409,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D89" s="4" t="inlineStr">
+      <c r="D89" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2438,7 +2431,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D90" s="4" t="inlineStr">
+      <c r="D90" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2460,7 +2453,7 @@
           <t>Samostatná garáž</t>
         </is>
       </c>
-      <c r="D91" s="4" t="inlineStr">
+      <c r="D91" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2482,7 +2475,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D92" s="4" t="inlineStr">
+      <c r="D92" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2504,7 +2497,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D93" s="4" t="inlineStr">
+      <c r="D93" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2526,7 +2519,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D94" s="4" t="inlineStr">
+      <c r="D94" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2548,7 +2541,7 @@
           <t>Reštaurácia</t>
         </is>
       </c>
-      <c r="D95" s="4" t="inlineStr">
+      <c r="D95" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2570,7 +2563,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D96" s="4" t="inlineStr">
+      <c r="D96" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2592,7 +2585,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D97" s="4" t="inlineStr">
+      <c r="D97" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2614,7 +2607,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D98" s="4" t="inlineStr">
+      <c r="D98" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2636,7 +2629,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D99" s="4" t="inlineStr">
+      <c r="D99" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2658,7 +2651,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D100" s="4" t="inlineStr">
+      <c r="D100" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2680,7 +2673,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D101" s="4" t="inlineStr">
+      <c r="D101" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2702,7 +2695,7 @@
           <t>Samostatná garáž</t>
         </is>
       </c>
-      <c r="D102" s="4" t="inlineStr">
+      <c r="D102" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2724,7 +2717,7 @@
           <t>Pozemok pre bytovú výstavbu</t>
         </is>
       </c>
-      <c r="D103" s="4" t="inlineStr">
+      <c r="D103" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2746,7 +2739,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D104" s="4" t="inlineStr">
+      <c r="D104" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2768,7 +2761,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D105" s="4" t="inlineStr">
+      <c r="D105" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2790,7 +2783,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D106" s="4" t="inlineStr">
+      <c r="D106" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2812,7 +2805,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D107" s="4" t="inlineStr">
+      <c r="D107" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2834,7 +2827,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D108" s="4" t="inlineStr">
+      <c r="D108" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2856,7 +2849,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D109" s="4" t="inlineStr">
+      <c r="D109" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2878,7 +2871,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D110" s="4" t="inlineStr">
+      <c r="D110" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2900,7 +2893,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D111" s="4" t="inlineStr">
+      <c r="D111" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2922,7 +2915,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D112" s="4" t="inlineStr">
+      <c r="D112" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2944,7 +2937,7 @@
           <t>Garsónka</t>
         </is>
       </c>
-      <c r="D113" s="4" t="inlineStr">
+      <c r="D113" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2966,7 +2959,7 @@
           <t>Garsónka</t>
         </is>
       </c>
-      <c r="D114" s="4" t="inlineStr">
+      <c r="D114" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -2988,7 +2981,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D115" s="4" t="inlineStr">
+      <c r="D115" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3010,7 +3003,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D116" s="4" t="inlineStr">
+      <c r="D116" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3032,7 +3025,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D117" s="4" t="inlineStr">
+      <c r="D117" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3054,7 +3047,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D118" s="4" t="inlineStr">
+      <c r="D118" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3076,7 +3069,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D119" s="4" t="inlineStr">
+      <c r="D119" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3098,7 +3091,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D120" s="4" t="inlineStr">
+      <c r="D120" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3120,7 +3113,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D121" s="4" t="inlineStr">
+      <c r="D121" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3142,7 +3135,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D122" s="4" t="inlineStr">
+      <c r="D122" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3164,7 +3157,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D123" s="4" t="inlineStr">
+      <c r="D123" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3186,7 +3179,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D124" s="4" t="inlineStr">
+      <c r="D124" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3208,7 +3201,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D125" s="4" t="inlineStr">
+      <c r="D125" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3230,7 +3223,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D126" s="4" t="inlineStr">
+      <c r="D126" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3252,7 +3245,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D127" s="4" t="inlineStr">
+      <c r="D127" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3274,7 +3267,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D128" s="4" t="inlineStr">
+      <c r="D128" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3296,7 +3289,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D129" s="4" t="inlineStr">
+      <c r="D129" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3318,7 +3311,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D130" s="4" t="inlineStr">
+      <c r="D130" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3340,7 +3333,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D131" s="4" t="inlineStr">
+      <c r="D131" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3362,7 +3355,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D132" s="4" t="inlineStr">
+      <c r="D132" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3384,7 +3377,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D133" s="4" t="inlineStr">
+      <c r="D133" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3406,7 +3399,7 @@
           <t>Double studio apartment</t>
         </is>
       </c>
-      <c r="D134" s="4" t="inlineStr">
+      <c r="D134" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3428,7 +3421,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D135" s="4" t="inlineStr">
+      <c r="D135" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3450,7 +3443,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D136" s="4" t="inlineStr">
+      <c r="D136" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3472,7 +3465,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D137" s="4" t="inlineStr">
+      <c r="D137" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3494,7 +3487,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D138" s="4" t="inlineStr">
+      <c r="D138" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3516,7 +3509,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D139" s="4" t="inlineStr">
+      <c r="D139" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3538,7 +3531,7 @@
           <t>Garsónka</t>
         </is>
       </c>
-      <c r="D140" s="4" t="inlineStr">
+      <c r="D140" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3560,7 +3553,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D141" s="4" t="inlineStr">
+      <c r="D141" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3582,7 +3575,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D142" s="4" t="inlineStr">
+      <c r="D142" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3604,7 +3597,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D143" s="4" t="inlineStr">
+      <c r="D143" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3626,7 +3619,7 @@
           <t>Polyfunkčná budova</t>
         </is>
       </c>
-      <c r="D144" s="4" t="inlineStr">
+      <c r="D144" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3648,7 +3641,7 @@
           <t>Chata / rekreačný dom</t>
         </is>
       </c>
-      <c r="D145" s="4" t="inlineStr">
+      <c r="D145" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3670,7 +3663,7 @@
           <t>Orná pôda</t>
         </is>
       </c>
-      <c r="D146" s="4" t="inlineStr">
+      <c r="D146" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3692,7 +3685,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D147" s="4" t="inlineStr">
+      <c r="D147" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3714,7 +3707,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D148" s="4" t="inlineStr">
+      <c r="D148" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3736,7 +3729,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D149" s="4" t="inlineStr">
+      <c r="D149" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3758,7 +3751,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D150" s="4" t="inlineStr">
+      <c r="D150" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3780,7 +3773,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D151" s="4" t="inlineStr">
+      <c r="D151" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3802,7 +3795,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D152" s="4" t="inlineStr">
+      <c r="D152" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3824,7 +3817,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D153" s="4" t="inlineStr">
+      <c r="D153" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3846,7 +3839,7 @@
           <t>Iný priestor</t>
         </is>
       </c>
-      <c r="D154" s="4" t="inlineStr">
+      <c r="D154" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3868,7 +3861,7 @@
           <t>5+ izbový byt</t>
         </is>
       </c>
-      <c r="D155" s="4" t="inlineStr">
+      <c r="D155" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3890,7 +3883,7 @@
           <t>Samostatná garáž</t>
         </is>
       </c>
-      <c r="D156" s="4" t="inlineStr">
+      <c r="D156" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3912,7 +3905,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D157" s="4" t="inlineStr">
+      <c r="D157" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3934,7 +3927,7 @@
           <t>Garsónka</t>
         </is>
       </c>
-      <c r="D158" s="4" t="inlineStr">
+      <c r="D158" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3956,7 +3949,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D159" s="4" t="inlineStr">
+      <c r="D159" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -3978,7 +3971,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D160" s="4" t="inlineStr">
+      <c r="D160" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4000,7 +3993,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D161" s="4" t="inlineStr">
+      <c r="D161" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4022,7 +4015,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D162" s="4" t="inlineStr">
+      <c r="D162" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4044,7 +4037,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D163" s="4" t="inlineStr">
+      <c r="D163" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4066,7 +4059,7 @@
           <t>Záhradná chatka</t>
         </is>
       </c>
-      <c r="D164" s="4" t="inlineStr">
+      <c r="D164" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4088,7 +4081,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D165" s="4" t="inlineStr">
+      <c r="D165" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4110,7 +4103,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D166" s="4" t="inlineStr">
+      <c r="D166" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4132,7 +4125,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D167" s="4" t="inlineStr">
+      <c r="D167" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4154,7 +4147,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D168" s="4" t="inlineStr">
+      <c r="D168" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4176,7 +4169,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D169" s="4" t="inlineStr">
+      <c r="D169" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4198,7 +4191,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D170" s="4" t="inlineStr">
+      <c r="D170" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4220,7 +4213,7 @@
           <t>Other type of apartment</t>
         </is>
       </c>
-      <c r="D171" s="4" t="inlineStr">
+      <c r="D171" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4242,7 +4235,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D172" s="4" t="inlineStr">
+      <c r="D172" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4264,7 +4257,7 @@
           <t>Pozemok pre bytovú výstavbu</t>
         </is>
       </c>
-      <c r="D173" s="4" t="inlineStr">
+      <c r="D173" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4286,7 +4279,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D174" s="4" t="inlineStr">
+      <c r="D174" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4308,7 +4301,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D175" s="4" t="inlineStr">
+      <c r="D175" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4330,7 +4323,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D176" s="4" t="inlineStr">
+      <c r="D176" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4352,7 +4345,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D177" s="4" t="inlineStr">
+      <c r="D177" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4374,7 +4367,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D178" s="4" t="inlineStr">
+      <c r="D178" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4396,7 +4389,7 @@
           <t>Záhrada</t>
         </is>
       </c>
-      <c r="D179" s="4" t="inlineStr">
+      <c r="D179" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4418,7 +4411,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D180" s="4" t="inlineStr">
+      <c r="D180" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4440,7 +4433,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D181" s="4" t="inlineStr">
+      <c r="D181" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4462,7 +4455,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D182" s="4" t="inlineStr">
+      <c r="D182" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4484,7 +4477,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D183" s="4" t="inlineStr">
+      <c r="D183" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4506,7 +4499,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D184" s="4" t="inlineStr">
+      <c r="D184" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4528,7 +4521,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D185" s="4" t="inlineStr">
+      <c r="D185" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4550,7 +4543,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D186" s="4" t="inlineStr">
+      <c r="D186" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4572,7 +4565,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D187" s="4" t="inlineStr">
+      <c r="D187" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4594,7 +4587,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D188" s="4" t="inlineStr">
+      <c r="D188" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4616,7 +4609,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D189" s="4" t="inlineStr">
+      <c r="D189" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4638,7 +4631,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D190" s="4" t="inlineStr">
+      <c r="D190" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4660,7 +4653,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D191" s="4" t="inlineStr">
+      <c r="D191" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4682,7 +4675,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D192" s="4" t="inlineStr">
+      <c r="D192" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4704,7 +4697,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D193" s="4" t="inlineStr">
+      <c r="D193" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4726,7 +4719,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D194" s="4" t="inlineStr">
+      <c r="D194" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4748,7 +4741,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D195" s="4" t="inlineStr">
+      <c r="D195" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4770,7 +4763,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D196" s="4" t="inlineStr">
+      <c r="D196" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4792,7 +4785,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D197" s="4" t="inlineStr">
+      <c r="D197" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4814,7 +4807,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D198" s="4" t="inlineStr">
+      <c r="D198" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4836,7 +4829,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D199" s="4" t="inlineStr">
+      <c r="D199" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4858,7 +4851,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D200" s="4" t="inlineStr">
+      <c r="D200" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4880,7 +4873,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D201" s="4" t="inlineStr">
+      <c r="D201" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4902,7 +4895,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D202" s="4" t="inlineStr">
+      <c r="D202" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4924,7 +4917,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D203" s="4" t="inlineStr">
+      <c r="D203" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4946,7 +4939,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D204" s="4" t="inlineStr">
+      <c r="D204" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4968,7 +4961,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D205" s="4" t="inlineStr">
+      <c r="D205" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -4990,7 +4983,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D206" s="4" t="inlineStr">
+      <c r="D206" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5012,7 +5005,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D207" s="4" t="inlineStr">
+      <c r="D207" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5034,7 +5027,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D208" s="4" t="inlineStr">
+      <c r="D208" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5056,7 +5049,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D209" s="4" t="inlineStr">
+      <c r="D209" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5078,7 +5071,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D210" s="4" t="inlineStr">
+      <c r="D210" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5100,7 +5093,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D211" s="4" t="inlineStr">
+      <c r="D211" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5122,7 +5115,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D212" s="4" t="inlineStr">
+      <c r="D212" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5144,7 +5137,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D213" s="4" t="inlineStr">
+      <c r="D213" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5166,7 +5159,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D214" s="4" t="inlineStr">
+      <c r="D214" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5188,7 +5181,7 @@
           <t>Garsónka</t>
         </is>
       </c>
-      <c r="D215" s="4" t="inlineStr">
+      <c r="D215" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5210,7 +5203,7 @@
           <t>Kancelárie</t>
         </is>
       </c>
-      <c r="D216" s="4" t="inlineStr">
+      <c r="D216" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5232,7 +5225,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D217" s="4" t="inlineStr">
+      <c r="D217" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5254,7 +5247,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D218" s="4" t="inlineStr">
+      <c r="D218" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5276,7 +5269,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D219" s="4" t="inlineStr">
+      <c r="D219" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5298,7 +5291,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D220" s="4" t="inlineStr">
+      <c r="D220" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5320,7 +5313,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D221" s="4" t="inlineStr">
+      <c r="D221" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5342,7 +5335,7 @@
           <t>Garsónka</t>
         </is>
       </c>
-      <c r="D222" s="4" t="inlineStr">
+      <c r="D222" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5364,7 +5357,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D223" s="4" t="inlineStr">
+      <c r="D223" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5386,7 +5379,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D224" s="4" t="inlineStr">
+      <c r="D224" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5408,7 +5401,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D225" s="4" t="inlineStr">
+      <c r="D225" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5430,7 +5423,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D226" s="4" t="inlineStr">
+      <c r="D226" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5452,7 +5445,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D227" s="4" t="inlineStr">
+      <c r="D227" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5474,7 +5467,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D228" s="4" t="inlineStr">
+      <c r="D228" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5496,7 +5489,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D229" s="4" t="inlineStr">
+      <c r="D229" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5518,7 +5511,7 @@
           <t>5+ izbový byt</t>
         </is>
       </c>
-      <c r="D230" s="4" t="inlineStr">
+      <c r="D230" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5540,7 +5533,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D231" s="4" t="inlineStr">
+      <c r="D231" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5562,7 +5555,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D232" s="4" t="inlineStr">
+      <c r="D232" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5584,7 +5577,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D233" s="4" t="inlineStr">
+      <c r="D233" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5606,7 +5599,7 @@
           <t>Rekreačný pozemok</t>
         </is>
       </c>
-      <c r="D234" s="4" t="inlineStr">
+      <c r="D234" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5628,7 +5621,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D235" s="4" t="inlineStr">
+      <c r="D235" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5650,7 +5643,7 @@
           <t>Other object for housing</t>
         </is>
       </c>
-      <c r="D236" s="4" t="inlineStr">
+      <c r="D236" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5672,7 +5665,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D237" s="4" t="inlineStr">
+      <c r="D237" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5694,7 +5687,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D238" s="4" t="inlineStr">
+      <c r="D238" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5716,7 +5709,7 @@
           <t>Iný priestor</t>
         </is>
       </c>
-      <c r="D239" s="4" t="inlineStr">
+      <c r="D239" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5738,7 +5731,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D240" s="4" t="inlineStr">
+      <c r="D240" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5760,7 +5753,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D241" s="4" t="inlineStr">
+      <c r="D241" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5782,7 +5775,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D242" s="4" t="inlineStr">
+      <c r="D242" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5804,7 +5797,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D243" s="4" t="inlineStr">
+      <c r="D243" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5826,7 +5819,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D244" s="4" t="inlineStr">
+      <c r="D244" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5848,7 +5841,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D245" s="4" t="inlineStr">
+      <c r="D245" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5870,7 +5863,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D246" s="4" t="inlineStr">
+      <c r="D246" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5892,7 +5885,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D247" s="4" t="inlineStr">
+      <c r="D247" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5914,7 +5907,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D248" s="4" t="inlineStr">
+      <c r="D248" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5936,7 +5929,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D249" s="4" t="inlineStr">
+      <c r="D249" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5958,7 +5951,7 @@
           <t>Záhradná chatka</t>
         </is>
       </c>
-      <c r="D250" s="4" t="inlineStr">
+      <c r="D250" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -5980,7 +5973,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D251" s="4" t="inlineStr">
+      <c r="D251" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6002,7 +5995,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D252" s="4" t="inlineStr">
+      <c r="D252" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6024,7 +6017,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D253" s="4" t="inlineStr">
+      <c r="D253" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6046,7 +6039,7 @@
           <t>Mezonet</t>
         </is>
       </c>
-      <c r="D254" s="4" t="inlineStr">
+      <c r="D254" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6068,7 +6061,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D255" s="4" t="inlineStr">
+      <c r="D255" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6090,7 +6083,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D256" s="4" t="inlineStr">
+      <c r="D256" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6112,7 +6105,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D257" s="4" t="inlineStr">
+      <c r="D257" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6134,7 +6127,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D258" s="4" t="inlineStr">
+      <c r="D258" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6156,7 +6149,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D259" s="4" t="inlineStr">
+      <c r="D259" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6178,7 +6171,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D260" s="4" t="inlineStr">
+      <c r="D260" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6200,7 +6193,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D261" s="4" t="inlineStr">
+      <c r="D261" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6222,7 +6215,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D262" s="4" t="inlineStr">
+      <c r="D262" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6244,7 +6237,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D263" s="4" t="inlineStr">
+      <c r="D263" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6266,7 +6259,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D264" s="4" t="inlineStr">
+      <c r="D264" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6288,7 +6281,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D265" s="4" t="inlineStr">
+      <c r="D265" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6310,7 +6303,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D266" s="4" t="inlineStr">
+      <c r="D266" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6332,7 +6325,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D267" s="4" t="inlineStr">
+      <c r="D267" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6354,7 +6347,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D268" s="4" t="inlineStr">
+      <c r="D268" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6376,7 +6369,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D269" s="4" t="inlineStr">
+      <c r="D269" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6398,7 +6391,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D270" s="4" t="inlineStr">
+      <c r="D270" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6420,7 +6413,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D271" s="4" t="inlineStr">
+      <c r="D271" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6442,7 +6435,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D272" s="4" t="inlineStr">
+      <c r="D272" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6464,7 +6457,7 @@
           <t>Reštauračné priestory</t>
         </is>
       </c>
-      <c r="D273" s="4" t="inlineStr">
+      <c r="D273" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6486,7 +6479,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D274" s="4" t="inlineStr">
+      <c r="D274" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6508,7 +6501,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D275" s="4" t="inlineStr">
+      <c r="D275" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6530,7 +6523,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D276" s="4" t="inlineStr">
+      <c r="D276" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6552,7 +6545,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D277" s="4" t="inlineStr">
+      <c r="D277" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6574,7 +6567,7 @@
           <t>Obchodné priestory</t>
         </is>
       </c>
-      <c r="D278" s="4" t="inlineStr">
+      <c r="D278" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6596,7 +6589,7 @@
           <t>Záhrada</t>
         </is>
       </c>
-      <c r="D279" s="4" t="inlineStr">
+      <c r="D279" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6618,7 +6611,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D280" s="4" t="inlineStr">
+      <c r="D280" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6640,7 +6633,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D281" s="4" t="inlineStr">
+      <c r="D281" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6662,7 +6655,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D282" s="4" t="inlineStr">
+      <c r="D282" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6684,7 +6677,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D283" s="4" t="inlineStr">
+      <c r="D283" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6706,7 +6699,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D284" s="4" t="inlineStr">
+      <c r="D284" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6728,7 +6721,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D285" s="4" t="inlineStr">
+      <c r="D285" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6750,7 +6743,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D286" s="4" t="inlineStr">
+      <c r="D286" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6772,7 +6765,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D287" s="4" t="inlineStr">
+      <c r="D287" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6794,7 +6787,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D288" s="4" t="inlineStr">
+      <c r="D288" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6816,7 +6809,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D289" s="4" t="inlineStr">
+      <c r="D289" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6838,7 +6831,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D290" s="4" t="inlineStr">
+      <c r="D290" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6860,7 +6853,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D291" s="4" t="inlineStr">
+      <c r="D291" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6882,7 +6875,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D292" s="4" t="inlineStr">
+      <c r="D292" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6904,7 +6897,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D293" s="4" t="inlineStr">
+      <c r="D293" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6926,7 +6919,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D294" s="4" t="inlineStr">
+      <c r="D294" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6948,7 +6941,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D295" s="4" t="inlineStr">
+      <c r="D295" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6970,7 +6963,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D296" s="4" t="inlineStr">
+      <c r="D296" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -6992,7 +6985,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D297" s="4" t="inlineStr">
+      <c r="D297" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7014,7 +7007,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D298" s="4" t="inlineStr">
+      <c r="D298" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7036,7 +7029,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D299" s="4" t="inlineStr">
+      <c r="D299" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7058,7 +7051,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D300" s="4" t="inlineStr">
+      <c r="D300" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7080,7 +7073,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D301" s="4" t="inlineStr">
+      <c r="D301" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7102,7 +7095,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D302" s="4" t="inlineStr">
+      <c r="D302" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7124,7 +7117,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D303" s="4" t="inlineStr">
+      <c r="D303" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7146,7 +7139,7 @@
           <t>Samostatná garáž</t>
         </is>
       </c>
-      <c r="D304" s="4" t="inlineStr">
+      <c r="D304" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7168,7 +7161,7 @@
           <t>Záhrada</t>
         </is>
       </c>
-      <c r="D305" s="4" t="inlineStr">
+      <c r="D305" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7190,7 +7183,7 @@
           <t>Samostatná garáž</t>
         </is>
       </c>
-      <c r="D306" s="4" t="inlineStr">
+      <c r="D306" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7212,7 +7205,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D307" s="4" t="inlineStr">
+      <c r="D307" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7234,7 +7227,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D308" s="4" t="inlineStr">
+      <c r="D308" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7256,7 +7249,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D309" s="4" t="inlineStr">
+      <c r="D309" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7278,7 +7271,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D310" s="4" t="inlineStr">
+      <c r="D310" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7300,7 +7293,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D311" s="4" t="inlineStr">
+      <c r="D311" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7322,7 +7315,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D312" s="4" t="inlineStr">
+      <c r="D312" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7344,7 +7337,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D313" s="4" t="inlineStr">
+      <c r="D313" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7366,7 +7359,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D314" s="4" t="inlineStr">
+      <c r="D314" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7388,7 +7381,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D315" s="4" t="inlineStr">
+      <c r="D315" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7410,7 +7403,7 @@
           <t>Mobilný dom</t>
         </is>
       </c>
-      <c r="D316" s="4" t="inlineStr">
+      <c r="D316" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7432,7 +7425,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D317" s="4" t="inlineStr">
+      <c r="D317" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7454,7 +7447,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D318" s="4" t="inlineStr">
+      <c r="D318" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7476,7 +7469,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D319" s="4" t="inlineStr">
+      <c r="D319" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7498,7 +7491,7 @@
           <t>Administratívna budova</t>
         </is>
       </c>
-      <c r="D320" s="4" t="inlineStr">
+      <c r="D320" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7520,7 +7513,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D321" s="4" t="inlineStr">
+      <c r="D321" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7542,7 +7535,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D322" s="4" t="inlineStr">
+      <c r="D322" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7564,7 +7557,7 @@
           <t>Garsónka</t>
         </is>
       </c>
-      <c r="D323" s="4" t="inlineStr">
+      <c r="D323" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7586,7 +7579,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D324" s="4" t="inlineStr">
+      <c r="D324" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7608,7 +7601,7 @@
           <t>Garsónka</t>
         </is>
       </c>
-      <c r="D325" s="4" t="inlineStr">
+      <c r="D325" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7630,7 +7623,7 @@
           <t>Zmiešaná zóna</t>
         </is>
       </c>
-      <c r="D326" s="4" t="inlineStr">
+      <c r="D326" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7652,7 +7645,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D327" s="4" t="inlineStr">
+      <c r="D327" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7674,7 +7667,7 @@
           <t>Samostatná garáž</t>
         </is>
       </c>
-      <c r="D328" s="4" t="inlineStr">
+      <c r="D328" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7696,7 +7689,7 @@
           <t>Chata / rekreačný dom</t>
         </is>
       </c>
-      <c r="D329" s="4" t="inlineStr">
+      <c r="D329" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7718,7 +7711,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D330" s="4" t="inlineStr">
+      <c r="D330" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7740,7 +7733,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D331" s="4" t="inlineStr">
+      <c r="D331" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7762,7 +7755,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D332" s="4" t="inlineStr">
+      <c r="D332" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7784,7 +7777,7 @@
           <t>Polyfunkčná budova</t>
         </is>
       </c>
-      <c r="D333" s="4" t="inlineStr">
+      <c r="D333" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7806,7 +7799,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D334" s="4" t="inlineStr">
+      <c r="D334" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7828,7 +7821,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D335" s="4" t="inlineStr">
+      <c r="D335" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7850,7 +7843,7 @@
           <t>Reštauračné priestory</t>
         </is>
       </c>
-      <c r="D336" s="4" t="inlineStr">
+      <c r="D336" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7872,7 +7865,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D337" s="4" t="inlineStr">
+      <c r="D337" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7894,7 +7887,7 @@
           <t>Pozemok pre bytovú výstavbu</t>
         </is>
       </c>
-      <c r="D338" s="4" t="inlineStr">
+      <c r="D338" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7916,7 +7909,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D339" s="4" t="inlineStr">
+      <c r="D339" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7938,7 +7931,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D340" s="4" t="inlineStr">
+      <c r="D340" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7960,7 +7953,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D341" s="4" t="inlineStr">
+      <c r="D341" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -7982,7 +7975,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D342" s="4" t="inlineStr">
+      <c r="D342" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8004,7 +7997,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D343" s="4" t="inlineStr">
+      <c r="D343" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8026,7 +8019,7 @@
           <t>Záhrada</t>
         </is>
       </c>
-      <c r="D344" s="4" t="inlineStr">
+      <c r="D344" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8048,7 +8041,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D345" s="4" t="inlineStr">
+      <c r="D345" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8070,7 +8063,7 @@
           <t>Double studio apartment</t>
         </is>
       </c>
-      <c r="D346" s="4" t="inlineStr">
+      <c r="D346" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8092,7 +8085,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D347" s="4" t="inlineStr">
+      <c r="D347" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8114,7 +8107,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D348" s="4" t="inlineStr">
+      <c r="D348" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8136,7 +8129,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D349" s="4" t="inlineStr">
+      <c r="D349" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8158,7 +8151,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D350" s="4" t="inlineStr">
+      <c r="D350" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8180,7 +8173,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D351" s="4" t="inlineStr">
+      <c r="D351" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8202,7 +8195,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D352" s="4" t="inlineStr">
+      <c r="D352" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8224,7 +8217,7 @@
           <t>Pozemok pre rodinný dom</t>
         </is>
       </c>
-      <c r="D353" s="4" t="inlineStr">
+      <c r="D353" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8246,7 +8239,7 @@
           <t>Chata / rekreačný dom</t>
         </is>
       </c>
-      <c r="D354" s="4" t="inlineStr">
+      <c r="D354" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8268,7 +8261,7 @@
           <t>Samostatná garáž</t>
         </is>
       </c>
-      <c r="D355" s="4" t="inlineStr">
+      <c r="D355" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8290,7 +8283,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D356" s="4" t="inlineStr">
+      <c r="D356" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8312,7 +8305,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D357" s="4" t="inlineStr">
+      <c r="D357" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8334,7 +8327,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D358" s="4" t="inlineStr">
+      <c r="D358" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8356,7 +8349,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D359" s="4" t="inlineStr">
+      <c r="D359" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8378,7 +8371,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D360" s="4" t="inlineStr">
+      <c r="D360" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8400,7 +8393,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D361" s="4" t="inlineStr">
+      <c r="D361" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8422,7 +8415,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D362" s="4" t="inlineStr">
+      <c r="D362" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8444,7 +8437,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D363" s="4" t="inlineStr">
+      <c r="D363" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8466,7 +8459,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D364" s="4" t="inlineStr">
+      <c r="D364" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8488,7 +8481,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D365" s="4" t="inlineStr">
+      <c r="D365" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8510,7 +8503,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D366" s="4" t="inlineStr">
+      <c r="D366" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8532,7 +8525,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D367" s="4" t="inlineStr">
+      <c r="D367" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8554,7 +8547,7 @@
           <t>1-izbový byt</t>
         </is>
       </c>
-      <c r="D368" s="4" t="inlineStr">
+      <c r="D368" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8576,7 +8569,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D369" s="4" t="inlineStr">
+      <c r="D369" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8598,7 +8591,7 @@
           <t>Zrub / chalupa</t>
         </is>
       </c>
-      <c r="D370" s="4" t="inlineStr">
+      <c r="D370" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8620,7 +8613,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D371" s="4" t="inlineStr">
+      <c r="D371" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8642,7 +8635,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D372" s="4" t="inlineStr">
+      <c r="D372" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8664,7 +8657,7 @@
           <t>2-izbový byt</t>
         </is>
       </c>
-      <c r="D373" s="4" t="inlineStr">
+      <c r="D373" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8686,7 +8679,7 @@
           <t>4-izbový byt</t>
         </is>
       </c>
-      <c r="D374" s="4" t="inlineStr">
+      <c r="D374" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8708,7 +8701,7 @@
           <t>Rodinný dom</t>
         </is>
       </c>
-      <c r="D375" s="4" t="inlineStr">
+      <c r="D375" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8730,7 +8723,7 @@
           <t>Obchodné priestory</t>
         </is>
       </c>
-      <c r="D376" s="4" t="inlineStr">
+      <c r="D376" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8752,7 +8745,7 @@
           <t>3-izbový byt</t>
         </is>
       </c>
-      <c r="D377" s="4" t="inlineStr">
+      <c r="D377" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -8774,7 +8767,7 @@
           <t>Zrub / chalupa</t>
         </is>
       </c>
-      <c r="D378" s="4" t="inlineStr">
+      <c r="D378" s="2" t="inlineStr">
         <is>
           <t>otvoriť ponuku</t>
         </is>
@@ -9179,14 +9172,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Súhrn</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>Ponúk celkom</t>
         </is>
@@ -9196,31 +9189,31 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>Aktualizované</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>23.10.2026 15:59</t>
+          <t>23.10.2026 20:37</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="7" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Podľa okresu</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>Položka</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Počet</t>
         </is>
@@ -9307,19 +9300,19 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Podľa kategórie</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>Položka</t>
         </is>
       </c>
-      <c r="B18" s="6" t="inlineStr">
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>Počet</t>
         </is>

</xml_diff>